<commit_message>
Update Excel to use guest mode numbers
</commit_message>
<xml_diff>
--- a/retirement_planner.xlsx
+++ b/retirement_planner.xlsx
@@ -1137,7 +1137,7 @@
         <v>5</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1187,7 +1187,7 @@
         <v>13</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>200000</v>
+        <v>300000</v>
       </c>
       <c r="D8" s="4" t="s">
         <v>14</v>
@@ -1201,7 +1201,7 @@
         <v>15</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>1750000</v>
+        <v>3000000</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>16</v>
@@ -1215,13 +1215,13 @@
         <v>17</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>200000</v>
+        <v>500000</v>
       </c>
       <c r="D10" s="4" t="s">
         <v>18</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>76000</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1235,7 +1235,7 @@
         <v>20</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>11000</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1251,7 +1251,7 @@
         <v>22</v>
       </c>
       <c r="B13" s="6" t="n">
-        <v>120000</v>
+        <v>250000</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1259,7 +1259,7 @@
         <v>23</v>
       </c>
       <c r="B14" s="6" t="n">
-        <v>107000</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1275,7 +1275,7 @@
         <v>25</v>
       </c>
       <c r="B16" s="6" t="n">
-        <v>1000000</v>
+        <v>500000</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1373,7 +1373,7 @@
         <v>37</v>
       </c>
       <c r="B30" s="6" t="n">
-        <v>2250</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1381,7 +1381,7 @@
         <v>38</v>
       </c>
       <c r="B31" s="6" t="n">
-        <v>13500</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1421,7 +1421,7 @@
         <v>43</v>
       </c>
       <c r="B36" s="6" t="n">
-        <v>650000</v>
+        <v>800000</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1581,7 +1581,7 @@
       </c>
       <c r="B3" s="11" t="n">
         <f aca="false">Inputs!B9</f>
-        <v>1750000</v>
+        <v>3000000</v>
       </c>
       <c r="C3" s="11" t="n">
         <f aca="false">IF(65&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,65-Inputs!B25),0)</f>
@@ -1613,7 +1613,7 @@
       </c>
       <c r="J3" s="11" t="n">
         <f aca="false">MAX(0,B3-E3)</f>
-        <v>1578950</v>
+        <v>2828950</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1622,7 +1622,7 @@
       </c>
       <c r="B4" s="14" t="n">
         <f aca="false">J3</f>
-        <v>1578950</v>
+        <v>2828950</v>
       </c>
       <c r="C4" s="14" t="n">
         <f aca="false">IF(66&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,66-Inputs!B25),0)</f>
@@ -1654,7 +1654,7 @@
       </c>
       <c r="J4" s="14" t="n">
         <f aca="false">MAX(0,B4-E4)</f>
-        <v>1407900</v>
+        <v>2657900</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1663,7 +1663,7 @@
       </c>
       <c r="B5" s="11" t="n">
         <f aca="false">J4</f>
-        <v>1407900</v>
+        <v>2657900</v>
       </c>
       <c r="C5" s="11" t="n">
         <f aca="false">IF(67&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,67-Inputs!B25),0)</f>
@@ -1695,7 +1695,7 @@
       </c>
       <c r="J5" s="11" t="n">
         <f aca="false">MAX(0,B5-E5)</f>
-        <v>1277364.4</v>
+        <v>2527364.4</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1704,7 +1704,7 @@
       </c>
       <c r="B6" s="14" t="n">
         <f aca="false">J5</f>
-        <v>1277364.4</v>
+        <v>2527364.4</v>
       </c>
       <c r="C6" s="14" t="n">
         <f aca="false">IF(68&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,68-Inputs!B25),0)</f>
@@ -1736,7 +1736,7 @@
       </c>
       <c r="J6" s="14" t="n">
         <f aca="false">MAX(0,B6-E6)</f>
-        <v>1147841.66</v>
+        <v>2397841.66</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1745,7 +1745,7 @@
       </c>
       <c r="B7" s="11" t="n">
         <f aca="false">J6</f>
-        <v>1147841.66</v>
+        <v>2397841.66</v>
       </c>
       <c r="C7" s="11" t="n">
         <f aca="false">IF(69&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,69-Inputs!B25),0)</f>
@@ -1777,7 +1777,7 @@
       </c>
       <c r="J7" s="11" t="n">
         <f aca="false">MAX(0,B7-E7)</f>
-        <v>1019357.1015</v>
+        <v>2269357.1015</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1786,7 +1786,7 @@
       </c>
       <c r="B8" s="14" t="n">
         <f aca="false">J7</f>
-        <v>1019357.1015</v>
+        <v>2269357.1015</v>
       </c>
       <c r="C8" s="14" t="n">
         <f aca="false">IF(70&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,70-Inputs!B25),0)</f>
@@ -1818,7 +1818,7 @@
       </c>
       <c r="J8" s="14" t="n">
         <f aca="false">MAX(0,B8-E8)</f>
-        <v>891936.6790375</v>
+        <v>2141936.6790375</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1827,7 +1827,7 @@
       </c>
       <c r="B9" s="11" t="n">
         <f aca="false">J8</f>
-        <v>891936.6790375</v>
+        <v>2141936.6790375</v>
       </c>
       <c r="C9" s="11" t="n">
         <f aca="false">IF(71&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,71-Inputs!B25),0)</f>
@@ -1859,7 +1859,7 @@
       </c>
       <c r="J9" s="11" t="n">
         <f aca="false">MAX(0,B9-E9)</f>
-        <v>765606.996013437</v>
+        <v>2015606.99601344</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1868,7 +1868,7 @@
       </c>
       <c r="B10" s="14" t="n">
         <f aca="false">J9</f>
-        <v>765606.996013437</v>
+        <v>2015606.99601344</v>
       </c>
       <c r="C10" s="14" t="n">
         <f aca="false">IF(72&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,72-Inputs!B25),0)</f>
@@ -1900,7 +1900,7 @@
       </c>
       <c r="J10" s="14" t="n">
         <f aca="false">MAX(0,B10-E10)</f>
-        <v>640395.320913773</v>
+        <v>1890395.32091377</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1909,7 +1909,7 @@
       </c>
       <c r="B11" s="17" t="n">
         <f aca="false">J10</f>
-        <v>640395.320913773</v>
+        <v>1890395.32091377</v>
       </c>
       <c r="C11" s="17" t="n">
         <f aca="false">IF(73&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,73-Inputs!B25),0)</f>
@@ -1941,7 +1941,7 @@
       </c>
       <c r="J11" s="17" t="n">
         <f aca="false">MAX(0,B11-E11)</f>
-        <v>516329.603936618</v>
+        <v>1766329.60393662</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1950,7 +1950,7 @@
       </c>
       <c r="B12" s="17" t="n">
         <f aca="false">J11</f>
-        <v>516329.603936618</v>
+        <v>1766329.60393662</v>
       </c>
       <c r="C12" s="17" t="n">
         <f aca="false">IF(74&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,74-Inputs!B25),0)</f>
@@ -1982,7 +1982,7 @@
       </c>
       <c r="J12" s="17" t="n">
         <f aca="false">MAX(0,B12-E12)</f>
-        <v>393438.494035033</v>
+        <v>1643438.49403503</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1991,7 +1991,7 @@
       </c>
       <c r="B13" s="17" t="n">
         <f aca="false">J12</f>
-        <v>393438.494035033</v>
+        <v>1643438.49403503</v>
       </c>
       <c r="C13" s="17" t="n">
         <f aca="false">IF(75&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,75-Inputs!B25),0)</f>
@@ -2023,7 +2023,7 @@
       </c>
       <c r="J13" s="17" t="n">
         <f aca="false">MAX(0,B13-E13)</f>
-        <v>271751.356385909</v>
+        <v>1521751.35638591</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="B14" s="17" t="n">
         <f aca="false">J13</f>
-        <v>271751.356385909</v>
+        <v>1521751.35638591</v>
       </c>
       <c r="C14" s="17" t="n">
         <f aca="false">IF(76&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,76-Inputs!B25),0)</f>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="J14" s="17" t="n">
         <f aca="false">MAX(0,B14-E14)</f>
-        <v>151298.290295557</v>
+        <v>1401298.29029556</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2073,7 +2073,7 @@
       </c>
       <c r="B15" s="17" t="n">
         <f aca="false">J14</f>
-        <v>151298.290295557</v>
+        <v>1401298.29029556</v>
       </c>
       <c r="C15" s="17" t="n">
         <f aca="false">IF(77&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,77-Inputs!B25),0)</f>
@@ -2105,7 +2105,7 @@
       </c>
       <c r="J15" s="17" t="n">
         <f aca="false">MAX(0,B15-E15)</f>
-        <v>32110.1475529454</v>
+        <v>1282110.14755295</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2114,7 +2114,7 @@
       </c>
       <c r="B16" s="17" t="n">
         <f aca="false">J15</f>
-        <v>32110.1475529454</v>
+        <v>1282110.14755295</v>
       </c>
       <c r="C16" s="17" t="n">
         <f aca="false">IF(78&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,78-Inputs!B25),0)</f>
@@ -2146,7 +2146,7 @@
       </c>
       <c r="J16" s="17" t="n">
         <f aca="false">MAX(0,B16-E16)</f>
-        <v>0</v>
+        <v>1164218.55124177</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2155,7 +2155,7 @@
       </c>
       <c r="B17" s="17" t="n">
         <f aca="false">J16</f>
-        <v>0</v>
+        <v>1164218.55124177</v>
       </c>
       <c r="C17" s="17" t="n">
         <f aca="false">IF(79&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,79-Inputs!B25),0)</f>
@@ -2187,7 +2187,7 @@
       </c>
       <c r="J17" s="17" t="n">
         <f aca="false">MAX(0,B17-E17)</f>
-        <v>0</v>
+        <v>1047655.91502281</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2196,7 +2196,7 @@
       </c>
       <c r="B18" s="17" t="n">
         <f aca="false">J17</f>
-        <v>0</v>
+        <v>1047655.91502281</v>
       </c>
       <c r="C18" s="17" t="n">
         <f aca="false">IF(80&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,80-Inputs!B25),0)</f>
@@ -2228,7 +2228,7 @@
       </c>
       <c r="J18" s="17" t="n">
         <f aca="false">MAX(0,B18-E18)</f>
-        <v>0</v>
+        <v>932455.462898383</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2237,7 +2237,7 @@
       </c>
       <c r="B19" s="17" t="n">
         <f aca="false">J18</f>
-        <v>0</v>
+        <v>932455.462898383</v>
       </c>
       <c r="C19" s="17" t="n">
         <f aca="false">IF(81&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,81-Inputs!B25),0)</f>
@@ -2269,7 +2269,7 @@
       </c>
       <c r="J19" s="17" t="n">
         <f aca="false">MAX(0,B19-E19)</f>
-        <v>0</v>
+        <v>818651.249470843</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2278,7 +2278,7 @@
       </c>
       <c r="B20" s="17" t="n">
         <f aca="false">J19</f>
-        <v>0</v>
+        <v>818651.249470843</v>
       </c>
       <c r="C20" s="17" t="n">
         <f aca="false">IF(82&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,82-Inputs!B25),0)</f>
@@ -2310,7 +2310,7 @@
       </c>
       <c r="J20" s="17" t="n">
         <f aca="false">MAX(0,B20-E20)</f>
-        <v>0</v>
+        <v>706278.180707614</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2319,7 +2319,7 @@
       </c>
       <c r="B21" s="17" t="n">
         <f aca="false">J20</f>
-        <v>0</v>
+        <v>706278.180707614</v>
       </c>
       <c r="C21" s="17" t="n">
         <f aca="false">IF(83&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,83-Inputs!B25),0)</f>
@@ -2351,7 +2351,7 @@
       </c>
       <c r="J21" s="17" t="n">
         <f aca="false">MAX(0,B21-E21)</f>
-        <v>0</v>
+        <v>595372.035225304</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2360,7 +2360,7 @@
       </c>
       <c r="B22" s="17" t="n">
         <f aca="false">J21</f>
-        <v>0</v>
+        <v>595372.035225304</v>
       </c>
       <c r="C22" s="17" t="n">
         <f aca="false">IF(84&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,84-Inputs!B25),0)</f>
@@ -2392,7 +2392,7 @@
       </c>
       <c r="J22" s="17" t="n">
         <f aca="false">MAX(0,B22-E22)</f>
-        <v>0</v>
+        <v>485969.486105936</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2401,7 +2401,7 @@
       </c>
       <c r="B23" s="17" t="n">
         <f aca="false">J22</f>
-        <v>0</v>
+        <v>485969.486105936</v>
       </c>
       <c r="C23" s="17" t="n">
         <f aca="false">IF(85&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,85-Inputs!B25),0)</f>
@@ -2433,7 +2433,7 @@
       </c>
       <c r="J23" s="17" t="n">
         <f aca="false">MAX(0,B23-E23)</f>
-        <v>0</v>
+        <v>378108.123258585</v>
       </c>
     </row>
   </sheetData>
@@ -2553,11 +2553,11 @@
       </c>
       <c r="C3" s="11" t="n">
         <f aca="false">Inputs!B30*12</f>
-        <v>27000</v>
+        <v>36000</v>
       </c>
       <c r="D3" s="11" t="n">
         <f aca="false">Inputs!B31+Inputs!B32</f>
-        <v>15000</v>
+        <v>16500</v>
       </c>
       <c r="E3" s="11" t="n">
         <f aca="false">IF(55&lt;65,Inputs!B35*12,0)</f>
@@ -2569,7 +2569,7 @@
       </c>
       <c r="G3" s="20" t="n">
         <f aca="false">B3+C3+D3+E3+F3</f>
-        <v>137820</v>
+        <v>148320</v>
       </c>
       <c r="H3" s="11" t="n">
         <f aca="false">IF(65&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,65-Inputs!B25),0)</f>
@@ -2605,7 +2605,7 @@
       </c>
       <c r="P3" s="21" t="n">
         <f aca="false">H3+I3+J3+K3+L3-G3-N3-O3</f>
-        <v>-5402.885</v>
+        <v>-15902.885</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2618,11 +2618,11 @@
       </c>
       <c r="C4" s="14" t="n">
         <f aca="false">Inputs!B30*12</f>
-        <v>27000</v>
+        <v>36000</v>
       </c>
       <c r="D4" s="14" t="n">
         <f aca="false">Inputs!B31+Inputs!B32</f>
-        <v>15000</v>
+        <v>16500</v>
       </c>
       <c r="E4" s="14" t="n">
         <f aca="false">IF(56&lt;65,Inputs!B35*12,0)</f>
@@ -2634,7 +2634,7 @@
       </c>
       <c r="G4" s="22" t="n">
         <f aca="false">B4+C4+D4+E4+F4</f>
-        <v>140451</v>
+        <v>150951</v>
       </c>
       <c r="H4" s="14" t="n">
         <f aca="false">IF(66&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,66-Inputs!B25),0)</f>
@@ -2670,7 +2670,7 @@
       </c>
       <c r="P4" s="23" t="n">
         <f aca="false">H4+I4+J4+K4+L4-G4-N4-O4</f>
-        <v>-8033.885</v>
+        <v>-18533.885</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2683,11 +2683,11 @@
       </c>
       <c r="C5" s="11" t="n">
         <f aca="false">Inputs!B30*12</f>
-        <v>27000</v>
+        <v>36000</v>
       </c>
       <c r="D5" s="11" t="n">
         <f aca="false">Inputs!B31+Inputs!B32</f>
-        <v>15000</v>
+        <v>16500</v>
       </c>
       <c r="E5" s="11" t="n">
         <f aca="false">IF(57&lt;65,Inputs!B35*12,0)</f>
@@ -2699,7 +2699,7 @@
       </c>
       <c r="G5" s="20" t="n">
         <f aca="false">B5+C5+D5+E5+F5</f>
-        <v>143163.15</v>
+        <v>153663.15</v>
       </c>
       <c r="H5" s="11" t="n">
         <f aca="false">IF(67&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,67-Inputs!B25),0)</f>
@@ -2735,7 +2735,7 @@
       </c>
       <c r="P5" s="21" t="n">
         <f aca="false">H5+I5+J5+K5+L5-G5-N5-O5</f>
-        <v>-1015.66771999996</v>
+        <v>-11515.66772</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2748,11 +2748,11 @@
       </c>
       <c r="C6" s="14" t="n">
         <f aca="false">Inputs!B30*12</f>
-        <v>27000</v>
+        <v>36000</v>
       </c>
       <c r="D6" s="14" t="n">
         <f aca="false">Inputs!B31+Inputs!B32</f>
-        <v>15000</v>
+        <v>16500</v>
       </c>
       <c r="E6" s="14" t="n">
         <f aca="false">IF(58&lt;65,Inputs!B35*12,0)</f>
@@ -2764,7 +2764,7 @@
       </c>
       <c r="G6" s="22" t="n">
         <f aca="false">B6+C6+D6+E6+F6</f>
-        <v>145958.9955</v>
+        <v>156458.9955</v>
       </c>
       <c r="H6" s="14" t="n">
         <f aca="false">IF(68&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,68-Inputs!B25),0)</f>
@@ -2800,7 +2800,7 @@
       </c>
       <c r="P6" s="23" t="n">
         <f aca="false">H6+I6+J6+K6+L6-G6-N6-O6</f>
-        <v>-3568.25403799999</v>
+        <v>-14068.254038</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2813,11 +2813,11 @@
       </c>
       <c r="C7" s="11" t="n">
         <f aca="false">Inputs!B30*12</f>
-        <v>27000</v>
+        <v>36000</v>
       </c>
       <c r="D7" s="11" t="n">
         <f aca="false">Inputs!B31+Inputs!B32</f>
-        <v>15000</v>
+        <v>16500</v>
       </c>
       <c r="E7" s="11" t="n">
         <f aca="false">IF(59&lt;65,Inputs!B35*12,0)</f>
@@ -2829,7 +2829,7 @@
       </c>
       <c r="G7" s="20" t="n">
         <f aca="false">B7+C7+D7+E7+F7</f>
-        <v>148841.163915</v>
+        <v>159341.163915</v>
       </c>
       <c r="H7" s="11" t="n">
         <f aca="false">IF(69&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,69-Inputs!B25),0)</f>
@@ -2865,7 +2865,7 @@
       </c>
       <c r="P7" s="21" t="n">
         <f aca="false">H7+I7+J7+K7+L7-G7-N7-O7</f>
-        <v>-6201.08179145001</v>
+        <v>-16701.08179145</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2878,11 +2878,11 @@
       </c>
       <c r="C8" s="14" t="n">
         <f aca="false">Inputs!B30*12</f>
-        <v>27000</v>
+        <v>36000</v>
       </c>
       <c r="D8" s="14" t="n">
         <f aca="false">Inputs!B31+Inputs!B32</f>
-        <v>15000</v>
+        <v>16500</v>
       </c>
       <c r="E8" s="14" t="n">
         <f aca="false">IF(60&lt;65,Inputs!B35*12,0)</f>
@@ -2894,7 +2894,7 @@
       </c>
       <c r="G8" s="22" t="n">
         <f aca="false">B8+C8+D8+E8+F8</f>
-        <v>151812.36730995</v>
+        <v>162312.36730995</v>
       </c>
       <c r="H8" s="14" t="n">
         <f aca="false">IF(70&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,70-Inputs!B25),0)</f>
@@ -2930,7 +2930,7 @@
       </c>
       <c r="P8" s="23" t="n">
         <f aca="false">H8+I8+J8+K8+L8-G8-N8-O8</f>
-        <v>-8916.71100831127</v>
+        <v>-19416.7110083113</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2943,11 +2943,11 @@
       </c>
       <c r="C9" s="11" t="n">
         <f aca="false">Inputs!B30*12</f>
-        <v>27000</v>
+        <v>36000</v>
       </c>
       <c r="D9" s="11" t="n">
         <f aca="false">Inputs!B31+Inputs!B32</f>
-        <v>15000</v>
+        <v>16500</v>
       </c>
       <c r="E9" s="11" t="n">
         <f aca="false">IF(61&lt;65,Inputs!B35*12,0)</f>
@@ -2959,7 +2959,7 @@
       </c>
       <c r="G9" s="20" t="n">
         <f aca="false">B9+C9+D9+E9+F9</f>
-        <v>154875.405230624</v>
+        <v>165375.405230624</v>
       </c>
       <c r="H9" s="11" t="n">
         <f aca="false">IF(71&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,71-Inputs!B25),0)</f>
@@ -2995,7 +2995,7 @@
       </c>
       <c r="P9" s="21" t="n">
         <f aca="false">H9+I9+J9+K9+L9-G9-N9-O9</f>
-        <v>-11717.7853964438</v>
+        <v>-22217.7853964438</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="C10" s="14" t="n">
         <f aca="false">Inputs!B30*12</f>
-        <v>27000</v>
+        <v>36000</v>
       </c>
       <c r="D10" s="14" t="n">
         <f aca="false">Inputs!B31+Inputs!B32</f>
-        <v>15000</v>
+        <v>16500</v>
       </c>
       <c r="E10" s="14" t="n">
         <f aca="false">IF(62&lt;65,Inputs!B35*12,0)</f>
@@ -3024,7 +3024,7 @@
       </c>
       <c r="G10" s="22" t="n">
         <f aca="false">B10+C10+D10+E10+F10</f>
-        <v>158033.167633986</v>
+        <v>168533.167633986</v>
       </c>
       <c r="H10" s="14" t="n">
         <f aca="false">IF(72&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,72-Inputs!B25),0)</f>
@@ -3060,7 +3060,7 @@
       </c>
       <c r="P10" s="23" t="n">
         <f aca="false">H10+I10+J10+K10+L10-G10-N10-O10</f>
-        <v>-14607.0351789518</v>
+        <v>-25107.0351789518</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3073,11 +3073,11 @@
       </c>
       <c r="C11" s="17" t="n">
         <f aca="false">Inputs!B30*12</f>
-        <v>27000</v>
+        <v>36000</v>
       </c>
       <c r="D11" s="17" t="n">
         <f aca="false">Inputs!B31+Inputs!B32</f>
-        <v>15000</v>
+        <v>16500</v>
       </c>
       <c r="E11" s="17" t="n">
         <f aca="false">IF(63&lt;65,Inputs!B35*12,0)</f>
@@ -3089,7 +3089,7 @@
       </c>
       <c r="G11" s="24" t="n">
         <f aca="false">B11+C11+D11+E11+F11</f>
-        <v>161288.637921772</v>
+        <v>171788.637921772</v>
       </c>
       <c r="H11" s="17" t="n">
         <f aca="false">IF(73&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,73-Inputs!B25),0)</f>
@@ -3125,7 +3125,7 @@
       </c>
       <c r="P11" s="25" t="n">
         <f aca="false">H11+I11+J11+K11+L11-G11-N11-O11</f>
-        <v>-17587.2800303614</v>
+        <v>-28087.2800303614</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3138,11 +3138,11 @@
       </c>
       <c r="C12" s="17" t="n">
         <f aca="false">Inputs!B30*12</f>
-        <v>27000</v>
+        <v>36000</v>
       </c>
       <c r="D12" s="17" t="n">
         <f aca="false">Inputs!B31+Inputs!B32</f>
-        <v>15000</v>
+        <v>16500</v>
       </c>
       <c r="E12" s="17" t="n">
         <f aca="false">IF(64&lt;65,Inputs!B35*12,0)</f>
@@ -3154,7 +3154,7 @@
       </c>
       <c r="G12" s="24" t="n">
         <f aca="false">B12+C12+D12+E12+F12</f>
-        <v>164644.896081129</v>
+        <v>175144.896081129</v>
       </c>
       <c r="H12" s="17" t="n">
         <f aca="false">IF(74&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,74-Inputs!B25),0)</f>
@@ -3190,7 +3190,7 @@
       </c>
       <c r="P12" s="25" t="n">
         <f aca="false">H12+I12+J12+K12+L12-G12-N12-O12</f>
-        <v>-20661.4321174336</v>
+        <v>-31161.4321174336</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3203,11 +3203,11 @@
       </c>
       <c r="C13" s="17" t="n">
         <f aca="false">Inputs!B30*12</f>
-        <v>27000</v>
+        <v>36000</v>
       </c>
       <c r="D13" s="17" t="n">
         <f aca="false">Inputs!B31+Inputs!B32</f>
-        <v>15000</v>
+        <v>16500</v>
       </c>
       <c r="E13" s="17" t="n">
         <f aca="false">IF(65&lt;65,Inputs!B35*12,0)</f>
@@ -3219,7 +3219,7 @@
       </c>
       <c r="G13" s="24" t="n">
         <f aca="false">B13+C13+D13+E13+F13</f>
-        <v>158505.121936352</v>
+        <v>169005.121936352</v>
       </c>
       <c r="H13" s="17" t="n">
         <f aca="false">IF(75&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,75-Inputs!B25),0)</f>
@@ -3255,7 +3255,7 @@
       </c>
       <c r="P13" s="25" t="n">
         <f aca="false">H13+I13+J13+K13+L13-G13-N13-O13</f>
-        <v>9599.50075143549</v>
+        <v>-900.499248564507</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3268,11 +3268,11 @@
       </c>
       <c r="C14" s="17" t="n">
         <f aca="false">Inputs!B30*12</f>
-        <v>27000</v>
+        <v>36000</v>
       </c>
       <c r="D14" s="17" t="n">
         <f aca="false">Inputs!B31+Inputs!B32</f>
-        <v>15000</v>
+        <v>16500</v>
       </c>
       <c r="E14" s="17" t="n">
         <f aca="false">IF(66&lt;65,Inputs!B35*12,0)</f>
@@ -3284,7 +3284,7 @@
       </c>
       <c r="G14" s="24" t="n">
         <f aca="false">B14+C14+D14+E14+F14</f>
-        <v>162072.598515872</v>
+        <v>172572.598515872</v>
       </c>
       <c r="H14" s="17" t="n">
         <f aca="false">IF(76&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,76-Inputs!B25),0)</f>
@@ -3320,7 +3320,7 @@
       </c>
       <c r="P14" s="25" t="n">
         <f aca="false">H14+I14+J14+K14+L14-G14-N14-O14</f>
-        <v>6924.21186411068</v>
+        <v>-3575.78813588932</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3333,11 +3333,11 @@
       </c>
       <c r="C15" s="17" t="n">
         <f aca="false">Inputs!B30*12</f>
-        <v>27000</v>
+        <v>36000</v>
       </c>
       <c r="D15" s="17" t="n">
         <f aca="false">Inputs!B31+Inputs!B32</f>
-        <v>15000</v>
+        <v>16500</v>
       </c>
       <c r="E15" s="17" t="n">
         <f aca="false">IF(67&lt;65,Inputs!B35*12,0)</f>
@@ -3349,7 +3349,7 @@
       </c>
       <c r="G15" s="24" t="n">
         <f aca="false">B15+C15+D15+E15+F15</f>
-        <v>165750.715538848</v>
+        <v>176250.715538848</v>
       </c>
       <c r="H15" s="17" t="n">
         <f aca="false">IF(77&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,77-Inputs!B25),0)</f>
@@ -3385,7 +3385,7 @@
       </c>
       <c r="P15" s="25" t="n">
         <f aca="false">H15+I15+J15+K15+L15-G15-N15-O15</f>
-        <v>4160.5872256337</v>
+        <v>-6339.4127743663</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3398,11 +3398,11 @@
       </c>
       <c r="C16" s="17" t="n">
         <f aca="false">Inputs!B30*12</f>
-        <v>27000</v>
+        <v>36000</v>
       </c>
       <c r="D16" s="17" t="n">
         <f aca="false">Inputs!B31+Inputs!B32</f>
-        <v>15000</v>
+        <v>16500</v>
       </c>
       <c r="E16" s="17" t="n">
         <f aca="false">IF(68&lt;65,Inputs!B35*12,0)</f>
@@ -3414,7 +3414,7 @@
       </c>
       <c r="G16" s="24" t="n">
         <f aca="false">B16+C16+D16+E16+F16</f>
-        <v>169542.973025889</v>
+        <v>180042.973025889</v>
       </c>
       <c r="H16" s="17" t="n">
         <f aca="false">IF(78&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,78-Inputs!B25),0)</f>
@@ -3450,7 +3450,7 @@
       </c>
       <c r="P16" s="25" t="n">
         <f aca="false">H16+I16+J16+K16+L16-G16-N16-O16</f>
-        <v>1305.68443270496</v>
+        <v>-9194.31556729504</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3463,11 +3463,11 @@
       </c>
       <c r="C17" s="17" t="n">
         <f aca="false">Inputs!B30*12</f>
-        <v>27000</v>
+        <v>36000</v>
       </c>
       <c r="D17" s="17" t="n">
         <f aca="false">Inputs!B31+Inputs!B32</f>
-        <v>15000</v>
+        <v>16500</v>
       </c>
       <c r="E17" s="17" t="n">
         <f aca="false">IF(69&lt;65,Inputs!B35*12,0)</f>
@@ -3479,7 +3479,7 @@
       </c>
       <c r="G17" s="24" t="n">
         <f aca="false">B17+C17+D17+E17+F17</f>
-        <v>173452.985038585</v>
+        <v>183952.985038585</v>
       </c>
       <c r="H17" s="17" t="n">
         <f aca="false">IF(79&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,79-Inputs!B25),0)</f>
@@ -3515,7 +3515,7 @@
       </c>
       <c r="P17" s="25" t="n">
         <f aca="false">H17+I17+J17+K17+L17-G17-N17-O17</f>
-        <v>-1643.53901852602</v>
+        <v>-12143.539018526</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3528,11 +3528,11 @@
       </c>
       <c r="C18" s="17" t="n">
         <f aca="false">Inputs!B30*12</f>
-        <v>27000</v>
+        <v>36000</v>
       </c>
       <c r="D18" s="17" t="n">
         <f aca="false">Inputs!B31+Inputs!B32</f>
-        <v>15000</v>
+        <v>16500</v>
       </c>
       <c r="E18" s="17" t="n">
         <f aca="false">IF(70&lt;65,Inputs!B35*12,0)</f>
@@ -3544,7 +3544,7 @@
       </c>
       <c r="G18" s="24" t="n">
         <f aca="false">B18+C18+D18+E18+F18</f>
-        <v>177484.483552758</v>
+        <v>187984.483552758</v>
       </c>
       <c r="H18" s="17" t="n">
         <f aca="false">IF(80&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,80-Inputs!B25),0)</f>
@@ -3580,7 +3580,7 @@
       </c>
       <c r="P18" s="25" t="n">
         <f aca="false">H18+I18+J18+K18+L18-G18-N18-O18</f>
-        <v>-4690.2292571972</v>
+        <v>-15190.2292571972</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3593,11 +3593,11 @@
       </c>
       <c r="C19" s="17" t="n">
         <f aca="false">Inputs!B30*12</f>
-        <v>27000</v>
+        <v>36000</v>
       </c>
       <c r="D19" s="17" t="n">
         <f aca="false">Inputs!B31+Inputs!B32</f>
-        <v>15000</v>
+        <v>16500</v>
       </c>
       <c r="E19" s="17" t="n">
         <f aca="false">IF(71&lt;65,Inputs!B35*12,0)</f>
@@ -3609,7 +3609,7 @@
       </c>
       <c r="G19" s="24" t="n">
         <f aca="false">B19+C19+D19+E19+F19</f>
-        <v>181641.322470506</v>
+        <v>192141.322470506</v>
       </c>
       <c r="H19" s="17" t="n">
         <f aca="false">IF(81&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,81-Inputs!B25),0)</f>
@@ -3645,7 +3645,7 @@
       </c>
       <c r="P19" s="25" t="n">
         <f aca="false">H19+I19+J19+K19+L19-G19-N19-O19</f>
-        <v>-7837.63969255681</v>
+        <v>-18337.6396925568</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C20" s="17" t="n">
         <f aca="false">Inputs!B30*12</f>
-        <v>27000</v>
+        <v>36000</v>
       </c>
       <c r="D20" s="17" t="n">
         <f aca="false">Inputs!B31+Inputs!B32</f>
-        <v>15000</v>
+        <v>16500</v>
       </c>
       <c r="E20" s="17" t="n">
         <f aca="false">IF(72&lt;65,Inputs!B35*12,0)</f>
@@ -3674,7 +3674,7 @@
       </c>
       <c r="G20" s="24" t="n">
         <f aca="false">B20+C20+D20+E20+F20</f>
-        <v>185927.481776345</v>
+        <v>196427.481776345</v>
       </c>
       <c r="H20" s="17" t="n">
         <f aca="false">IF(82&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,82-Inputs!B25),0)</f>
@@ -3710,7 +3710,7 @@
       </c>
       <c r="P20" s="25" t="n">
         <f aca="false">H20+I20+J20+K20+L20-G20-N20-O20</f>
-        <v>-11089.1348039474</v>
+        <v>-21589.1348039474</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3723,11 +3723,11 @@
       </c>
       <c r="C21" s="17" t="n">
         <f aca="false">Inputs!B30*12</f>
-        <v>27000</v>
+        <v>36000</v>
       </c>
       <c r="D21" s="17" t="n">
         <f aca="false">Inputs!B31+Inputs!B32</f>
-        <v>15000</v>
+        <v>16500</v>
       </c>
       <c r="E21" s="17" t="n">
         <f aca="false">IF(73&lt;65,Inputs!B35*12,0)</f>
@@ -3739,7 +3739,7 @@
       </c>
       <c r="G21" s="24" t="n">
         <f aca="false">B21+C21+D21+E21+F21</f>
-        <v>190347.071842946</v>
+        <v>200847.071842946</v>
       </c>
       <c r="H21" s="17" t="n">
         <f aca="false">IF(83&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,83-Inputs!B25),0)</f>
@@ -3775,7 +3775,7 @@
       </c>
       <c r="P21" s="25" t="n">
         <f aca="false">H21+I21+J21+K21+L21-G21-N21-O21</f>
-        <v>-14448.1940712382</v>
+        <v>-24948.1940712382</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3788,11 +3788,11 @@
       </c>
       <c r="C22" s="17" t="n">
         <f aca="false">Inputs!B30*12</f>
-        <v>27000</v>
+        <v>36000</v>
       </c>
       <c r="D22" s="17" t="n">
         <f aca="false">Inputs!B31+Inputs!B32</f>
-        <v>15000</v>
+        <v>16500</v>
       </c>
       <c r="E22" s="17" t="n">
         <f aca="false">IF(74&lt;65,Inputs!B35*12,0)</f>
@@ -3804,7 +3804,7 @@
       </c>
       <c r="G22" s="24" t="n">
         <f aca="false">B22+C22+D22+E22+F22</f>
-        <v>194904.33789221</v>
+        <v>205404.33789221</v>
       </c>
       <c r="H22" s="17" t="n">
         <f aca="false">IF(84&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,84-Inputs!B25),0)</f>
@@ -3840,7 +3840,7 @@
       </c>
       <c r="P22" s="25" t="n">
         <f aca="false">H22+I22+J22+K22+L22-G22-N22-O22</f>
-        <v>-17918.4160512098</v>
+        <v>-28418.4160512098</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3853,11 +3853,11 @@
       </c>
       <c r="C23" s="17" t="n">
         <f aca="false">Inputs!B30*12</f>
-        <v>27000</v>
+        <v>36000</v>
       </c>
       <c r="D23" s="17" t="n">
         <f aca="false">Inputs!B31+Inputs!B32</f>
-        <v>15000</v>
+        <v>16500</v>
       </c>
       <c r="E23" s="17" t="n">
         <f aca="false">IF(75&lt;65,Inputs!B35*12,0)</f>
@@ -3869,7 +3869,7 @@
       </c>
       <c r="G23" s="24" t="n">
         <f aca="false">B23+C23+D23+E23+F23</f>
-        <v>199603.664617651</v>
+        <v>210103.664617651</v>
       </c>
       <c r="H23" s="17" t="n">
         <f aca="false">IF(85&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,85-Inputs!B25),0)</f>
@@ -3905,7 +3905,7 @@
       </c>
       <c r="P23" s="25" t="n">
         <f aca="false">H23+I23+J23+K23+L23-G23-N23-O23</f>
-        <v>-21503.5226056258</v>
+        <v>-32003.5226056258</v>
       </c>
     </row>
   </sheetData>
@@ -3987,35 +3987,35 @@
       </c>
       <c r="B3" s="11" t="n">
         <f aca="false">'Roth Conversion'!J3</f>
-        <v>1578950</v>
+        <v>2828950</v>
       </c>
       <c r="C3" s="11" t="n">
         <f aca="false">(Inputs!B10+Inputs!B13)*(1+Inputs!B19)-'Withdrawal Plan'!K3</f>
-        <v>345600</v>
+        <v>810000</v>
       </c>
       <c r="D3" s="11" t="n">
         <f aca="false">Inputs!E11*(1+Inputs!B19)</f>
-        <v>11880</v>
+        <v>10800</v>
       </c>
       <c r="E3" s="11" t="n">
         <f aca="false">Inputs!E10*(1+Inputs!B19)</f>
-        <v>82080</v>
+        <v>54000</v>
       </c>
       <c r="F3" s="11" t="n">
         <f aca="false">MAX(0,Inputs!B14*(1+Inputs!B19)-'Withdrawal Plan'!M3)</f>
-        <v>113340</v>
+        <v>105780</v>
       </c>
       <c r="G3" s="11" t="n">
         <f aca="false">MAX(0,Inputs!B16*(1+Inputs!B19)-'Withdrawal Plan'!L3)</f>
-        <v>1080000</v>
+        <v>540000</v>
       </c>
       <c r="H3" s="20" t="n">
         <f aca="false">SUM(B3:G3)</f>
-        <v>3211850</v>
+        <v>4349530</v>
       </c>
       <c r="I3" s="21" t="n">
         <f aca="false">H3+Inputs!B36</f>
-        <v>3861850</v>
+        <v>5149530</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4024,35 +4024,35 @@
       </c>
       <c r="B4" s="14" t="n">
         <f aca="false">'Roth Conversion'!J4</f>
-        <v>1407900</v>
+        <v>2657900</v>
       </c>
       <c r="C4" s="14" t="n">
         <f aca="false">MAX(0,C3*(1+Inputs!B19)-'Withdrawal Plan'!K4)</f>
-        <v>373248</v>
+        <v>874800</v>
       </c>
       <c r="D4" s="14" t="n">
         <f aca="false">D3*(1+Inputs!B19)</f>
-        <v>12830.4</v>
+        <v>11664</v>
       </c>
       <c r="E4" s="14" t="n">
         <f aca="false">E3*(1+Inputs!B19)</f>
-        <v>88646.4</v>
+        <v>58320</v>
       </c>
       <c r="F4" s="14" t="n">
         <f aca="false">MAX(0,F3*(1+Inputs!B19)-'Withdrawal Plan'!M4)</f>
-        <v>120076.2</v>
+        <v>111911.4</v>
       </c>
       <c r="G4" s="14" t="n">
         <f aca="false">MAX(0,G3*(1+Inputs!B19)-'Withdrawal Plan'!L4)</f>
-        <v>1166400</v>
+        <v>583200</v>
       </c>
       <c r="H4" s="22" t="n">
         <f aca="false">SUM(B4:G4)</f>
-        <v>3169101</v>
+        <v>4297795.4</v>
       </c>
       <c r="I4" s="23" t="n">
         <f aca="false">H4+Inputs!B36</f>
-        <v>3819101</v>
+        <v>5097795.4</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4061,35 +4061,35 @@
       </c>
       <c r="B5" s="11" t="n">
         <f aca="false">'Roth Conversion'!J5</f>
-        <v>1277364.4</v>
+        <v>2527364.4</v>
       </c>
       <c r="C5" s="11" t="n">
         <f aca="false">MAX(0,C4*(1+Inputs!B19)-'Withdrawal Plan'!K5)</f>
-        <v>403107.84</v>
+        <v>944784</v>
       </c>
       <c r="D5" s="11" t="n">
         <f aca="false">D4*(1+Inputs!B19)</f>
-        <v>13856.832</v>
+        <v>12597.12</v>
       </c>
       <c r="E5" s="11" t="n">
         <f aca="false">E4*(1+Inputs!B19)</f>
-        <v>95738.112</v>
+        <v>62985.6</v>
       </c>
       <c r="F5" s="11" t="n">
         <f aca="false">MAX(0,F4*(1+Inputs!B19)-'Withdrawal Plan'!M5)</f>
-        <v>127234.746</v>
+        <v>118416.762</v>
       </c>
       <c r="G5" s="11" t="n">
         <f aca="false">MAX(0,G4*(1+Inputs!B19)-'Withdrawal Plan'!L5)</f>
-        <v>1259712</v>
+        <v>629856</v>
       </c>
       <c r="H5" s="20" t="n">
         <f aca="false">SUM(B5:G5)</f>
-        <v>3177013.93</v>
+        <v>4296003.882</v>
       </c>
       <c r="I5" s="21" t="n">
         <f aca="false">H5+Inputs!B36</f>
-        <v>3827013.93</v>
+        <v>5096003.882</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4098,35 +4098,35 @@
       </c>
       <c r="B6" s="14" t="n">
         <f aca="false">'Roth Conversion'!J6</f>
-        <v>1147841.66</v>
+        <v>2397841.66</v>
       </c>
       <c r="C6" s="14" t="n">
         <f aca="false">MAX(0,C5*(1+Inputs!B19)-'Withdrawal Plan'!K6)</f>
-        <v>435356.4672</v>
+        <v>1020366.72</v>
       </c>
       <c r="D6" s="14" t="n">
         <f aca="false">D5*(1+Inputs!B19)</f>
-        <v>14965.37856</v>
+        <v>13604.8896</v>
       </c>
       <c r="E6" s="14" t="n">
         <f aca="false">E5*(1+Inputs!B19)</f>
-        <v>103397.16096</v>
+        <v>68024.448</v>
       </c>
       <c r="F6" s="14" t="n">
         <f aca="false">MAX(0,F5*(1+Inputs!B19)-'Withdrawal Plan'!M6)</f>
-        <v>134843.59818</v>
+        <v>125320.17546</v>
       </c>
       <c r="G6" s="14" t="n">
         <f aca="false">MAX(0,G5*(1+Inputs!B19)-'Withdrawal Plan'!L6)</f>
-        <v>1360488.96</v>
+        <v>680244.48</v>
       </c>
       <c r="H6" s="22" t="n">
         <f aca="false">SUM(B6:G6)</f>
-        <v>3196893.2249</v>
+        <v>4305402.37306</v>
       </c>
       <c r="I6" s="23" t="n">
         <f aca="false">H6+Inputs!B36</f>
-        <v>3846893.2249</v>
+        <v>5105402.37306</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4135,35 +4135,35 @@
       </c>
       <c r="B7" s="11" t="n">
         <f aca="false">'Roth Conversion'!J7</f>
-        <v>1019357.1015</v>
+        <v>2269357.1015</v>
       </c>
       <c r="C7" s="11" t="n">
         <f aca="false">MAX(0,C6*(1+Inputs!B19)-'Withdrawal Plan'!K7)</f>
-        <v>470184.984576</v>
+        <v>1101996.0576</v>
       </c>
       <c r="D7" s="11" t="n">
         <f aca="false">D6*(1+Inputs!B19)</f>
-        <v>16162.6088448</v>
+        <v>14693.280768</v>
       </c>
       <c r="E7" s="11" t="n">
         <f aca="false">E6*(1+Inputs!B19)</f>
-        <v>111668.9338368</v>
+        <v>73466.40384</v>
       </c>
       <c r="F7" s="11" t="n">
         <f aca="false">MAX(0,F6*(1+Inputs!B19)-'Withdrawal Plan'!M7)</f>
-        <v>142932.6621594</v>
+        <v>132647.3656218</v>
       </c>
       <c r="G7" s="11" t="n">
         <f aca="false">MAX(0,G6*(1+Inputs!B19)-'Withdrawal Plan'!L7)</f>
-        <v>1469328.0768</v>
+        <v>734664.0384</v>
       </c>
       <c r="H7" s="20" t="n">
         <f aca="false">SUM(B7:G7)</f>
-        <v>3229634.367717</v>
+        <v>4326824.2477298</v>
       </c>
       <c r="I7" s="21" t="n">
         <f aca="false">H7+Inputs!B36</f>
-        <v>3879634.367717</v>
+        <v>5126824.2477298</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4172,35 +4172,35 @@
       </c>
       <c r="B8" s="14" t="n">
         <f aca="false">'Roth Conversion'!J8</f>
-        <v>891936.6790375</v>
+        <v>2141936.6790375</v>
       </c>
       <c r="C8" s="14" t="n">
         <f aca="false">MAX(0,C7*(1+Inputs!B19)-'Withdrawal Plan'!K8)</f>
-        <v>507799.78334208</v>
+        <v>1190155.742208</v>
       </c>
       <c r="D8" s="14" t="n">
         <f aca="false">D7*(1+Inputs!B19)</f>
-        <v>17455.617552384</v>
+        <v>15868.74322944</v>
       </c>
       <c r="E8" s="14" t="n">
         <f aca="false">E7*(1+Inputs!B19)</f>
-        <v>120602.448543744</v>
+        <v>79343.7161472</v>
       </c>
       <c r="F8" s="14" t="n">
         <f aca="false">MAX(0,F7*(1+Inputs!B19)-'Withdrawal Plan'!M8)</f>
-        <v>151533.930063402</v>
+        <v>140425.809802794</v>
       </c>
       <c r="G8" s="14" t="n">
         <f aca="false">MAX(0,G7*(1+Inputs!B19)-'Withdrawal Plan'!L8)</f>
-        <v>1586874.322944</v>
+        <v>793437.161472</v>
       </c>
       <c r="H8" s="22" t="n">
         <f aca="false">SUM(B8:G8)</f>
-        <v>3276202.78148311</v>
+        <v>4361167.85189694</v>
       </c>
       <c r="I8" s="23" t="n">
         <f aca="false">H8+Inputs!B36</f>
-        <v>3926202.78148311</v>
+        <v>5161167.85189694</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4209,35 +4209,35 @@
       </c>
       <c r="B9" s="11" t="n">
         <f aca="false">'Roth Conversion'!J9</f>
-        <v>765606.996013437</v>
+        <v>2015606.99601344</v>
       </c>
       <c r="C9" s="11" t="n">
         <f aca="false">MAX(0,C8*(1+Inputs!B19)-'Withdrawal Plan'!K9)</f>
-        <v>548423.766009447</v>
+        <v>1285368.20158464</v>
       </c>
       <c r="D9" s="11" t="n">
         <f aca="false">D8*(1+Inputs!B19)</f>
-        <v>18852.0669565747</v>
+        <v>17138.2426877952</v>
       </c>
       <c r="E9" s="11" t="n">
         <f aca="false">E8*(1+Inputs!B19)</f>
-        <v>130250.644427244</v>
+        <v>85691.213438976</v>
       </c>
       <c r="F9" s="11" t="n">
         <f aca="false">MAX(0,F8*(1+Inputs!B19)-'Withdrawal Plan'!M9)</f>
-        <v>160681.632146287</v>
+        <v>148684.86226483</v>
       </c>
       <c r="G9" s="11" t="n">
         <f aca="false">MAX(0,G8*(1+Inputs!B19)-'Withdrawal Plan'!L9)</f>
-        <v>1713824.26877952</v>
+        <v>856912.13438976</v>
       </c>
       <c r="H9" s="20" t="n">
         <f aca="false">SUM(B9:G9)</f>
-        <v>3337639.37433251</v>
+        <v>4409401.65037944</v>
       </c>
       <c r="I9" s="21" t="n">
         <f aca="false">H9+Inputs!B36</f>
-        <v>3987639.37433251</v>
+        <v>5209401.65037944</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4246,35 +4246,35 @@
       </c>
       <c r="B10" s="14" t="n">
         <f aca="false">'Roth Conversion'!J10</f>
-        <v>640395.320913773</v>
+        <v>1890395.32091377</v>
       </c>
       <c r="C10" s="14" t="n">
         <f aca="false">MAX(0,C9*(1+Inputs!B19)-'Withdrawal Plan'!K10)</f>
-        <v>592297.667290203</v>
+        <v>1388197.65771141</v>
       </c>
       <c r="D10" s="14" t="n">
         <f aca="false">D9*(1+Inputs!B19)</f>
-        <v>20360.2323131007</v>
+        <v>18509.3021028188</v>
       </c>
       <c r="E10" s="14" t="n">
         <f aca="false">E9*(1+Inputs!B19)</f>
-        <v>140670.695981423</v>
+        <v>92546.5105140941</v>
       </c>
       <c r="F10" s="14" t="n">
         <f aca="false">MAX(0,F9*(1+Inputs!B19)-'Withdrawal Plan'!M10)</f>
-        <v>170412.399779693</v>
+        <v>157455.88830772</v>
       </c>
       <c r="G10" s="14" t="n">
         <f aca="false">MAX(0,G9*(1+Inputs!B19)-'Withdrawal Plan'!L10)</f>
-        <v>1850930.21028188</v>
+        <v>925465.105140941</v>
       </c>
       <c r="H10" s="22" t="n">
         <f aca="false">SUM(B10:G10)</f>
-        <v>3415066.52656007</v>
+        <v>4472569.78469076</v>
       </c>
       <c r="I10" s="23" t="n">
         <f aca="false">H10+Inputs!B36</f>
-        <v>4065066.52656007</v>
+        <v>5272569.78469076</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4283,35 +4283,35 @@
       </c>
       <c r="B11" s="17" t="n">
         <f aca="false">'Roth Conversion'!J11</f>
-        <v>516329.603936618</v>
+        <v>1766329.60393662</v>
       </c>
       <c r="C11" s="17" t="n">
         <f aca="false">MAX(0,C10*(1+Inputs!B19)-'Withdrawal Plan'!K11)</f>
-        <v>639681.480673419</v>
+        <v>1499253.47032833</v>
       </c>
       <c r="D11" s="17" t="n">
         <f aca="false">D10*(1+Inputs!B19)</f>
-        <v>21989.0508981488</v>
+        <v>19990.0462710443</v>
       </c>
       <c r="E11" s="17" t="n">
         <f aca="false">E10*(1+Inputs!B19)</f>
-        <v>151924.351659937</v>
+        <v>99950.2313552217</v>
       </c>
       <c r="F11" s="17" t="n">
         <f aca="false">MAX(0,F10*(1+Inputs!B19)-'Withdrawal Plan'!M11)</f>
-        <v>180765.440676857</v>
+        <v>166772.408287125</v>
       </c>
       <c r="G11" s="17" t="n">
         <f aca="false">MAX(0,G10*(1+Inputs!B19)-'Withdrawal Plan'!L11)</f>
-        <v>1999004.62710443</v>
+        <v>999502.313552217</v>
       </c>
       <c r="H11" s="24" t="n">
         <f aca="false">SUM(B11:G11)</f>
-        <v>3509694.55494941</v>
+        <v>4551798.07373055</v>
       </c>
       <c r="I11" s="25" t="n">
         <f aca="false">H11+Inputs!B36</f>
-        <v>4159694.55494941</v>
+        <v>5351798.07373055</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4320,35 +4320,35 @@
       </c>
       <c r="B12" s="17" t="n">
         <f aca="false">'Roth Conversion'!J12</f>
-        <v>393438.494035033</v>
+        <v>1643438.49403503</v>
       </c>
       <c r="C12" s="17" t="n">
         <f aca="false">MAX(0,C11*(1+Inputs!B19)-'Withdrawal Plan'!K12)</f>
-        <v>690855.999127292</v>
+        <v>1619193.74795459</v>
       </c>
       <c r="D12" s="17" t="n">
         <f aca="false">D11*(1+Inputs!B19)</f>
-        <v>23748.1749700007</v>
+        <v>21589.2499727279</v>
       </c>
       <c r="E12" s="17" t="n">
         <f aca="false">E11*(1+Inputs!B19)</f>
-        <v>164078.299792732</v>
+        <v>107946.249863639</v>
       </c>
       <c r="F12" s="17" t="n">
         <f aca="false">MAX(0,F11*(1+Inputs!B19)-'Withdrawal Plan'!M12)</f>
-        <v>191782.727291533</v>
+        <v>176670.252310623</v>
       </c>
       <c r="G12" s="17" t="n">
         <f aca="false">MAX(0,G11*(1+Inputs!B19)-'Withdrawal Plan'!L12)</f>
-        <v>2158924.99727279</v>
+        <v>1079462.49863639</v>
       </c>
       <c r="H12" s="24" t="n">
         <f aca="false">SUM(B12:G12)</f>
-        <v>3622828.69248938</v>
+        <v>4648300.49277301</v>
       </c>
       <c r="I12" s="25" t="n">
         <f aca="false">H12+Inputs!B36</f>
-        <v>4272828.69248938</v>
+        <v>5448300.49277301</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4357,35 +4357,35 @@
       </c>
       <c r="B13" s="17" t="n">
         <f aca="false">'Roth Conversion'!J13</f>
-        <v>271751.356385909</v>
+        <v>1521751.35638591</v>
       </c>
       <c r="C13" s="17" t="n">
         <f aca="false">MAX(0,C12*(1+Inputs!B19)-'Withdrawal Plan'!K13)</f>
-        <v>746124.479057476</v>
+        <v>1748729.24779096</v>
       </c>
       <c r="D13" s="17" t="n">
         <f aca="false">D12*(1+Inputs!B19)</f>
-        <v>25648.0289676007</v>
+        <v>23316.3899705461</v>
       </c>
       <c r="E13" s="17" t="n">
         <f aca="false">E12*(1+Inputs!B19)</f>
-        <v>177204.56377615</v>
+        <v>116581.949852731</v>
       </c>
       <c r="F13" s="17" t="n">
         <f aca="false">MAX(0,F12*(1+Inputs!B19)-'Withdrawal Plan'!M13)</f>
-        <v>203509.19940341</v>
+        <v>187187.726424027</v>
       </c>
       <c r="G13" s="17" t="n">
         <f aca="false">MAX(0,G12*(1+Inputs!B19)-'Withdrawal Plan'!L13)</f>
-        <v>2331638.99705461</v>
+        <v>1165819.49852731</v>
       </c>
       <c r="H13" s="24" t="n">
         <f aca="false">SUM(B13:G13)</f>
-        <v>3755876.62464516</v>
+        <v>4763386.16895148</v>
       </c>
       <c r="I13" s="25" t="n">
         <f aca="false">H13+Inputs!B36</f>
-        <v>4405876.62464516</v>
+        <v>5563386.16895148</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4394,35 +4394,35 @@
       </c>
       <c r="B14" s="17" t="n">
         <f aca="false">'Roth Conversion'!J14</f>
-        <v>151298.290295557</v>
+        <v>1401298.29029556</v>
       </c>
       <c r="C14" s="17" t="n">
         <f aca="false">MAX(0,C13*(1+Inputs!B19)-'Withdrawal Plan'!K14)</f>
-        <v>805814.437382074</v>
+        <v>1888627.58761424</v>
       </c>
       <c r="D14" s="17" t="n">
         <f aca="false">D13*(1+Inputs!B19)</f>
-        <v>27699.8712850088</v>
+        <v>25181.7011681898</v>
       </c>
       <c r="E14" s="17" t="n">
         <f aca="false">E13*(1+Inputs!B19)</f>
-        <v>191380.928878243</v>
+        <v>125908.505840949</v>
       </c>
       <c r="F14" s="17" t="n">
         <f aca="false">MAX(0,F13*(1+Inputs!B19)-'Withdrawal Plan'!M14)</f>
-        <v>215992.981980664</v>
+        <v>198365.791162931</v>
       </c>
       <c r="G14" s="17" t="n">
         <f aca="false">MAX(0,G13*(1+Inputs!B19)-'Withdrawal Plan'!L14)</f>
-        <v>2518170.11681898</v>
+        <v>1259085.05840949</v>
       </c>
       <c r="H14" s="24" t="n">
         <f aca="false">SUM(B14:G14)</f>
-        <v>3910356.62664053</v>
+        <v>4898466.93449135</v>
       </c>
       <c r="I14" s="25" t="n">
         <f aca="false">H14+Inputs!B36</f>
-        <v>4560356.62664053</v>
+        <v>5698466.93449135</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4431,35 +4431,35 @@
       </c>
       <c r="B15" s="17" t="n">
         <f aca="false">'Roth Conversion'!J15</f>
-        <v>32110.1475529454</v>
+        <v>1282110.14755295</v>
       </c>
       <c r="C15" s="17" t="n">
         <f aca="false">MAX(0,C14*(1+Inputs!B19)-'Withdrawal Plan'!K15)</f>
-        <v>870279.59237264</v>
+        <v>2039717.79462337</v>
       </c>
       <c r="D15" s="17" t="n">
         <f aca="false">D14*(1+Inputs!B19)</f>
-        <v>29915.8609878095</v>
+        <v>27196.237261645</v>
       </c>
       <c r="E15" s="17" t="n">
         <f aca="false">E14*(1+Inputs!B19)</f>
-        <v>206691.403188502</v>
+        <v>135981.186308225</v>
       </c>
       <c r="F15" s="17" t="n">
         <f aca="false">MAX(0,F14*(1+Inputs!B19)-'Withdrawal Plan'!M15)</f>
-        <v>229285.619495348</v>
+        <v>210248.253412196</v>
       </c>
       <c r="G15" s="17" t="n">
         <f aca="false">MAX(0,G14*(1+Inputs!B19)-'Withdrawal Plan'!L15)</f>
-        <v>2719623.7261645</v>
+        <v>1359811.86308225</v>
       </c>
       <c r="H15" s="24" t="n">
         <f aca="false">SUM(B15:G15)</f>
-        <v>4087906.34976174</v>
+        <v>5055065.48224064</v>
       </c>
       <c r="I15" s="25" t="n">
         <f aca="false">H15+Inputs!B36</f>
-        <v>4737906.34976174</v>
+        <v>5855065.48224064</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4468,35 +4468,35 @@
       </c>
       <c r="B16" s="17" t="n">
         <f aca="false">'Roth Conversion'!J16</f>
-        <v>0</v>
+        <v>1164218.55124177</v>
       </c>
       <c r="C16" s="17" t="n">
         <f aca="false">MAX(0,C15*(1+Inputs!B19)-'Withdrawal Plan'!K16)</f>
-        <v>939901.959762451</v>
+        <v>2202895.21819324</v>
       </c>
       <c r="D16" s="17" t="n">
         <f aca="false">D15*(1+Inputs!B19)</f>
-        <v>32309.1298668342</v>
+        <v>29371.9362425766</v>
       </c>
       <c r="E16" s="17" t="n">
         <f aca="false">E15*(1+Inputs!B19)</f>
-        <v>223226.715443582</v>
+        <v>146859.681212883</v>
       </c>
       <c r="F16" s="17" t="n">
         <f aca="false">MAX(0,F15*(1+Inputs!B19)-'Withdrawal Plan'!M16)</f>
-        <v>243442.327959018</v>
+        <v>222881.972589215</v>
       </c>
       <c r="G16" s="17" t="n">
         <f aca="false">MAX(0,G15*(1+Inputs!B19)-'Withdrawal Plan'!L16)</f>
-        <v>2937193.62425766</v>
+        <v>1468596.81212883</v>
       </c>
       <c r="H16" s="24" t="n">
         <f aca="false">SUM(B16:G16)</f>
-        <v>4376073.75728955</v>
+        <v>5234824.17160852</v>
       </c>
       <c r="I16" s="25" t="n">
         <f aca="false">H16+Inputs!B36</f>
-        <v>5026073.75728955</v>
+        <v>6034824.17160852</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4505,35 +4505,35 @@
       </c>
       <c r="B17" s="17" t="n">
         <f aca="false">'Roth Conversion'!J17</f>
-        <v>0</v>
+        <v>1047655.91502281</v>
       </c>
       <c r="C17" s="17" t="n">
         <f aca="false">MAX(0,C16*(1+Inputs!B19)-'Withdrawal Plan'!K17)</f>
-        <v>1015094.11654345</v>
+        <v>2379126.8356487</v>
       </c>
       <c r="D17" s="17" t="n">
         <f aca="false">D16*(1+Inputs!B19)</f>
-        <v>34893.860256181</v>
+        <v>31721.6911419827</v>
       </c>
       <c r="E17" s="17" t="n">
         <f aca="false">E16*(1+Inputs!B19)</f>
-        <v>241084.852679069</v>
+        <v>158608.455709914</v>
       </c>
       <c r="F17" s="17" t="n">
         <f aca="false">MAX(0,F16*(1+Inputs!B19)-'Withdrawal Plan'!M17)</f>
-        <v>258522.266044984</v>
+        <v>236317.082245596</v>
       </c>
       <c r="G17" s="17" t="n">
         <f aca="false">MAX(0,G16*(1+Inputs!B19)-'Withdrawal Plan'!L17)</f>
-        <v>3172169.11419827</v>
+        <v>1586084.55709914</v>
       </c>
       <c r="H17" s="24" t="n">
         <f aca="false">SUM(B17:G17)</f>
-        <v>4721764.20972195</v>
+        <v>5439514.53686815</v>
       </c>
       <c r="I17" s="25" t="n">
         <f aca="false">H17+Inputs!B36</f>
-        <v>5371764.20972195</v>
+        <v>6239514.53686815</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4542,35 +4542,35 @@
       </c>
       <c r="B18" s="17" t="n">
         <f aca="false">'Roth Conversion'!J18</f>
-        <v>0</v>
+        <v>932455.462898383</v>
       </c>
       <c r="C18" s="17" t="n">
         <f aca="false">MAX(0,C17*(1+Inputs!B19)-'Withdrawal Plan'!K18)</f>
-        <v>1096301.64586692</v>
+        <v>2569456.9825006</v>
       </c>
       <c r="D18" s="17" t="n">
         <f aca="false">D17*(1+Inputs!B19)</f>
-        <v>37685.3690766755</v>
+        <v>34259.4264333413</v>
       </c>
       <c r="E18" s="17" t="n">
         <f aca="false">E17*(1+Inputs!B19)</f>
-        <v>260371.640893394</v>
+        <v>171297.132166707</v>
       </c>
       <c r="F18" s="17" t="n">
         <f aca="false">MAX(0,F17*(1+Inputs!B19)-'Withdrawal Plan'!M18)</f>
-        <v>274588.82677029</v>
+        <v>250607.228266951</v>
       </c>
       <c r="G18" s="17" t="n">
         <f aca="false">MAX(0,G17*(1+Inputs!B19)-'Withdrawal Plan'!L18)</f>
-        <v>3425942.64333413</v>
+        <v>1712971.32166707</v>
       </c>
       <c r="H18" s="24" t="n">
         <f aca="false">SUM(B18:G18)</f>
-        <v>5094890.12594142</v>
+        <v>5671047.55393305</v>
       </c>
       <c r="I18" s="25" t="n">
         <f aca="false">H18+Inputs!B36</f>
-        <v>5744890.12594142</v>
+        <v>6471047.55393305</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4579,35 +4579,35 @@
       </c>
       <c r="B19" s="17" t="n">
         <f aca="false">'Roth Conversion'!J19</f>
-        <v>0</v>
+        <v>818651.249470843</v>
       </c>
       <c r="C19" s="17" t="n">
         <f aca="false">MAX(0,C18*(1+Inputs!B19)-'Withdrawal Plan'!K19)</f>
-        <v>1184005.77753628</v>
+        <v>2775013.54110065</v>
       </c>
       <c r="D19" s="17" t="n">
         <f aca="false">D18*(1+Inputs!B19)</f>
-        <v>40700.1986028095</v>
+        <v>37000.1805480087</v>
       </c>
       <c r="E19" s="17" t="n">
         <f aca="false">E18*(1+Inputs!B19)</f>
-        <v>281201.372164866</v>
+        <v>185000.902740043</v>
       </c>
       <c r="F19" s="17" t="n">
         <f aca="false">MAX(0,F18*(1+Inputs!B19)-'Withdrawal Plan'!M19)</f>
-        <v>291709.951325705</v>
+        <v>265809.824942099</v>
       </c>
       <c r="G19" s="17" t="n">
         <f aca="false">MAX(0,G18*(1+Inputs!B19)-'Withdrawal Plan'!L19)</f>
-        <v>3700018.05480087</v>
+        <v>1850009.02740043</v>
       </c>
       <c r="H19" s="24" t="n">
         <f aca="false">SUM(B19:G19)</f>
-        <v>5497635.35443052</v>
+        <v>5931484.72620207</v>
       </c>
       <c r="I19" s="25" t="n">
         <f aca="false">H19+Inputs!B36</f>
-        <v>6147635.35443052</v>
+        <v>6731484.72620207</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4616,35 +4616,35 @@
       </c>
       <c r="B20" s="17" t="n">
         <f aca="false">'Roth Conversion'!J20</f>
-        <v>0</v>
+        <v>706278.180707614</v>
       </c>
       <c r="C20" s="17" t="n">
         <f aca="false">MAX(0,C19*(1+Inputs!B19)-'Withdrawal Plan'!K20)</f>
-        <v>1278726.23973918</v>
+        <v>2997014.6243887</v>
       </c>
       <c r="D20" s="17" t="n">
         <f aca="false">D19*(1+Inputs!B19)</f>
-        <v>43956.2144910343</v>
+        <v>39960.1949918494</v>
       </c>
       <c r="E20" s="17" t="n">
         <f aca="false">E19*(1+Inputs!B19)</f>
-        <v>303697.481938055</v>
+        <v>199800.974959247</v>
       </c>
       <c r="F20" s="17" t="n">
         <f aca="false">MAX(0,F19*(1+Inputs!B19)-'Withdrawal Plan'!M20)</f>
-        <v>309958.466766243</v>
+        <v>281986.330271949</v>
       </c>
       <c r="G20" s="17" t="n">
         <f aca="false">MAX(0,G19*(1+Inputs!B19)-'Withdrawal Plan'!L20)</f>
-        <v>3996019.49918493</v>
+        <v>1998009.74959247</v>
       </c>
       <c r="H20" s="24" t="n">
         <f aca="false">SUM(B20:G20)</f>
-        <v>5932357.90211945</v>
+        <v>6223050.05491183</v>
       </c>
       <c r="I20" s="25" t="n">
         <f aca="false">H20+Inputs!B36</f>
-        <v>6582357.90211945</v>
+        <v>7023050.05491183</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4653,35 +4653,35 @@
       </c>
       <c r="B21" s="17" t="n">
         <f aca="false">'Roth Conversion'!J21</f>
-        <v>0</v>
+        <v>595372.035225304</v>
       </c>
       <c r="C21" s="17" t="n">
         <f aca="false">MAX(0,C20*(1+Inputs!B19)-'Withdrawal Plan'!K21)</f>
-        <v>1381024.33891831</v>
+        <v>3236775.7943398</v>
       </c>
       <c r="D21" s="17" t="n">
         <f aca="false">D20*(1+Inputs!B19)</f>
-        <v>47472.711650317</v>
+        <v>43157.0105911973</v>
       </c>
       <c r="E21" s="17" t="n">
         <f aca="false">E20*(1+Inputs!B19)</f>
-        <v>327993.2804931</v>
+        <v>215785.052955986</v>
       </c>
       <c r="F21" s="17" t="n">
         <f aca="false">MAX(0,F20*(1+Inputs!B19)-'Withdrawal Plan'!M21)</f>
-        <v>329412.449408749</v>
+        <v>299202.54199491</v>
       </c>
       <c r="G21" s="17" t="n">
         <f aca="false">MAX(0,G20*(1+Inputs!B19)-'Withdrawal Plan'!L21)</f>
-        <v>4315701.05911973</v>
+        <v>2157850.52955986</v>
       </c>
       <c r="H21" s="24" t="n">
         <f aca="false">SUM(B21:G21)</f>
-        <v>6401603.83959021</v>
+        <v>6548142.96466706</v>
       </c>
       <c r="I21" s="25" t="n">
         <f aca="false">H21+Inputs!B36</f>
-        <v>7051603.83959021</v>
+        <v>7348142.96466706</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4690,35 +4690,35 @@
       </c>
       <c r="B22" s="17" t="n">
         <f aca="false">'Roth Conversion'!J22</f>
-        <v>0</v>
+        <v>485969.486105936</v>
       </c>
       <c r="C22" s="17" t="n">
         <f aca="false">MAX(0,C21*(1+Inputs!B19)-'Withdrawal Plan'!K22)</f>
-        <v>1491506.28603178</v>
+        <v>3495717.85788698</v>
       </c>
       <c r="D22" s="17" t="n">
         <f aca="false">D21*(1+Inputs!B19)</f>
-        <v>51270.5285823424</v>
+        <v>46609.5714384931</v>
       </c>
       <c r="E22" s="17" t="n">
         <f aca="false">E21*(1+Inputs!B19)</f>
-        <v>354232.742932547</v>
+        <v>233047.857192465</v>
       </c>
       <c r="F22" s="17" t="n">
         <f aca="false">MAX(0,F21*(1+Inputs!B19)-'Withdrawal Plan'!M22)</f>
-        <v>350155.615927715</v>
+        <v>317528.915920769</v>
       </c>
       <c r="G22" s="17" t="n">
         <f aca="false">MAX(0,G21*(1+Inputs!B19)-'Withdrawal Plan'!L22)</f>
-        <v>4660957.14384931</v>
+        <v>2330478.57192465</v>
       </c>
       <c r="H22" s="24" t="n">
         <f aca="false">SUM(B22:G22)</f>
-        <v>6908122.31732369</v>
+        <v>6909352.2604693</v>
       </c>
       <c r="I22" s="25" t="n">
         <f aca="false">H22+Inputs!B36</f>
-        <v>7558122.31732369</v>
+        <v>7709352.2604693</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4727,35 +4727,35 @@
       </c>
       <c r="B23" s="17" t="n">
         <f aca="false">'Roth Conversion'!J23</f>
-        <v>0</v>
+        <v>378108.123258585</v>
       </c>
       <c r="C23" s="17" t="n">
         <f aca="false">MAX(0,C22*(1+Inputs!B19)-'Withdrawal Plan'!K23)</f>
-        <v>1610826.78891432</v>
+        <v>3775375.28651794</v>
       </c>
       <c r="D23" s="17" t="n">
         <f aca="false">D22*(1+Inputs!B19)</f>
-        <v>55372.1708689298</v>
+        <v>50338.3371535725</v>
       </c>
       <c r="E23" s="17" t="n">
         <f aca="false">E22*(1+Inputs!B19)</f>
-        <v>382571.362367151</v>
+        <v>251691.685767863</v>
       </c>
       <c r="F23" s="17" t="n">
         <f aca="false">MAX(0,F22*(1+Inputs!B19)-'Withdrawal Plan'!M23)</f>
-        <v>372277.744296511</v>
+        <v>337040.90828901</v>
       </c>
       <c r="G23" s="17" t="n">
         <f aca="false">MAX(0,G22*(1+Inputs!B19)-'Withdrawal Plan'!L23)</f>
-        <v>5033833.71535725</v>
+        <v>2516916.85767863</v>
       </c>
       <c r="H23" s="24" t="n">
         <f aca="false">SUM(B23:G23)</f>
-        <v>7454881.78180417</v>
+        <v>7309471.1986656</v>
       </c>
       <c r="I23" s="25" t="n">
         <f aca="false">H23+Inputs!B36</f>
-        <v>8104881.78180417</v>
+        <v>8109471.1986656</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix guest age to 56 and wife age calculation
</commit_message>
<xml_diff>
--- a/retirement_planner.xlsx
+++ b/retirement_planner.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="128">
   <si>
     <t xml:space="preserve">RETIREMENT PLANNING MODEL — INPUTS</t>
   </si>
@@ -282,7 +282,7 @@
 Surplus ($)</t>
   </si>
   <si>
-    <t xml:space="preserve">PORTFOLIO BALANCE PROJECTION  (Ages 65–85)</t>
+    <t xml:space="preserve">PORTFOLIO BALANCE PROJECTION  (Ages 56–85)</t>
   </si>
   <si>
     <t xml:space="preserve">Trad 401k
@@ -315,6 +315,9 @@
   <si>
     <t xml:space="preserve">Net Worth
 +Home ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blue rows = working years (accumulation)  ·  Orange rows = RMD years (age 73+)  ·  White/cream = retirement years</t>
   </si>
   <si>
     <t xml:space="preserve">SOCIAL SECURITY START AGE COMPARISON</t>
@@ -446,7 +449,7 @@
     <numFmt numFmtId="165" formatCode="\$#,##0;&quot;($&quot;#,##0\);\-"/>
     <numFmt numFmtId="166" formatCode="0.0%;\(0.0%\);\-"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -557,6 +560,14 @@
     <font>
       <b val="true"/>
       <sz val="10"/>
+      <color rgb="FF1A3A6B"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
       <family val="0"/>
@@ -570,7 +581,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -616,6 +627,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF0E8"/>
+        <bgColor rgb="FFF8F4ED"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEAF0FB"/>
         <bgColor rgb="FFF8F4ED"/>
       </patternFill>
     </fill>
@@ -682,7 +699,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="43">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -787,7 +804,27 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -811,11 +848,11 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -865,7 +902,7 @@
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FFFFFDF7"/>
-      <rgbColor rgb="FFF8F4ED"/>
+      <rgbColor rgb="FFEAF0FB"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
@@ -879,7 +916,7 @@
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFF8F4ED"/>
       <rgbColor rgb="FFEFE9DF"/>
       <rgbColor rgb="FFFFF0E8"/>
       <rgbColor rgb="FF99CCFF"/>
@@ -1131,7 +1168,7 @@
         <v>4</v>
       </c>
       <c r="B4" s="5" t="n">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>5</v>
@@ -2560,7 +2597,7 @@
         <v>16500</v>
       </c>
       <c r="E3" s="11" t="n">
-        <f aca="false">IF(55&lt;65,Inputs!B35*12,0)</f>
+        <f aca="false">IF(60&lt;65,Inputs!B35*12,0)</f>
         <v>9600</v>
       </c>
       <c r="F3" s="11" t="n">
@@ -2576,7 +2613,7 @@
         <v>0</v>
       </c>
       <c r="I3" s="11" t="n">
-        <f aca="false">IF(55&gt;=Inputs!B26,Inputs!B23*12*0.5*(1+Inputs!B21)^MAX(0,55-Inputs!B26),0)</f>
+        <f aca="false">IF(60&gt;=Inputs!B26,Inputs!B23*12*0.5*(1+Inputs!B21)^MAX(0,60-Inputs!B26),0)</f>
         <v>0</v>
       </c>
       <c r="J3" s="11" t="n">
@@ -2625,7 +2662,7 @@
         <v>16500</v>
       </c>
       <c r="E4" s="14" t="n">
-        <f aca="false">IF(56&lt;65,Inputs!B35*12,0)</f>
+        <f aca="false">IF(61&lt;65,Inputs!B35*12,0)</f>
         <v>9600</v>
       </c>
       <c r="F4" s="14" t="n">
@@ -2641,7 +2678,7 @@
         <v>0</v>
       </c>
       <c r="I4" s="14" t="n">
-        <f aca="false">IF(56&gt;=Inputs!B26,Inputs!B23*12*0.5*(1+Inputs!B21)^MAX(0,56-Inputs!B26),0)</f>
+        <f aca="false">IF(61&gt;=Inputs!B26,Inputs!B23*12*0.5*(1+Inputs!B21)^MAX(0,61-Inputs!B26),0)</f>
         <v>0</v>
       </c>
       <c r="J4" s="14" t="n">
@@ -2690,7 +2727,7 @@
         <v>16500</v>
       </c>
       <c r="E5" s="11" t="n">
-        <f aca="false">IF(57&lt;65,Inputs!B35*12,0)</f>
+        <f aca="false">IF(62&lt;65,Inputs!B35*12,0)</f>
         <v>9600</v>
       </c>
       <c r="F5" s="11" t="n">
@@ -2706,7 +2743,7 @@
         <v>47664</v>
       </c>
       <c r="I5" s="11" t="n">
-        <f aca="false">IF(57&gt;=Inputs!B26,Inputs!B23*12*0.5*(1+Inputs!B21)^MAX(0,57-Inputs!B26),0)</f>
+        <f aca="false">IF(62&gt;=Inputs!B26,Inputs!B23*12*0.5*(1+Inputs!B21)^MAX(0,62-Inputs!B26),0)</f>
         <v>0</v>
       </c>
       <c r="J5" s="11" t="n">
@@ -2755,7 +2792,7 @@
         <v>16500</v>
       </c>
       <c r="E6" s="14" t="n">
-        <f aca="false">IF(58&lt;65,Inputs!B35*12,0)</f>
+        <f aca="false">IF(63&lt;65,Inputs!B35*12,0)</f>
         <v>9600</v>
       </c>
       <c r="F6" s="14" t="n">
@@ -2771,7 +2808,7 @@
         <v>48855.6</v>
       </c>
       <c r="I6" s="14" t="n">
-        <f aca="false">IF(58&gt;=Inputs!B26,Inputs!B23*12*0.5*(1+Inputs!B21)^MAX(0,58-Inputs!B26),0)</f>
+        <f aca="false">IF(63&gt;=Inputs!B26,Inputs!B23*12*0.5*(1+Inputs!B21)^MAX(0,63-Inputs!B26),0)</f>
         <v>0</v>
       </c>
       <c r="J6" s="14" t="n">
@@ -2820,7 +2857,7 @@
         <v>16500</v>
       </c>
       <c r="E7" s="11" t="n">
-        <f aca="false">IF(59&lt;65,Inputs!B35*12,0)</f>
+        <f aca="false">IF(64&lt;65,Inputs!B35*12,0)</f>
         <v>9600</v>
       </c>
       <c r="F7" s="11" t="n">
@@ -2836,7 +2873,7 @@
         <v>50076.99</v>
       </c>
       <c r="I7" s="11" t="n">
-        <f aca="false">IF(59&gt;=Inputs!B26,Inputs!B23*12*0.5*(1+Inputs!B21)^MAX(0,59-Inputs!B26),0)</f>
+        <f aca="false">IF(64&gt;=Inputs!B26,Inputs!B23*12*0.5*(1+Inputs!B21)^MAX(0,64-Inputs!B26),0)</f>
         <v>0</v>
       </c>
       <c r="J7" s="11" t="n">
@@ -2885,8 +2922,8 @@
         <v>16500</v>
       </c>
       <c r="E8" s="14" t="n">
-        <f aca="false">IF(60&lt;65,Inputs!B35*12,0)</f>
-        <v>9600</v>
+        <f aca="false">IF(65&lt;65,Inputs!B35*12,0)</f>
+        <v>0</v>
       </c>
       <c r="F8" s="14" t="n">
         <f aca="false">Inputs!B33*12*(1+Inputs!B34)^5</f>
@@ -2894,15 +2931,15 @@
       </c>
       <c r="G8" s="22" t="n">
         <f aca="false">B8+C8+D8+E8+F8</f>
-        <v>162312.36730995</v>
+        <v>152712.36730995</v>
       </c>
       <c r="H8" s="14" t="n">
         <f aca="false">IF(70&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,70-Inputs!B25),0)</f>
         <v>51328.91475</v>
       </c>
       <c r="I8" s="14" t="n">
-        <f aca="false">IF(60&gt;=Inputs!B26,Inputs!B23*12*0.5*(1+Inputs!B21)^MAX(0,60-Inputs!B26),0)</f>
-        <v>0</v>
+        <f aca="false">IF(65&gt;=Inputs!B26,Inputs!B23*12*0.5*(1+Inputs!B21)^MAX(0,65-Inputs!B26),0)</f>
+        <v>23832</v>
       </c>
       <c r="J8" s="14" t="n">
         <f aca="false">'Roth Conversion'!E8</f>
@@ -2930,7 +2967,7 @@
       </c>
       <c r="P8" s="23" t="n">
         <f aca="false">H8+I8+J8+K8+L8-G8-N8-O8</f>
-        <v>-19416.7110083113</v>
+        <v>14015.2889916887</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2950,8 +2987,8 @@
         <v>16500</v>
       </c>
       <c r="E9" s="11" t="n">
-        <f aca="false">IF(61&lt;65,Inputs!B35*12,0)</f>
-        <v>9600</v>
+        <f aca="false">IF(66&lt;65,Inputs!B35*12,0)</f>
+        <v>0</v>
       </c>
       <c r="F9" s="11" t="n">
         <f aca="false">Inputs!B33*12*(1+Inputs!B34)^6</f>
@@ -2959,15 +2996,15 @@
       </c>
       <c r="G9" s="20" t="n">
         <f aca="false">B9+C9+D9+E9+F9</f>
-        <v>165375.405230624</v>
+        <v>155775.405230624</v>
       </c>
       <c r="H9" s="11" t="n">
         <f aca="false">IF(71&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,71-Inputs!B25),0)</f>
         <v>52612.13761875</v>
       </c>
       <c r="I9" s="11" t="n">
-        <f aca="false">IF(61&gt;=Inputs!B26,Inputs!B23*12*0.5*(1+Inputs!B21)^MAX(0,61-Inputs!B26),0)</f>
-        <v>0</v>
+        <f aca="false">IF(66&gt;=Inputs!B26,Inputs!B23*12*0.5*(1+Inputs!B21)^MAX(0,66-Inputs!B26),0)</f>
+        <v>24427.8</v>
       </c>
       <c r="J9" s="11" t="n">
         <f aca="false">'Roth Conversion'!E9</f>
@@ -2995,7 +3032,7 @@
       </c>
       <c r="P9" s="21" t="n">
         <f aca="false">H9+I9+J9+K9+L9-G9-N9-O9</f>
-        <v>-22217.7853964438</v>
+        <v>11810.0146035562</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3015,8 +3052,8 @@
         <v>16500</v>
       </c>
       <c r="E10" s="14" t="n">
-        <f aca="false">IF(62&lt;65,Inputs!B35*12,0)</f>
-        <v>9600</v>
+        <f aca="false">IF(67&lt;65,Inputs!B35*12,0)</f>
+        <v>0</v>
       </c>
       <c r="F10" s="14" t="n">
         <f aca="false">Inputs!B33*12*(1+Inputs!B34)^7</f>
@@ -3024,15 +3061,15 @@
       </c>
       <c r="G10" s="22" t="n">
         <f aca="false">B10+C10+D10+E10+F10</f>
-        <v>168533.167633986</v>
+        <v>158933.167633986</v>
       </c>
       <c r="H10" s="14" t="n">
         <f aca="false">IF(72&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,72-Inputs!B25),0)</f>
         <v>53927.4410592187</v>
       </c>
       <c r="I10" s="14" t="n">
-        <f aca="false">IF(62&gt;=Inputs!B26,Inputs!B23*12*0.5*(1+Inputs!B21)^MAX(0,62-Inputs!B26),0)</f>
-        <v>0</v>
+        <f aca="false">IF(67&gt;=Inputs!B26,Inputs!B23*12*0.5*(1+Inputs!B21)^MAX(0,67-Inputs!B26),0)</f>
+        <v>25038.495</v>
       </c>
       <c r="J10" s="14" t="n">
         <f aca="false">'Roth Conversion'!E10</f>
@@ -3060,7 +3097,7 @@
       </c>
       <c r="P10" s="23" t="n">
         <f aca="false">H10+I10+J10+K10+L10-G10-N10-O10</f>
-        <v>-25107.0351789518</v>
+        <v>9531.45982104821</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3080,8 +3117,8 @@
         <v>16500</v>
       </c>
       <c r="E11" s="17" t="n">
-        <f aca="false">IF(63&lt;65,Inputs!B35*12,0)</f>
-        <v>9600</v>
+        <f aca="false">IF(68&lt;65,Inputs!B35*12,0)</f>
+        <v>0</v>
       </c>
       <c r="F11" s="17" t="n">
         <f aca="false">Inputs!B33*12*(1+Inputs!B34)^8</f>
@@ -3089,15 +3126,15 @@
       </c>
       <c r="G11" s="24" t="n">
         <f aca="false">B11+C11+D11+E11+F11</f>
-        <v>171788.637921772</v>
+        <v>162188.637921772</v>
       </c>
       <c r="H11" s="17" t="n">
         <f aca="false">IF(73&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,73-Inputs!B25),0)</f>
         <v>55275.6270856992</v>
       </c>
       <c r="I11" s="17" t="n">
-        <f aca="false">IF(63&gt;=Inputs!B26,Inputs!B23*12*0.5*(1+Inputs!B21)^MAX(0,63-Inputs!B26),0)</f>
-        <v>0</v>
+        <f aca="false">IF(68&gt;=Inputs!B26,Inputs!B23*12*0.5*(1+Inputs!B21)^MAX(0,68-Inputs!B26),0)</f>
+        <v>25664.457375</v>
       </c>
       <c r="J11" s="17" t="n">
         <f aca="false">'Roth Conversion'!E11</f>
@@ -3125,7 +3162,7 @@
       </c>
       <c r="P11" s="25" t="n">
         <f aca="false">H11+I11+J11+K11+L11-G11-N11-O11</f>
-        <v>-28087.2800303614</v>
+        <v>7177.17734463854</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3145,8 +3182,8 @@
         <v>16500</v>
       </c>
       <c r="E12" s="17" t="n">
-        <f aca="false">IF(64&lt;65,Inputs!B35*12,0)</f>
-        <v>9600</v>
+        <f aca="false">IF(69&lt;65,Inputs!B35*12,0)</f>
+        <v>0</v>
       </c>
       <c r="F12" s="17" t="n">
         <f aca="false">Inputs!B33*12*(1+Inputs!B34)^9</f>
@@ -3154,15 +3191,15 @@
       </c>
       <c r="G12" s="24" t="n">
         <f aca="false">B12+C12+D12+E12+F12</f>
-        <v>175144.896081129</v>
+        <v>165544.896081129</v>
       </c>
       <c r="H12" s="17" t="n">
         <f aca="false">IF(74&gt;=Inputs!B25,IF(Inputs!B25=65,Inputs!B22*12,IF(Inputs!B25=70,Inputs!B24*12,Inputs!B23*12))*(1+Inputs!B21)^MAX(0,74-Inputs!B25),0)</f>
         <v>56657.5177628417</v>
       </c>
       <c r="I12" s="17" t="n">
-        <f aca="false">IF(64&gt;=Inputs!B26,Inputs!B23*12*0.5*(1+Inputs!B21)^MAX(0,64-Inputs!B26),0)</f>
-        <v>0</v>
+        <f aca="false">IF(69&gt;=Inputs!B26,Inputs!B23*12*0.5*(1+Inputs!B21)^MAX(0,69-Inputs!B26),0)</f>
+        <v>26306.068809375</v>
       </c>
       <c r="J12" s="17" t="n">
         <f aca="false">'Roth Conversion'!E12</f>
@@ -3190,7 +3227,7 @@
       </c>
       <c r="P12" s="25" t="n">
         <f aca="false">H12+I12+J12+K12+L12-G12-N12-O12</f>
-        <v>-31161.4321174336</v>
+        <v>4744.63669194142</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3210,7 +3247,7 @@
         <v>16500</v>
       </c>
       <c r="E13" s="17" t="n">
-        <f aca="false">IF(65&lt;65,Inputs!B35*12,0)</f>
+        <f aca="false">IF(70&lt;65,Inputs!B35*12,0)</f>
         <v>0</v>
       </c>
       <c r="F13" s="17" t="n">
@@ -3226,8 +3263,8 @@
         <v>58073.9557069127</v>
       </c>
       <c r="I13" s="17" t="n">
-        <f aca="false">IF(65&gt;=Inputs!B26,Inputs!B23*12*0.5*(1+Inputs!B21)^MAX(0,65-Inputs!B26),0)</f>
-        <v>23832</v>
+        <f aca="false">IF(70&gt;=Inputs!B26,Inputs!B23*12*0.5*(1+Inputs!B21)^MAX(0,70-Inputs!B26),0)</f>
+        <v>26963.7205296094</v>
       </c>
       <c r="J13" s="17" t="n">
         <f aca="false">'Roth Conversion'!E13</f>
@@ -3255,7 +3292,7 @@
       </c>
       <c r="P13" s="25" t="n">
         <f aca="false">H13+I13+J13+K13+L13-G13-N13-O13</f>
-        <v>-900.499248564507</v>
+        <v>2231.22128104485</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3275,7 +3312,7 @@
         <v>16500</v>
       </c>
       <c r="E14" s="17" t="n">
-        <f aca="false">IF(66&lt;65,Inputs!B35*12,0)</f>
+        <f aca="false">IF(71&lt;65,Inputs!B35*12,0)</f>
         <v>0</v>
       </c>
       <c r="F14" s="17" t="n">
@@ -3291,8 +3328,8 @@
         <v>59525.8045995855</v>
       </c>
       <c r="I14" s="17" t="n">
-        <f aca="false">IF(66&gt;=Inputs!B26,Inputs!B23*12*0.5*(1+Inputs!B21)^MAX(0,66-Inputs!B26),0)</f>
-        <v>24427.8</v>
+        <f aca="false">IF(71&gt;=Inputs!B26,Inputs!B23*12*0.5*(1+Inputs!B21)^MAX(0,71-Inputs!B26),0)</f>
+        <v>27637.8135428496</v>
       </c>
       <c r="J14" s="17" t="n">
         <f aca="false">'Roth Conversion'!E14</f>
@@ -3320,7 +3357,7 @@
       </c>
       <c r="P14" s="25" t="n">
         <f aca="false">H14+I14+J14+K14+L14-G14-N14-O14</f>
-        <v>-3575.78813588932</v>
+        <v>-365.774593039748</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3340,7 +3377,7 @@
         <v>16500</v>
       </c>
       <c r="E15" s="17" t="n">
-        <f aca="false">IF(67&lt;65,Inputs!B35*12,0)</f>
+        <f aca="false">IF(72&lt;65,Inputs!B35*12,0)</f>
         <v>0</v>
       </c>
       <c r="F15" s="17" t="n">
@@ -3356,8 +3393,8 @@
         <v>61013.9497145751</v>
       </c>
       <c r="I15" s="17" t="n">
-        <f aca="false">IF(67&gt;=Inputs!B26,Inputs!B23*12*0.5*(1+Inputs!B21)^MAX(0,67-Inputs!B26),0)</f>
-        <v>25038.495</v>
+        <f aca="false">IF(72&gt;=Inputs!B26,Inputs!B23*12*0.5*(1+Inputs!B21)^MAX(0,72-Inputs!B26),0)</f>
+        <v>28328.7588814208</v>
       </c>
       <c r="J15" s="17" t="n">
         <f aca="false">'Roth Conversion'!E15</f>
@@ -3385,7 +3422,7 @@
       </c>
       <c r="P15" s="25" t="n">
         <f aca="false">H15+I15+J15+K15+L15-G15-N15-O15</f>
-        <v>-6339.4127743663</v>
+        <v>-3049.14889294547</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3405,7 +3442,7 @@
         <v>16500</v>
       </c>
       <c r="E16" s="17" t="n">
-        <f aca="false">IF(68&lt;65,Inputs!B35*12,0)</f>
+        <f aca="false">IF(73&lt;65,Inputs!B35*12,0)</f>
         <v>0</v>
       </c>
       <c r="F16" s="17" t="n">
@@ -3421,8 +3458,8 @@
         <v>62539.2984574395</v>
       </c>
       <c r="I16" s="17" t="n">
-        <f aca="false">IF(68&gt;=Inputs!B26,Inputs!B23*12*0.5*(1+Inputs!B21)^MAX(0,68-Inputs!B26),0)</f>
-        <v>25664.457375</v>
+        <f aca="false">IF(73&gt;=Inputs!B26,Inputs!B23*12*0.5*(1+Inputs!B21)^MAX(0,73-Inputs!B26),0)</f>
+        <v>29036.9778534564</v>
       </c>
       <c r="J16" s="17" t="n">
         <f aca="false">'Roth Conversion'!E16</f>
@@ -3450,7 +3487,7 @@
       </c>
       <c r="P16" s="25" t="n">
         <f aca="false">H16+I16+J16+K16+L16-G16-N16-O16</f>
-        <v>-9194.31556729504</v>
+        <v>-5821.79508883867</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3470,7 +3507,7 @@
         <v>16500</v>
       </c>
       <c r="E17" s="17" t="n">
-        <f aca="false">IF(69&lt;65,Inputs!B35*12,0)</f>
+        <f aca="false">IF(74&lt;65,Inputs!B35*12,0)</f>
         <v>0</v>
       </c>
       <c r="F17" s="17" t="n">
@@ -3486,8 +3523,8 @@
         <v>64102.7809188755</v>
       </c>
       <c r="I17" s="17" t="n">
-        <f aca="false">IF(69&gt;=Inputs!B26,Inputs!B23*12*0.5*(1+Inputs!B21)^MAX(0,69-Inputs!B26),0)</f>
-        <v>26306.068809375</v>
+        <f aca="false">IF(74&gt;=Inputs!B26,Inputs!B23*12*0.5*(1+Inputs!B21)^MAX(0,74-Inputs!B26),0)</f>
+        <v>29762.9022997928</v>
       </c>
       <c r="J17" s="17" t="n">
         <f aca="false">'Roth Conversion'!E17</f>
@@ -3515,7 +3552,7 @@
       </c>
       <c r="P17" s="25" t="n">
         <f aca="false">H17+I17+J17+K17+L17-G17-N17-O17</f>
-        <v>-12143.539018526</v>
+        <v>-8686.70552810827</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3535,7 +3572,7 @@
         <v>16500</v>
       </c>
       <c r="E18" s="17" t="n">
-        <f aca="false">IF(70&lt;65,Inputs!B35*12,0)</f>
+        <f aca="false">IF(75&lt;65,Inputs!B35*12,0)</f>
         <v>0</v>
       </c>
       <c r="F18" s="17" t="n">
@@ -3551,8 +3588,8 @@
         <v>65705.3504418474</v>
       </c>
       <c r="I18" s="17" t="n">
-        <f aca="false">IF(70&gt;=Inputs!B26,Inputs!B23*12*0.5*(1+Inputs!B21)^MAX(0,70-Inputs!B26),0)</f>
-        <v>26963.7205296094</v>
+        <f aca="false">IF(75&gt;=Inputs!B26,Inputs!B23*12*0.5*(1+Inputs!B21)^MAX(0,75-Inputs!B26),0)</f>
+        <v>30506.9748572876</v>
       </c>
       <c r="J18" s="17" t="n">
         <f aca="false">'Roth Conversion'!E18</f>
@@ -3580,7 +3617,7 @@
       </c>
       <c r="P18" s="25" t="n">
         <f aca="false">H18+I18+J18+K18+L18-G18-N18-O18</f>
-        <v>-15190.2292571972</v>
+        <v>-11646.974929519</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3600,7 +3637,7 @@
         <v>16500</v>
       </c>
       <c r="E19" s="17" t="n">
-        <f aca="false">IF(71&lt;65,Inputs!B35*12,0)</f>
+        <f aca="false">IF(76&lt;65,Inputs!B35*12,0)</f>
         <v>0</v>
       </c>
       <c r="F19" s="17" t="n">
@@ -3616,8 +3653,8 @@
         <v>67347.9842028936</v>
       </c>
       <c r="I19" s="17" t="n">
-        <f aca="false">IF(71&gt;=Inputs!B26,Inputs!B23*12*0.5*(1+Inputs!B21)^MAX(0,71-Inputs!B26),0)</f>
-        <v>27637.8135428496</v>
+        <f aca="false">IF(76&gt;=Inputs!B26,Inputs!B23*12*0.5*(1+Inputs!B21)^MAX(0,76-Inputs!B26),0)</f>
+        <v>31269.6492287198</v>
       </c>
       <c r="J19" s="17" t="n">
         <f aca="false">'Roth Conversion'!E19</f>
@@ -3645,7 +3682,7 @@
       </c>
       <c r="P19" s="25" t="n">
         <f aca="false">H19+I19+J19+K19+L19-G19-N19-O19</f>
-        <v>-18337.6396925568</v>
+        <v>-14705.8040066866</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3665,7 +3702,7 @@
         <v>16500</v>
       </c>
       <c r="E20" s="17" t="n">
-        <f aca="false">IF(72&lt;65,Inputs!B35*12,0)</f>
+        <f aca="false">IF(77&lt;65,Inputs!B35*12,0)</f>
         <v>0</v>
       </c>
       <c r="F20" s="17" t="n">
@@ -3681,8 +3718,8 @@
         <v>69031.6838079659</v>
       </c>
       <c r="I20" s="17" t="n">
-        <f aca="false">IF(72&gt;=Inputs!B26,Inputs!B23*12*0.5*(1+Inputs!B21)^MAX(0,72-Inputs!B26),0)</f>
-        <v>28328.7588814208</v>
+        <f aca="false">IF(77&gt;=Inputs!B26,Inputs!B23*12*0.5*(1+Inputs!B21)^MAX(0,77-Inputs!B26),0)</f>
+        <v>32051.3904594378</v>
       </c>
       <c r="J20" s="17" t="n">
         <f aca="false">'Roth Conversion'!E20</f>
@@ -3710,7 +3747,7 @@
       </c>
       <c r="P20" s="25" t="n">
         <f aca="false">H20+I20+J20+K20+L20-G20-N20-O20</f>
-        <v>-21589.1348039474</v>
+        <v>-17866.5032259305</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3730,7 +3767,7 @@
         <v>16500</v>
       </c>
       <c r="E21" s="17" t="n">
-        <f aca="false">IF(73&lt;65,Inputs!B35*12,0)</f>
+        <f aca="false">IF(78&lt;65,Inputs!B35*12,0)</f>
         <v>0</v>
       </c>
       <c r="F21" s="17" t="n">
@@ -3746,8 +3783,8 @@
         <v>70757.475903165</v>
       </c>
       <c r="I21" s="17" t="n">
-        <f aca="false">IF(73&gt;=Inputs!B26,Inputs!B23*12*0.5*(1+Inputs!B21)^MAX(0,73-Inputs!B26),0)</f>
-        <v>29036.9778534564</v>
+        <f aca="false">IF(78&gt;=Inputs!B26,Inputs!B23*12*0.5*(1+Inputs!B21)^MAX(0,78-Inputs!B26),0)</f>
+        <v>32852.6752209237</v>
       </c>
       <c r="J21" s="17" t="n">
         <f aca="false">'Roth Conversion'!E21</f>
@@ -3775,7 +3812,7 @@
       </c>
       <c r="P21" s="25" t="n">
         <f aca="false">H21+I21+J21+K21+L21-G21-N21-O21</f>
-        <v>-24948.1940712382</v>
+        <v>-21132.4967037709</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3795,7 +3832,7 @@
         <v>16500</v>
       </c>
       <c r="E22" s="17" t="n">
-        <f aca="false">IF(74&lt;65,Inputs!B35*12,0)</f>
+        <f aca="false">IF(79&lt;65,Inputs!B35*12,0)</f>
         <v>0</v>
       </c>
       <c r="F22" s="17" t="n">
@@ -3811,8 +3848,8 @@
         <v>72526.4128007442</v>
       </c>
       <c r="I22" s="17" t="n">
-        <f aca="false">IF(74&gt;=Inputs!B26,Inputs!B23*12*0.5*(1+Inputs!B21)^MAX(0,74-Inputs!B26),0)</f>
-        <v>29762.9022997928</v>
+        <f aca="false">IF(79&gt;=Inputs!B26,Inputs!B23*12*0.5*(1+Inputs!B21)^MAX(0,79-Inputs!B26),0)</f>
+        <v>33673.9921014468</v>
       </c>
       <c r="J22" s="17" t="n">
         <f aca="false">'Roth Conversion'!E22</f>
@@ -3840,7 +3877,7 @@
       </c>
       <c r="P22" s="25" t="n">
         <f aca="false">H22+I22+J22+K22+L22-G22-N22-O22</f>
-        <v>-28418.4160512098</v>
+        <v>-24507.3262495558</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3860,7 +3897,7 @@
         <v>16500</v>
       </c>
       <c r="E23" s="17" t="n">
-        <f aca="false">IF(75&lt;65,Inputs!B35*12,0)</f>
+        <f aca="false">IF(80&lt;65,Inputs!B35*12,0)</f>
         <v>0</v>
       </c>
       <c r="F23" s="17" t="n">
@@ -3876,8 +3913,8 @@
         <v>74339.5731207628</v>
       </c>
       <c r="I23" s="17" t="n">
-        <f aca="false">IF(75&gt;=Inputs!B26,Inputs!B23*12*0.5*(1+Inputs!B21)^MAX(0,75-Inputs!B26),0)</f>
-        <v>30506.9748572876</v>
+        <f aca="false">IF(80&gt;=Inputs!B26,Inputs!B23*12*0.5*(1+Inputs!B21)^MAX(0,80-Inputs!B26),0)</f>
+        <v>34515.8419039829</v>
       </c>
       <c r="J23" s="17" t="n">
         <f aca="false">'Roth Conversion'!E23</f>
@@ -3905,7 +3942,7 @@
       </c>
       <c r="P23" s="25" t="n">
         <f aca="false">H23+I23+J23+K23+L23-G23-N23-O23</f>
-        <v>-32003.5226056258</v>
+        <v>-27994.6555589304</v>
       </c>
     </row>
   </sheetData>
@@ -3928,7 +3965,7 @@
     <tabColor rgb="FF1A3A6B"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
@@ -3982,644 +4019,644 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="10" t="n">
+      <c r="A3" s="26" t="n">
+        <v>56</v>
+      </c>
+      <c r="B3" s="27" t="n">
+        <f aca="false">Inputs!B9+Inputs!B11*(1+Inputs!B12/100)</f>
+        <v>3037518.75</v>
+      </c>
+      <c r="C3" s="27" t="n">
+        <f aca="false">(Inputs!B10+Inputs!B13)*(1+Inputs!B19)</f>
+        <v>810000</v>
+      </c>
+      <c r="D3" s="27" t="n">
+        <f aca="false">Inputs!E11*(1+Inputs!B19)</f>
+        <v>10800</v>
+      </c>
+      <c r="E3" s="27" t="n">
+        <f aca="false">Inputs!E10*(1+Inputs!B19)</f>
+        <v>54000</v>
+      </c>
+      <c r="F3" s="27" t="n">
+        <f aca="false">(Inputs!B14+Inputs!B15)*(1+Inputs!B19)</f>
+        <v>116640</v>
+      </c>
+      <c r="G3" s="27" t="n">
+        <f aca="false">Inputs!B16*(1+Inputs!B19)</f>
+        <v>540000</v>
+      </c>
+      <c r="H3" s="28" t="n">
+        <f aca="false">SUM(B3:G3)</f>
+        <v>4568958.75</v>
+      </c>
+      <c r="I3" s="29" t="n">
+        <f aca="false">H3+Inputs!B36</f>
+        <v>5368958.75</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="26" t="n">
+        <v>57</v>
+      </c>
+      <c r="B4" s="27" t="n">
+        <f aca="false">B3*(1+Inputs!B19)+Inputs!B11*(1+Inputs!B12/100)</f>
+        <v>3318039</v>
+      </c>
+      <c r="C4" s="27" t="n">
+        <f aca="false">C3*(1+Inputs!B19)</f>
+        <v>874800</v>
+      </c>
+      <c r="D4" s="27" t="n">
+        <f aca="false">D3*(1+Inputs!B19)</f>
+        <v>11664</v>
+      </c>
+      <c r="E4" s="27" t="n">
+        <f aca="false">E3*(1+Inputs!B19)</f>
+        <v>58320</v>
+      </c>
+      <c r="F4" s="27" t="n">
+        <f aca="false">(F3+Inputs!B15)*(1+Inputs!B19)</f>
+        <v>134611.2</v>
+      </c>
+      <c r="G4" s="27" t="n">
+        <f aca="false">G3*(1+Inputs!B19)</f>
+        <v>583200</v>
+      </c>
+      <c r="H4" s="28" t="n">
+        <f aca="false">SUM(B4:G4)</f>
+        <v>4980634.2</v>
+      </c>
+      <c r="I4" s="29" t="n">
+        <f aca="false">H4+Inputs!B36</f>
+        <v>5780634.2</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="26" t="n">
+        <v>58</v>
+      </c>
+      <c r="B5" s="27" t="n">
+        <f aca="false">B4*(1+Inputs!B19)+Inputs!B11*(1+Inputs!B12/100)</f>
+        <v>3621000.87</v>
+      </c>
+      <c r="C5" s="27" t="n">
+        <f aca="false">C4*(1+Inputs!B19)</f>
+        <v>944784</v>
+      </c>
+      <c r="D5" s="27" t="n">
+        <f aca="false">D4*(1+Inputs!B19)</f>
+        <v>12597.12</v>
+      </c>
+      <c r="E5" s="27" t="n">
+        <f aca="false">E4*(1+Inputs!B19)</f>
+        <v>62985.6</v>
+      </c>
+      <c r="F5" s="27" t="n">
+        <f aca="false">(F4+Inputs!B15)*(1+Inputs!B19)</f>
+        <v>154020.096</v>
+      </c>
+      <c r="G5" s="27" t="n">
+        <f aca="false">G4*(1+Inputs!B19)</f>
+        <v>629856</v>
+      </c>
+      <c r="H5" s="28" t="n">
+        <f aca="false">SUM(B5:G5)</f>
+        <v>5425243.686</v>
+      </c>
+      <c r="I5" s="29" t="n">
+        <f aca="false">H5+Inputs!B36</f>
+        <v>6225243.686</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="26" t="n">
+        <v>59</v>
+      </c>
+      <c r="B6" s="27" t="n">
+        <f aca="false">B5*(1+Inputs!B19)+Inputs!B11*(1+Inputs!B12/100)</f>
+        <v>3948199.6896</v>
+      </c>
+      <c r="C6" s="27" t="n">
+        <f aca="false">C5*(1+Inputs!B19)</f>
+        <v>1020366.72</v>
+      </c>
+      <c r="D6" s="27" t="n">
+        <f aca="false">D5*(1+Inputs!B19)</f>
+        <v>13604.8896</v>
+      </c>
+      <c r="E6" s="27" t="n">
+        <f aca="false">E5*(1+Inputs!B19)</f>
+        <v>68024.448</v>
+      </c>
+      <c r="F6" s="27" t="n">
+        <f aca="false">(F5+Inputs!B15)*(1+Inputs!B19)</f>
+        <v>174981.70368</v>
+      </c>
+      <c r="G6" s="27" t="n">
+        <f aca="false">G5*(1+Inputs!B19)</f>
+        <v>680244.48</v>
+      </c>
+      <c r="H6" s="28" t="n">
+        <f aca="false">SUM(B6:G6)</f>
+        <v>5905421.93088</v>
+      </c>
+      <c r="I6" s="29" t="n">
+        <f aca="false">H6+Inputs!B36</f>
+        <v>6705421.93088</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="26" t="n">
+        <v>60</v>
+      </c>
+      <c r="B7" s="27" t="n">
+        <f aca="false">B6*(1+Inputs!B19)+Inputs!B11*(1+Inputs!B12/100)</f>
+        <v>4301574.414768</v>
+      </c>
+      <c r="C7" s="27" t="n">
+        <f aca="false">C6*(1+Inputs!B19)</f>
+        <v>1101996.0576</v>
+      </c>
+      <c r="D7" s="27" t="n">
+        <f aca="false">D6*(1+Inputs!B19)</f>
+        <v>14693.280768</v>
+      </c>
+      <c r="E7" s="27" t="n">
+        <f aca="false">E6*(1+Inputs!B19)</f>
+        <v>73466.40384</v>
+      </c>
+      <c r="F7" s="27" t="n">
+        <f aca="false">(F6+Inputs!B15)*(1+Inputs!B19)</f>
+        <v>197620.2399744</v>
+      </c>
+      <c r="G7" s="27" t="n">
+        <f aca="false">G6*(1+Inputs!B19)</f>
+        <v>734664.0384</v>
+      </c>
+      <c r="H7" s="28" t="n">
+        <f aca="false">SUM(B7:G7)</f>
+        <v>6424014.4353504</v>
+      </c>
+      <c r="I7" s="29" t="n">
+        <f aca="false">H7+Inputs!B36</f>
+        <v>7224014.4353504</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="26" t="n">
+        <v>61</v>
+      </c>
+      <c r="B8" s="27" t="n">
+        <f aca="false">B7*(1+Inputs!B19)+Inputs!B11*(1+Inputs!B12/100)</f>
+        <v>4683219.11794944</v>
+      </c>
+      <c r="C8" s="27" t="n">
+        <f aca="false">C7*(1+Inputs!B19)</f>
+        <v>1190155.742208</v>
+      </c>
+      <c r="D8" s="27" t="n">
+        <f aca="false">D7*(1+Inputs!B19)</f>
+        <v>15868.74322944</v>
+      </c>
+      <c r="E8" s="27" t="n">
+        <f aca="false">E7*(1+Inputs!B19)</f>
+        <v>79343.7161472</v>
+      </c>
+      <c r="F8" s="27" t="n">
+        <f aca="false">(F7+Inputs!B15)*(1+Inputs!B19)</f>
+        <v>222069.859172352</v>
+      </c>
+      <c r="G8" s="27" t="n">
+        <f aca="false">G7*(1+Inputs!B19)</f>
+        <v>793437.161472</v>
+      </c>
+      <c r="H8" s="28" t="n">
+        <f aca="false">SUM(B8:G8)</f>
+        <v>6984094.34017843</v>
+      </c>
+      <c r="I8" s="29" t="n">
+        <f aca="false">H8+Inputs!B36</f>
+        <v>7784094.34017843</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="26" t="n">
+        <v>62</v>
+      </c>
+      <c r="B9" s="27" t="n">
+        <f aca="false">B8*(1+Inputs!B19)+Inputs!B11*(1+Inputs!B12/100)</f>
+        <v>5095395.3973854</v>
+      </c>
+      <c r="C9" s="27" t="n">
+        <f aca="false">C8*(1+Inputs!B19)</f>
+        <v>1285368.20158464</v>
+      </c>
+      <c r="D9" s="27" t="n">
+        <f aca="false">D8*(1+Inputs!B19)</f>
+        <v>17138.2426877952</v>
+      </c>
+      <c r="E9" s="27" t="n">
+        <f aca="false">E8*(1+Inputs!B19)</f>
+        <v>85691.213438976</v>
+      </c>
+      <c r="F9" s="27" t="n">
+        <f aca="false">(F8+Inputs!B15)*(1+Inputs!B19)</f>
+        <v>248475.44790614</v>
+      </c>
+      <c r="G9" s="27" t="n">
+        <f aca="false">G8*(1+Inputs!B19)</f>
+        <v>856912.13438976</v>
+      </c>
+      <c r="H9" s="28" t="n">
+        <f aca="false">SUM(B9:G9)</f>
+        <v>7588980.63739271</v>
+      </c>
+      <c r="I9" s="29" t="n">
+        <f aca="false">H9+Inputs!B36</f>
+        <v>8388980.63739271</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="26" t="n">
+        <v>63</v>
+      </c>
+      <c r="B10" s="27" t="n">
+        <f aca="false">B9*(1+Inputs!B19)+Inputs!B11*(1+Inputs!B12/100)</f>
+        <v>5540545.77917623</v>
+      </c>
+      <c r="C10" s="27" t="n">
+        <f aca="false">C9*(1+Inputs!B19)</f>
+        <v>1388197.65771141</v>
+      </c>
+      <c r="D10" s="27" t="n">
+        <f aca="false">D9*(1+Inputs!B19)</f>
+        <v>18509.3021028188</v>
+      </c>
+      <c r="E10" s="27" t="n">
+        <f aca="false">E9*(1+Inputs!B19)</f>
+        <v>92546.5105140941</v>
+      </c>
+      <c r="F10" s="27" t="n">
+        <f aca="false">(F9+Inputs!B15)*(1+Inputs!B19)</f>
+        <v>276993.483738632</v>
+      </c>
+      <c r="G10" s="27" t="n">
+        <f aca="false">G9*(1+Inputs!B19)</f>
+        <v>925465.105140941</v>
+      </c>
+      <c r="H10" s="28" t="n">
+        <f aca="false">SUM(B10:G10)</f>
+        <v>8242257.83838413</v>
+      </c>
+      <c r="I10" s="29" t="n">
+        <f aca="false">H10+Inputs!B36</f>
+        <v>9042257.83838413</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="26" t="n">
+        <v>64</v>
+      </c>
+      <c r="B11" s="27" t="n">
+        <f aca="false">B10*(1+Inputs!B19)+Inputs!B11*(1+Inputs!B12/100)</f>
+        <v>6021308.19151033</v>
+      </c>
+      <c r="C11" s="27" t="n">
+        <f aca="false">C10*(1+Inputs!B19)</f>
+        <v>1499253.47032833</v>
+      </c>
+      <c r="D11" s="27" t="n">
+        <f aca="false">D10*(1+Inputs!B19)</f>
+        <v>19990.0462710443</v>
+      </c>
+      <c r="E11" s="27" t="n">
+        <f aca="false">E10*(1+Inputs!B19)</f>
+        <v>99950.2313552217</v>
+      </c>
+      <c r="F11" s="27" t="n">
+        <f aca="false">(F10+Inputs!B15)*(1+Inputs!B19)</f>
+        <v>307792.962437722</v>
+      </c>
+      <c r="G11" s="27" t="n">
+        <f aca="false">G10*(1+Inputs!B19)</f>
+        <v>999502.313552217</v>
+      </c>
+      <c r="H11" s="28" t="n">
+        <f aca="false">SUM(B11:G11)</f>
+        <v>8947797.21545486</v>
+      </c>
+      <c r="I11" s="29" t="n">
+        <f aca="false">H11+Inputs!B36</f>
+        <v>9747797.21545486</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="10" t="n">
         <v>65</v>
       </c>
-      <c r="B3" s="11" t="n">
+      <c r="B12" s="14" t="n">
         <f aca="false">'Roth Conversion'!J3</f>
         <v>2828950</v>
       </c>
-      <c r="C3" s="11" t="n">
-        <f aca="false">(Inputs!B10+Inputs!B13)*(1+Inputs!B19)-'Withdrawal Plan'!K3</f>
-        <v>810000</v>
-      </c>
-      <c r="D3" s="11" t="n">
-        <f aca="false">Inputs!E11*(1+Inputs!B19)</f>
-        <v>10800</v>
-      </c>
-      <c r="E3" s="11" t="n">
-        <f aca="false">Inputs!E10*(1+Inputs!B19)</f>
-        <v>54000</v>
-      </c>
-      <c r="F3" s="11" t="n">
-        <f aca="false">MAX(0,Inputs!B14*(1+Inputs!B19)-'Withdrawal Plan'!M3)</f>
-        <v>105780</v>
-      </c>
-      <c r="G3" s="11" t="n">
-        <f aca="false">MAX(0,Inputs!B16*(1+Inputs!B19)-'Withdrawal Plan'!L3)</f>
-        <v>540000</v>
-      </c>
-      <c r="H3" s="20" t="n">
-        <f aca="false">SUM(B3:G3)</f>
-        <v>4349530</v>
-      </c>
-      <c r="I3" s="21" t="n">
-        <f aca="false">H3+Inputs!B36</f>
-        <v>5149530</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="10" t="n">
+      <c r="C12" s="14" t="n">
+        <f aca="false">MAX(0,C11*(1+Inputs!B19)-'Withdrawal Plan'!K3)</f>
+        <v>1619193.74795459</v>
+      </c>
+      <c r="D12" s="14" t="n">
+        <f aca="false">D11*(1+Inputs!B19)</f>
+        <v>21589.2499727279</v>
+      </c>
+      <c r="E12" s="14" t="n">
+        <f aca="false">E11*(1+Inputs!B19)</f>
+        <v>107946.249863639</v>
+      </c>
+      <c r="F12" s="14" t="n">
+        <f aca="false">MAX(0,F11*(1+Inputs!B19)-'Withdrawal Plan'!M3)</f>
+        <v>330196.39943274</v>
+      </c>
+      <c r="G12" s="14" t="n">
+        <f aca="false">MAX(0,G11*(1+Inputs!B19)-'Withdrawal Plan'!L3)</f>
+        <v>1079462.49863639</v>
+      </c>
+      <c r="H12" s="22" t="n">
+        <f aca="false">SUM(B12:G12)</f>
+        <v>5987338.14586009</v>
+      </c>
+      <c r="I12" s="23" t="n">
+        <f aca="false">H12+Inputs!B36</f>
+        <v>6787338.14586009</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="10" t="n">
         <v>66</v>
       </c>
-      <c r="B4" s="14" t="n">
+      <c r="B13" s="11" t="n">
         <f aca="false">'Roth Conversion'!J4</f>
         <v>2657900</v>
       </c>
-      <c r="C4" s="14" t="n">
-        <f aca="false">MAX(0,C3*(1+Inputs!B19)-'Withdrawal Plan'!K4)</f>
-        <v>874800</v>
-      </c>
-      <c r="D4" s="14" t="n">
-        <f aca="false">D3*(1+Inputs!B19)</f>
-        <v>11664</v>
-      </c>
-      <c r="E4" s="14" t="n">
-        <f aca="false">E3*(1+Inputs!B19)</f>
-        <v>58320</v>
-      </c>
-      <c r="F4" s="14" t="n">
-        <f aca="false">MAX(0,F3*(1+Inputs!B19)-'Withdrawal Plan'!M4)</f>
-        <v>111911.4</v>
-      </c>
-      <c r="G4" s="14" t="n">
-        <f aca="false">MAX(0,G3*(1+Inputs!B19)-'Withdrawal Plan'!L4)</f>
-        <v>583200</v>
-      </c>
-      <c r="H4" s="22" t="n">
-        <f aca="false">SUM(B4:G4)</f>
-        <v>4297795.4</v>
-      </c>
-      <c r="I4" s="23" t="n">
-        <f aca="false">H4+Inputs!B36</f>
-        <v>5097795.4</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="10" t="n">
+      <c r="C13" s="11" t="n">
+        <f aca="false">MAX(0,C12*(1+Inputs!B19)-'Withdrawal Plan'!K4)</f>
+        <v>1748729.24779096</v>
+      </c>
+      <c r="D13" s="11" t="n">
+        <f aca="false">D12*(1+Inputs!B19)</f>
+        <v>23316.3899705461</v>
+      </c>
+      <c r="E13" s="11" t="n">
+        <f aca="false">E12*(1+Inputs!B19)</f>
+        <v>116581.949852731</v>
+      </c>
+      <c r="F13" s="11" t="n">
+        <f aca="false">MAX(0,F12*(1+Inputs!B19)-'Withdrawal Plan'!M4)</f>
+        <v>354281.111387359</v>
+      </c>
+      <c r="G13" s="11" t="n">
+        <f aca="false">MAX(0,G12*(1+Inputs!B19)-'Withdrawal Plan'!L4)</f>
+        <v>1165819.49852731</v>
+      </c>
+      <c r="H13" s="20" t="n">
+        <f aca="false">SUM(B13:G13)</f>
+        <v>6066628.1975289</v>
+      </c>
+      <c r="I13" s="21" t="n">
+        <f aca="false">H13+Inputs!B36</f>
+        <v>6866628.1975289</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="10" t="n">
         <v>67</v>
       </c>
-      <c r="B5" s="11" t="n">
+      <c r="B14" s="14" t="n">
         <f aca="false">'Roth Conversion'!J5</f>
         <v>2527364.4</v>
       </c>
-      <c r="C5" s="11" t="n">
-        <f aca="false">MAX(0,C4*(1+Inputs!B19)-'Withdrawal Plan'!K5)</f>
-        <v>944784</v>
-      </c>
-      <c r="D5" s="11" t="n">
-        <f aca="false">D4*(1+Inputs!B19)</f>
-        <v>12597.12</v>
-      </c>
-      <c r="E5" s="11" t="n">
-        <f aca="false">E4*(1+Inputs!B19)</f>
-        <v>62985.6</v>
-      </c>
-      <c r="F5" s="11" t="n">
-        <f aca="false">MAX(0,F4*(1+Inputs!B19)-'Withdrawal Plan'!M5)</f>
-        <v>118416.762</v>
-      </c>
-      <c r="G5" s="11" t="n">
-        <f aca="false">MAX(0,G4*(1+Inputs!B19)-'Withdrawal Plan'!L5)</f>
-        <v>629856</v>
-      </c>
-      <c r="H5" s="20" t="n">
-        <f aca="false">SUM(B5:G5)</f>
-        <v>4296003.882</v>
-      </c>
-      <c r="I5" s="21" t="n">
-        <f aca="false">H5+Inputs!B36</f>
-        <v>5096003.882</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="10" t="n">
+      <c r="C14" s="14" t="n">
+        <f aca="false">MAX(0,C13*(1+Inputs!B19)-'Withdrawal Plan'!K5)</f>
+        <v>1888627.58761424</v>
+      </c>
+      <c r="D14" s="14" t="n">
+        <f aca="false">D13*(1+Inputs!B19)</f>
+        <v>25181.7011681898</v>
+      </c>
+      <c r="E14" s="14" t="n">
+        <f aca="false">E13*(1+Inputs!B19)</f>
+        <v>125908.505840949</v>
+      </c>
+      <c r="F14" s="14" t="n">
+        <f aca="false">MAX(0,F13*(1+Inputs!B19)-'Withdrawal Plan'!M5)</f>
+        <v>380176.050298348</v>
+      </c>
+      <c r="G14" s="14" t="n">
+        <f aca="false">MAX(0,G13*(1+Inputs!B19)-'Withdrawal Plan'!L5)</f>
+        <v>1259085.05840949</v>
+      </c>
+      <c r="H14" s="22" t="n">
+        <f aca="false">SUM(B14:G14)</f>
+        <v>6206343.30333121</v>
+      </c>
+      <c r="I14" s="23" t="n">
+        <f aca="false">H14+Inputs!B36</f>
+        <v>7006343.30333121</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="10" t="n">
         <v>68</v>
       </c>
-      <c r="B6" s="14" t="n">
+      <c r="B15" s="11" t="n">
         <f aca="false">'Roth Conversion'!J6</f>
         <v>2397841.66</v>
       </c>
-      <c r="C6" s="14" t="n">
-        <f aca="false">MAX(0,C5*(1+Inputs!B19)-'Withdrawal Plan'!K6)</f>
-        <v>1020366.72</v>
-      </c>
-      <c r="D6" s="14" t="n">
-        <f aca="false">D5*(1+Inputs!B19)</f>
-        <v>13604.8896</v>
-      </c>
-      <c r="E6" s="14" t="n">
-        <f aca="false">E5*(1+Inputs!B19)</f>
-        <v>68024.448</v>
-      </c>
-      <c r="F6" s="14" t="n">
-        <f aca="false">MAX(0,F5*(1+Inputs!B19)-'Withdrawal Plan'!M6)</f>
-        <v>125320.17546</v>
-      </c>
-      <c r="G6" s="14" t="n">
-        <f aca="false">MAX(0,G5*(1+Inputs!B19)-'Withdrawal Plan'!L6)</f>
-        <v>680244.48</v>
-      </c>
-      <c r="H6" s="22" t="n">
-        <f aca="false">SUM(B6:G6)</f>
-        <v>4305402.37306</v>
-      </c>
-      <c r="I6" s="23" t="n">
-        <f aca="false">H6+Inputs!B36</f>
-        <v>5105402.37306</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="10" t="n">
+      <c r="C15" s="11" t="n">
+        <f aca="false">MAX(0,C14*(1+Inputs!B19)-'Withdrawal Plan'!K6)</f>
+        <v>2039717.79462337</v>
+      </c>
+      <c r="D15" s="11" t="n">
+        <f aca="false">D14*(1+Inputs!B19)</f>
+        <v>27196.237261645</v>
+      </c>
+      <c r="E15" s="11" t="n">
+        <f aca="false">E14*(1+Inputs!B19)</f>
+        <v>135981.186308225</v>
+      </c>
+      <c r="F15" s="11" t="n">
+        <f aca="false">MAX(0,F14*(1+Inputs!B19)-'Withdrawal Plan'!M6)</f>
+        <v>408020.206822216</v>
+      </c>
+      <c r="G15" s="11" t="n">
+        <f aca="false">MAX(0,G14*(1+Inputs!B19)-'Withdrawal Plan'!L6)</f>
+        <v>1359811.86308225</v>
+      </c>
+      <c r="H15" s="20" t="n">
+        <f aca="false">SUM(B15:G15)</f>
+        <v>6368568.94809771</v>
+      </c>
+      <c r="I15" s="21" t="n">
+        <f aca="false">H15+Inputs!B36</f>
+        <v>7168568.94809771</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="10" t="n">
         <v>69</v>
       </c>
-      <c r="B7" s="11" t="n">
+      <c r="B16" s="14" t="n">
         <f aca="false">'Roth Conversion'!J7</f>
         <v>2269357.1015</v>
       </c>
-      <c r="C7" s="11" t="n">
-        <f aca="false">MAX(0,C6*(1+Inputs!B19)-'Withdrawal Plan'!K7)</f>
-        <v>1101996.0576</v>
-      </c>
-      <c r="D7" s="11" t="n">
-        <f aca="false">D6*(1+Inputs!B19)</f>
-        <v>14693.280768</v>
-      </c>
-      <c r="E7" s="11" t="n">
-        <f aca="false">E6*(1+Inputs!B19)</f>
-        <v>73466.40384</v>
-      </c>
-      <c r="F7" s="11" t="n">
-        <f aca="false">MAX(0,F6*(1+Inputs!B19)-'Withdrawal Plan'!M7)</f>
-        <v>132647.3656218</v>
-      </c>
-      <c r="G7" s="11" t="n">
-        <f aca="false">MAX(0,G6*(1+Inputs!B19)-'Withdrawal Plan'!L7)</f>
-        <v>734664.0384</v>
-      </c>
-      <c r="H7" s="20" t="n">
-        <f aca="false">SUM(B7:G7)</f>
-        <v>4326824.2477298</v>
-      </c>
-      <c r="I7" s="21" t="n">
-        <f aca="false">H7+Inputs!B36</f>
-        <v>5126824.2477298</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="n">
+      <c r="C16" s="14" t="n">
+        <f aca="false">MAX(0,C15*(1+Inputs!B19)-'Withdrawal Plan'!K7)</f>
+        <v>2202895.21819324</v>
+      </c>
+      <c r="D16" s="14" t="n">
+        <f aca="false">D15*(1+Inputs!B19)</f>
+        <v>29371.9362425766</v>
+      </c>
+      <c r="E16" s="14" t="n">
+        <f aca="false">E15*(1+Inputs!B19)</f>
+        <v>146859.681212883</v>
+      </c>
+      <c r="F16" s="14" t="n">
+        <f aca="false">MAX(0,F15*(1+Inputs!B19)-'Withdrawal Plan'!M7)</f>
+        <v>437963.399492993</v>
+      </c>
+      <c r="G16" s="14" t="n">
+        <f aca="false">MAX(0,G15*(1+Inputs!B19)-'Withdrawal Plan'!L7)</f>
+        <v>1468596.81212883</v>
+      </c>
+      <c r="H16" s="22" t="n">
+        <f aca="false">SUM(B16:G16)</f>
+        <v>6555044.14877053</v>
+      </c>
+      <c r="I16" s="23" t="n">
+        <f aca="false">H16+Inputs!B36</f>
+        <v>7355044.14877053</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="10" t="n">
         <v>70</v>
       </c>
-      <c r="B8" s="14" t="n">
+      <c r="B17" s="11" t="n">
         <f aca="false">'Roth Conversion'!J8</f>
         <v>2141936.6790375</v>
       </c>
-      <c r="C8" s="14" t="n">
-        <f aca="false">MAX(0,C7*(1+Inputs!B19)-'Withdrawal Plan'!K8)</f>
-        <v>1190155.742208</v>
-      </c>
-      <c r="D8" s="14" t="n">
-        <f aca="false">D7*(1+Inputs!B19)</f>
-        <v>15868.74322944</v>
-      </c>
-      <c r="E8" s="14" t="n">
-        <f aca="false">E7*(1+Inputs!B19)</f>
-        <v>79343.7161472</v>
-      </c>
-      <c r="F8" s="14" t="n">
-        <f aca="false">MAX(0,F7*(1+Inputs!B19)-'Withdrawal Plan'!M8)</f>
-        <v>140425.809802794</v>
-      </c>
-      <c r="G8" s="14" t="n">
-        <f aca="false">MAX(0,G7*(1+Inputs!B19)-'Withdrawal Plan'!L8)</f>
-        <v>793437.161472</v>
-      </c>
-      <c r="H8" s="22" t="n">
-        <f aca="false">SUM(B8:G8)</f>
-        <v>4361167.85189694</v>
-      </c>
-      <c r="I8" s="23" t="n">
-        <f aca="false">H8+Inputs!B36</f>
-        <v>5161167.85189694</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="10" t="n">
+      <c r="C17" s="11" t="n">
+        <f aca="false">MAX(0,C16*(1+Inputs!B19)-'Withdrawal Plan'!K8)</f>
+        <v>2379126.8356487</v>
+      </c>
+      <c r="D17" s="11" t="n">
+        <f aca="false">D16*(1+Inputs!B19)</f>
+        <v>31721.6911419827</v>
+      </c>
+      <c r="E17" s="11" t="n">
+        <f aca="false">E16*(1+Inputs!B19)</f>
+        <v>158608.455709914</v>
+      </c>
+      <c r="F17" s="11" t="n">
+        <f aca="false">MAX(0,F16*(1+Inputs!B19)-'Withdrawal Plan'!M8)</f>
+        <v>470167.126383683</v>
+      </c>
+      <c r="G17" s="11" t="n">
+        <f aca="false">MAX(0,G16*(1+Inputs!B19)-'Withdrawal Plan'!L8)</f>
+        <v>1586084.55709914</v>
+      </c>
+      <c r="H17" s="20" t="n">
+        <f aca="false">SUM(B17:G17)</f>
+        <v>6767645.34502092</v>
+      </c>
+      <c r="I17" s="21" t="n">
+        <f aca="false">H17+Inputs!B36</f>
+        <v>7567645.34502092</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="10" t="n">
         <v>71</v>
       </c>
-      <c r="B9" s="11" t="n">
+      <c r="B18" s="14" t="n">
         <f aca="false">'Roth Conversion'!J9</f>
         <v>2015606.99601344</v>
       </c>
-      <c r="C9" s="11" t="n">
-        <f aca="false">MAX(0,C8*(1+Inputs!B19)-'Withdrawal Plan'!K9)</f>
-        <v>1285368.20158464</v>
-      </c>
-      <c r="D9" s="11" t="n">
-        <f aca="false">D8*(1+Inputs!B19)</f>
-        <v>17138.2426877952</v>
-      </c>
-      <c r="E9" s="11" t="n">
-        <f aca="false">E8*(1+Inputs!B19)</f>
-        <v>85691.213438976</v>
-      </c>
-      <c r="F9" s="11" t="n">
-        <f aca="false">MAX(0,F8*(1+Inputs!B19)-'Withdrawal Plan'!M9)</f>
-        <v>148684.86226483</v>
-      </c>
-      <c r="G9" s="11" t="n">
-        <f aca="false">MAX(0,G8*(1+Inputs!B19)-'Withdrawal Plan'!L9)</f>
-        <v>856912.13438976</v>
-      </c>
-      <c r="H9" s="20" t="n">
-        <f aca="false">SUM(B9:G9)</f>
-        <v>4409401.65037944</v>
-      </c>
-      <c r="I9" s="21" t="n">
-        <f aca="false">H9+Inputs!B36</f>
-        <v>5209401.65037944</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="10" t="n">
+      <c r="C18" s="14" t="n">
+        <f aca="false">MAX(0,C17*(1+Inputs!B19)-'Withdrawal Plan'!K9)</f>
+        <v>2569456.9825006</v>
+      </c>
+      <c r="D18" s="14" t="n">
+        <f aca="false">D17*(1+Inputs!B19)</f>
+        <v>34259.4264333413</v>
+      </c>
+      <c r="E18" s="14" t="n">
+        <f aca="false">E17*(1+Inputs!B19)</f>
+        <v>171297.132166707</v>
+      </c>
+      <c r="F18" s="14" t="n">
+        <f aca="false">MAX(0,F17*(1+Inputs!B19)-'Withdrawal Plan'!M9)</f>
+        <v>504805.48417219</v>
+      </c>
+      <c r="G18" s="14" t="n">
+        <f aca="false">MAX(0,G17*(1+Inputs!B19)-'Withdrawal Plan'!L9)</f>
+        <v>1712971.32166707</v>
+      </c>
+      <c r="H18" s="22" t="n">
+        <f aca="false">SUM(B18:G18)</f>
+        <v>7008397.34295334</v>
+      </c>
+      <c r="I18" s="23" t="n">
+        <f aca="false">H18+Inputs!B36</f>
+        <v>7808397.34295334</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="10" t="n">
         <v>72</v>
       </c>
-      <c r="B10" s="14" t="n">
+      <c r="B19" s="11" t="n">
         <f aca="false">'Roth Conversion'!J10</f>
         <v>1890395.32091377</v>
       </c>
-      <c r="C10" s="14" t="n">
-        <f aca="false">MAX(0,C9*(1+Inputs!B19)-'Withdrawal Plan'!K10)</f>
-        <v>1388197.65771141</v>
-      </c>
-      <c r="D10" s="14" t="n">
-        <f aca="false">D9*(1+Inputs!B19)</f>
-        <v>18509.3021028188</v>
-      </c>
-      <c r="E10" s="14" t="n">
-        <f aca="false">E9*(1+Inputs!B19)</f>
-        <v>92546.5105140941</v>
-      </c>
-      <c r="F10" s="14" t="n">
-        <f aca="false">MAX(0,F9*(1+Inputs!B19)-'Withdrawal Plan'!M10)</f>
-        <v>157455.88830772</v>
-      </c>
-      <c r="G10" s="14" t="n">
-        <f aca="false">MAX(0,G9*(1+Inputs!B19)-'Withdrawal Plan'!L10)</f>
-        <v>925465.105140941</v>
-      </c>
-      <c r="H10" s="22" t="n">
-        <f aca="false">SUM(B10:G10)</f>
-        <v>4472569.78469076</v>
-      </c>
-      <c r="I10" s="23" t="n">
-        <f aca="false">H10+Inputs!B36</f>
-        <v>5272569.78469076</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="10" t="n">
+      <c r="C19" s="11" t="n">
+        <f aca="false">MAX(0,C18*(1+Inputs!B19)-'Withdrawal Plan'!K10)</f>
+        <v>2775013.54110065</v>
+      </c>
+      <c r="D19" s="11" t="n">
+        <f aca="false">D18*(1+Inputs!B19)</f>
+        <v>37000.1805480087</v>
+      </c>
+      <c r="E19" s="11" t="n">
+        <f aca="false">E18*(1+Inputs!B19)</f>
+        <v>185000.902740043</v>
+      </c>
+      <c r="F19" s="11" t="n">
+        <f aca="false">MAX(0,F18*(1+Inputs!B19)-'Withdrawal Plan'!M10)</f>
+        <v>542066.159967668</v>
+      </c>
+      <c r="G19" s="11" t="n">
+        <f aca="false">MAX(0,G18*(1+Inputs!B19)-'Withdrawal Plan'!L10)</f>
+        <v>1850009.02740043</v>
+      </c>
+      <c r="H19" s="20" t="n">
+        <f aca="false">SUM(B19:G19)</f>
+        <v>7279485.13267057</v>
+      </c>
+      <c r="I19" s="21" t="n">
+        <f aca="false">H19+Inputs!B36</f>
+        <v>8079485.13267057</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="10" t="n">
         <v>73</v>
       </c>
-      <c r="B11" s="17" t="n">
+      <c r="B20" s="17" t="n">
         <f aca="false">'Roth Conversion'!J11</f>
         <v>1766329.60393662</v>
       </c>
-      <c r="C11" s="17" t="n">
-        <f aca="false">MAX(0,C10*(1+Inputs!B19)-'Withdrawal Plan'!K11)</f>
-        <v>1499253.47032833</v>
-      </c>
-      <c r="D11" s="17" t="n">
-        <f aca="false">D10*(1+Inputs!B19)</f>
-        <v>19990.0462710443</v>
-      </c>
-      <c r="E11" s="17" t="n">
-        <f aca="false">E10*(1+Inputs!B19)</f>
-        <v>99950.2313552217</v>
-      </c>
-      <c r="F11" s="17" t="n">
-        <f aca="false">MAX(0,F10*(1+Inputs!B19)-'Withdrawal Plan'!M11)</f>
-        <v>166772.408287125</v>
-      </c>
-      <c r="G11" s="17" t="n">
-        <f aca="false">MAX(0,G10*(1+Inputs!B19)-'Withdrawal Plan'!L11)</f>
-        <v>999502.313552217</v>
-      </c>
-      <c r="H11" s="24" t="n">
-        <f aca="false">SUM(B11:G11)</f>
-        <v>4551798.07373055</v>
-      </c>
-      <c r="I11" s="25" t="n">
-        <f aca="false">H11+Inputs!B36</f>
-        <v>5351798.07373055</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="10" t="n">
-        <v>74</v>
-      </c>
-      <c r="B12" s="17" t="n">
-        <f aca="false">'Roth Conversion'!J12</f>
-        <v>1643438.49403503</v>
-      </c>
-      <c r="C12" s="17" t="n">
-        <f aca="false">MAX(0,C11*(1+Inputs!B19)-'Withdrawal Plan'!K12)</f>
-        <v>1619193.74795459</v>
-      </c>
-      <c r="D12" s="17" t="n">
-        <f aca="false">D11*(1+Inputs!B19)</f>
-        <v>21589.2499727279</v>
-      </c>
-      <c r="E12" s="17" t="n">
-        <f aca="false">E11*(1+Inputs!B19)</f>
-        <v>107946.249863639</v>
-      </c>
-      <c r="F12" s="17" t="n">
-        <f aca="false">MAX(0,F11*(1+Inputs!B19)-'Withdrawal Plan'!M12)</f>
-        <v>176670.252310623</v>
-      </c>
-      <c r="G12" s="17" t="n">
-        <f aca="false">MAX(0,G11*(1+Inputs!B19)-'Withdrawal Plan'!L12)</f>
-        <v>1079462.49863639</v>
-      </c>
-      <c r="H12" s="24" t="n">
-        <f aca="false">SUM(B12:G12)</f>
-        <v>4648300.49277301</v>
-      </c>
-      <c r="I12" s="25" t="n">
-        <f aca="false">H12+Inputs!B36</f>
-        <v>5448300.49277301</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="10" t="n">
-        <v>75</v>
-      </c>
-      <c r="B13" s="17" t="n">
-        <f aca="false">'Roth Conversion'!J13</f>
-        <v>1521751.35638591</v>
-      </c>
-      <c r="C13" s="17" t="n">
-        <f aca="false">MAX(0,C12*(1+Inputs!B19)-'Withdrawal Plan'!K13)</f>
-        <v>1748729.24779096</v>
-      </c>
-      <c r="D13" s="17" t="n">
-        <f aca="false">D12*(1+Inputs!B19)</f>
-        <v>23316.3899705461</v>
-      </c>
-      <c r="E13" s="17" t="n">
-        <f aca="false">E12*(1+Inputs!B19)</f>
-        <v>116581.949852731</v>
-      </c>
-      <c r="F13" s="17" t="n">
-        <f aca="false">MAX(0,F12*(1+Inputs!B19)-'Withdrawal Plan'!M13)</f>
-        <v>187187.726424027</v>
-      </c>
-      <c r="G13" s="17" t="n">
-        <f aca="false">MAX(0,G12*(1+Inputs!B19)-'Withdrawal Plan'!L13)</f>
-        <v>1165819.49852731</v>
-      </c>
-      <c r="H13" s="24" t="n">
-        <f aca="false">SUM(B13:G13)</f>
-        <v>4763386.16895148</v>
-      </c>
-      <c r="I13" s="25" t="n">
-        <f aca="false">H13+Inputs!B36</f>
-        <v>5563386.16895148</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="10" t="n">
-        <v>76</v>
-      </c>
-      <c r="B14" s="17" t="n">
-        <f aca="false">'Roth Conversion'!J14</f>
-        <v>1401298.29029556</v>
-      </c>
-      <c r="C14" s="17" t="n">
-        <f aca="false">MAX(0,C13*(1+Inputs!B19)-'Withdrawal Plan'!K14)</f>
-        <v>1888627.58761424</v>
-      </c>
-      <c r="D14" s="17" t="n">
-        <f aca="false">D13*(1+Inputs!B19)</f>
-        <v>25181.7011681898</v>
-      </c>
-      <c r="E14" s="17" t="n">
-        <f aca="false">E13*(1+Inputs!B19)</f>
-        <v>125908.505840949</v>
-      </c>
-      <c r="F14" s="17" t="n">
-        <f aca="false">MAX(0,F13*(1+Inputs!B19)-'Withdrawal Plan'!M14)</f>
-        <v>198365.791162931</v>
-      </c>
-      <c r="G14" s="17" t="n">
-        <f aca="false">MAX(0,G13*(1+Inputs!B19)-'Withdrawal Plan'!L14)</f>
-        <v>1259085.05840949</v>
-      </c>
-      <c r="H14" s="24" t="n">
-        <f aca="false">SUM(B14:G14)</f>
-        <v>4898466.93449135</v>
-      </c>
-      <c r="I14" s="25" t="n">
-        <f aca="false">H14+Inputs!B36</f>
-        <v>5698466.93449135</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="10" t="n">
-        <v>77</v>
-      </c>
-      <c r="B15" s="17" t="n">
-        <f aca="false">'Roth Conversion'!J15</f>
-        <v>1282110.14755295</v>
-      </c>
-      <c r="C15" s="17" t="n">
-        <f aca="false">MAX(0,C14*(1+Inputs!B19)-'Withdrawal Plan'!K15)</f>
-        <v>2039717.79462337</v>
-      </c>
-      <c r="D15" s="17" t="n">
-        <f aca="false">D14*(1+Inputs!B19)</f>
-        <v>27196.237261645</v>
-      </c>
-      <c r="E15" s="17" t="n">
-        <f aca="false">E14*(1+Inputs!B19)</f>
-        <v>135981.186308225</v>
-      </c>
-      <c r="F15" s="17" t="n">
-        <f aca="false">MAX(0,F14*(1+Inputs!B19)-'Withdrawal Plan'!M15)</f>
-        <v>210248.253412196</v>
-      </c>
-      <c r="G15" s="17" t="n">
-        <f aca="false">MAX(0,G14*(1+Inputs!B19)-'Withdrawal Plan'!L15)</f>
-        <v>1359811.86308225</v>
-      </c>
-      <c r="H15" s="24" t="n">
-        <f aca="false">SUM(B15:G15)</f>
-        <v>5055065.48224064</v>
-      </c>
-      <c r="I15" s="25" t="n">
-        <f aca="false">H15+Inputs!B36</f>
-        <v>5855065.48224064</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="10" t="n">
-        <v>78</v>
-      </c>
-      <c r="B16" s="17" t="n">
-        <f aca="false">'Roth Conversion'!J16</f>
-        <v>1164218.55124177</v>
-      </c>
-      <c r="C16" s="17" t="n">
-        <f aca="false">MAX(0,C15*(1+Inputs!B19)-'Withdrawal Plan'!K16)</f>
-        <v>2202895.21819324</v>
-      </c>
-      <c r="D16" s="17" t="n">
-        <f aca="false">D15*(1+Inputs!B19)</f>
-        <v>29371.9362425766</v>
-      </c>
-      <c r="E16" s="17" t="n">
-        <f aca="false">E15*(1+Inputs!B19)</f>
-        <v>146859.681212883</v>
-      </c>
-      <c r="F16" s="17" t="n">
-        <f aca="false">MAX(0,F15*(1+Inputs!B19)-'Withdrawal Plan'!M16)</f>
-        <v>222881.972589215</v>
-      </c>
-      <c r="G16" s="17" t="n">
-        <f aca="false">MAX(0,G15*(1+Inputs!B19)-'Withdrawal Plan'!L16)</f>
-        <v>1468596.81212883</v>
-      </c>
-      <c r="H16" s="24" t="n">
-        <f aca="false">SUM(B16:G16)</f>
-        <v>5234824.17160852</v>
-      </c>
-      <c r="I16" s="25" t="n">
-        <f aca="false">H16+Inputs!B36</f>
-        <v>6034824.17160852</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="10" t="n">
-        <v>79</v>
-      </c>
-      <c r="B17" s="17" t="n">
-        <f aca="false">'Roth Conversion'!J17</f>
-        <v>1047655.91502281</v>
-      </c>
-      <c r="C17" s="17" t="n">
-        <f aca="false">MAX(0,C16*(1+Inputs!B19)-'Withdrawal Plan'!K17)</f>
-        <v>2379126.8356487</v>
-      </c>
-      <c r="D17" s="17" t="n">
-        <f aca="false">D16*(1+Inputs!B19)</f>
-        <v>31721.6911419827</v>
-      </c>
-      <c r="E17" s="17" t="n">
-        <f aca="false">E16*(1+Inputs!B19)</f>
-        <v>158608.455709914</v>
-      </c>
-      <c r="F17" s="17" t="n">
-        <f aca="false">MAX(0,F16*(1+Inputs!B19)-'Withdrawal Plan'!M17)</f>
-        <v>236317.082245596</v>
-      </c>
-      <c r="G17" s="17" t="n">
-        <f aca="false">MAX(0,G16*(1+Inputs!B19)-'Withdrawal Plan'!L17)</f>
-        <v>1586084.55709914</v>
-      </c>
-      <c r="H17" s="24" t="n">
-        <f aca="false">SUM(B17:G17)</f>
-        <v>5439514.53686815</v>
-      </c>
-      <c r="I17" s="25" t="n">
-        <f aca="false">H17+Inputs!B36</f>
-        <v>6239514.53686815</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="10" t="n">
-        <v>80</v>
-      </c>
-      <c r="B18" s="17" t="n">
-        <f aca="false">'Roth Conversion'!J18</f>
-        <v>932455.462898383</v>
-      </c>
-      <c r="C18" s="17" t="n">
-        <f aca="false">MAX(0,C17*(1+Inputs!B19)-'Withdrawal Plan'!K18)</f>
-        <v>2569456.9825006</v>
-      </c>
-      <c r="D18" s="17" t="n">
-        <f aca="false">D17*(1+Inputs!B19)</f>
-        <v>34259.4264333413</v>
-      </c>
-      <c r="E18" s="17" t="n">
-        <f aca="false">E17*(1+Inputs!B19)</f>
-        <v>171297.132166707</v>
-      </c>
-      <c r="F18" s="17" t="n">
-        <f aca="false">MAX(0,F17*(1+Inputs!B19)-'Withdrawal Plan'!M18)</f>
-        <v>250607.228266951</v>
-      </c>
-      <c r="G18" s="17" t="n">
-        <f aca="false">MAX(0,G17*(1+Inputs!B19)-'Withdrawal Plan'!L18)</f>
-        <v>1712971.32166707</v>
-      </c>
-      <c r="H18" s="24" t="n">
-        <f aca="false">SUM(B18:G18)</f>
-        <v>5671047.55393305</v>
-      </c>
-      <c r="I18" s="25" t="n">
-        <f aca="false">H18+Inputs!B36</f>
-        <v>6471047.55393305</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="10" t="n">
-        <v>81</v>
-      </c>
-      <c r="B19" s="17" t="n">
-        <f aca="false">'Roth Conversion'!J19</f>
-        <v>818651.249470843</v>
-      </c>
-      <c r="C19" s="17" t="n">
-        <f aca="false">MAX(0,C18*(1+Inputs!B19)-'Withdrawal Plan'!K19)</f>
-        <v>2775013.54110065</v>
-      </c>
-      <c r="D19" s="17" t="n">
-        <f aca="false">D18*(1+Inputs!B19)</f>
-        <v>37000.1805480087</v>
-      </c>
-      <c r="E19" s="17" t="n">
-        <f aca="false">E18*(1+Inputs!B19)</f>
-        <v>185000.902740043</v>
-      </c>
-      <c r="F19" s="17" t="n">
-        <f aca="false">MAX(0,F18*(1+Inputs!B19)-'Withdrawal Plan'!M19)</f>
-        <v>265809.824942099</v>
-      </c>
-      <c r="G19" s="17" t="n">
-        <f aca="false">MAX(0,G18*(1+Inputs!B19)-'Withdrawal Plan'!L19)</f>
-        <v>1850009.02740043</v>
-      </c>
-      <c r="H19" s="24" t="n">
-        <f aca="false">SUM(B19:G19)</f>
-        <v>5931484.72620207</v>
-      </c>
-      <c r="I19" s="25" t="n">
-        <f aca="false">H19+Inputs!B36</f>
-        <v>6731484.72620207</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="10" t="n">
-        <v>82</v>
-      </c>
-      <c r="B20" s="17" t="n">
-        <f aca="false">'Roth Conversion'!J20</f>
-        <v>706278.180707614</v>
-      </c>
       <c r="C20" s="17" t="n">
-        <f aca="false">MAX(0,C19*(1+Inputs!B19)-'Withdrawal Plan'!K20)</f>
+        <f aca="false">MAX(0,C19*(1+Inputs!B19)-'Withdrawal Plan'!K11)</f>
         <v>2997014.6243887</v>
       </c>
       <c r="D20" s="17" t="n">
@@ -4631,32 +4668,32 @@
         <v>199800.974959247</v>
       </c>
       <c r="F20" s="17" t="n">
-        <f aca="false">MAX(0,F19*(1+Inputs!B19)-'Withdrawal Plan'!M20)</f>
-        <v>281986.330271949</v>
+        <f aca="false">MAX(0,F19*(1+Inputs!B19)-'Withdrawal Plan'!M11)</f>
+        <v>582151.50167987</v>
       </c>
       <c r="G20" s="17" t="n">
-        <f aca="false">MAX(0,G19*(1+Inputs!B19)-'Withdrawal Plan'!L20)</f>
+        <f aca="false">MAX(0,G19*(1+Inputs!B19)-'Withdrawal Plan'!L11)</f>
         <v>1998009.74959247</v>
       </c>
       <c r="H20" s="24" t="n">
         <f aca="false">SUM(B20:G20)</f>
-        <v>6223050.05491183</v>
+        <v>7583266.64954875</v>
       </c>
       <c r="I20" s="25" t="n">
         <f aca="false">H20+Inputs!B36</f>
-        <v>7023050.05491183</v>
+        <v>8383266.64954875</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="10" t="n">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="B21" s="17" t="n">
-        <f aca="false">'Roth Conversion'!J21</f>
-        <v>595372.035225304</v>
+        <f aca="false">'Roth Conversion'!J12</f>
+        <v>1643438.49403503</v>
       </c>
       <c r="C21" s="17" t="n">
-        <f aca="false">MAX(0,C20*(1+Inputs!B19)-'Withdrawal Plan'!K21)</f>
+        <f aca="false">MAX(0,C20*(1+Inputs!B19)-'Withdrawal Plan'!K12)</f>
         <v>3236775.7943398</v>
       </c>
       <c r="D21" s="17" t="n">
@@ -4668,32 +4705,32 @@
         <v>215785.052955986</v>
       </c>
       <c r="F21" s="17" t="n">
-        <f aca="false">MAX(0,F20*(1+Inputs!B19)-'Withdrawal Plan'!M21)</f>
-        <v>299202.54199491</v>
+        <f aca="false">MAX(0,F20*(1+Inputs!B19)-'Withdrawal Plan'!M12)</f>
+        <v>625279.673174787</v>
       </c>
       <c r="G21" s="17" t="n">
-        <f aca="false">MAX(0,G20*(1+Inputs!B19)-'Withdrawal Plan'!L21)</f>
+        <f aca="false">MAX(0,G20*(1+Inputs!B19)-'Withdrawal Plan'!L12)</f>
         <v>2157850.52955986</v>
       </c>
       <c r="H21" s="24" t="n">
         <f aca="false">SUM(B21:G21)</f>
-        <v>6548142.96466706</v>
+        <v>7922286.55465667</v>
       </c>
       <c r="I21" s="25" t="n">
         <f aca="false">H21+Inputs!B36</f>
-        <v>7348142.96466706</v>
+        <v>8722286.55465667</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="10" t="n">
-        <v>84</v>
+        <v>75</v>
       </c>
       <c r="B22" s="17" t="n">
-        <f aca="false">'Roth Conversion'!J22</f>
-        <v>485969.486105936</v>
+        <f aca="false">'Roth Conversion'!J13</f>
+        <v>1521751.35638591</v>
       </c>
       <c r="C22" s="17" t="n">
-        <f aca="false">MAX(0,C21*(1+Inputs!B19)-'Withdrawal Plan'!K22)</f>
+        <f aca="false">MAX(0,C21*(1+Inputs!B19)-'Withdrawal Plan'!K13)</f>
         <v>3495717.85788698</v>
       </c>
       <c r="D22" s="17" t="n">
@@ -4705,32 +4742,32 @@
         <v>233047.857192465</v>
       </c>
       <c r="F22" s="17" t="n">
-        <f aca="false">MAX(0,F21*(1+Inputs!B19)-'Withdrawal Plan'!M22)</f>
-        <v>317528.915920769</v>
+        <f aca="false">MAX(0,F21*(1+Inputs!B19)-'Withdrawal Plan'!M13)</f>
+        <v>671685.900957324</v>
       </c>
       <c r="G22" s="17" t="n">
-        <f aca="false">MAX(0,G21*(1+Inputs!B19)-'Withdrawal Plan'!L22)</f>
+        <f aca="false">MAX(0,G21*(1+Inputs!B19)-'Withdrawal Plan'!L13)</f>
         <v>2330478.57192465</v>
       </c>
       <c r="H22" s="24" t="n">
         <f aca="false">SUM(B22:G22)</f>
-        <v>6909352.2604693</v>
+        <v>8299291.11578583</v>
       </c>
       <c r="I22" s="25" t="n">
         <f aca="false">H22+Inputs!B36</f>
-        <v>7709352.2604693</v>
+        <v>9099291.11578583</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="n">
-        <v>85</v>
+        <v>76</v>
       </c>
       <c r="B23" s="17" t="n">
-        <f aca="false">'Roth Conversion'!J23</f>
-        <v>378108.123258585</v>
+        <f aca="false">'Roth Conversion'!J14</f>
+        <v>1401298.29029556</v>
       </c>
       <c r="C23" s="17" t="n">
-        <f aca="false">MAX(0,C22*(1+Inputs!B19)-'Withdrawal Plan'!K23)</f>
+        <f aca="false">MAX(0,C22*(1+Inputs!B19)-'Withdrawal Plan'!K14)</f>
         <v>3775375.28651794</v>
       </c>
       <c r="D23" s="17" t="n">
@@ -4742,25 +4779,372 @@
         <v>251691.685767863</v>
       </c>
       <c r="F23" s="17" t="n">
-        <f aca="false">MAX(0,F22*(1+Inputs!B19)-'Withdrawal Plan'!M23)</f>
-        <v>337040.90828901</v>
+        <f aca="false">MAX(0,F22*(1+Inputs!B19)-'Withdrawal Plan'!M14)</f>
+        <v>721623.819658892</v>
       </c>
       <c r="G23" s="17" t="n">
-        <f aca="false">MAX(0,G22*(1+Inputs!B19)-'Withdrawal Plan'!L23)</f>
+        <f aca="false">MAX(0,G22*(1+Inputs!B19)-'Withdrawal Plan'!L14)</f>
         <v>2516916.85767863</v>
       </c>
       <c r="H23" s="24" t="n">
         <f aca="false">SUM(B23:G23)</f>
-        <v>7309471.1986656</v>
+        <v>8717244.27707245</v>
       </c>
       <c r="I23" s="25" t="n">
         <f aca="false">H23+Inputs!B36</f>
-        <v>8109471.1986656</v>
-      </c>
+        <v>9517244.27707245</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="10" t="n">
+        <v>77</v>
+      </c>
+      <c r="B24" s="17" t="n">
+        <f aca="false">'Roth Conversion'!J15</f>
+        <v>1282110.14755295</v>
+      </c>
+      <c r="C24" s="17" t="n">
+        <f aca="false">MAX(0,C23*(1+Inputs!B19)-'Withdrawal Plan'!K15)</f>
+        <v>4077405.30943937</v>
+      </c>
+      <c r="D24" s="17" t="n">
+        <f aca="false">D23*(1+Inputs!B19)</f>
+        <v>54365.4041258583</v>
+      </c>
+      <c r="E24" s="17" t="n">
+        <f aca="false">E23*(1+Inputs!B19)</f>
+        <v>271827.020629292</v>
+      </c>
+      <c r="F24" s="17" t="n">
+        <f aca="false">MAX(0,F23*(1+Inputs!B19)-'Withdrawal Plan'!M15)</f>
+        <v>775366.924187834</v>
+      </c>
+      <c r="G24" s="17" t="n">
+        <f aca="false">MAX(0,G23*(1+Inputs!B19)-'Withdrawal Plan'!L15)</f>
+        <v>2718270.20629292</v>
+      </c>
+      <c r="H24" s="24" t="n">
+        <f aca="false">SUM(B24:G24)</f>
+        <v>9179345.01222822</v>
+      </c>
+      <c r="I24" s="25" t="n">
+        <f aca="false">H24+Inputs!B36</f>
+        <v>9979345.01222822</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="10" t="n">
+        <v>78</v>
+      </c>
+      <c r="B25" s="17" t="n">
+        <f aca="false">'Roth Conversion'!J16</f>
+        <v>1164218.55124177</v>
+      </c>
+      <c r="C25" s="17" t="n">
+        <f aca="false">MAX(0,C24*(1+Inputs!B19)-'Withdrawal Plan'!K16)</f>
+        <v>4403597.73419453</v>
+      </c>
+      <c r="D25" s="17" t="n">
+        <f aca="false">D24*(1+Inputs!B19)</f>
+        <v>58714.636455927</v>
+      </c>
+      <c r="E25" s="17" t="n">
+        <f aca="false">E24*(1+Inputs!B19)</f>
+        <v>293573.182279635</v>
+      </c>
+      <c r="F25" s="17" t="n">
+        <f aca="false">MAX(0,F24*(1+Inputs!B19)-'Withdrawal Plan'!M16)</f>
+        <v>833210.137026903</v>
+      </c>
+      <c r="G25" s="17" t="n">
+        <f aca="false">MAX(0,G24*(1+Inputs!B19)-'Withdrawal Plan'!L16)</f>
+        <v>2935731.82279635</v>
+      </c>
+      <c r="H25" s="24" t="n">
+        <f aca="false">SUM(B25:G25)</f>
+        <v>9689046.06399511</v>
+      </c>
+      <c r="I25" s="25" t="n">
+        <f aca="false">H25+Inputs!B36</f>
+        <v>10489046.0639951</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="10" t="n">
+        <v>79</v>
+      </c>
+      <c r="B26" s="17" t="n">
+        <f aca="false">'Roth Conversion'!J17</f>
+        <v>1047655.91502281</v>
+      </c>
+      <c r="C26" s="17" t="n">
+        <f aca="false">MAX(0,C25*(1+Inputs!B19)-'Withdrawal Plan'!K17)</f>
+        <v>4755885.55293009</v>
+      </c>
+      <c r="D26" s="17" t="n">
+        <f aca="false">D25*(1+Inputs!B19)</f>
+        <v>63411.8073724012</v>
+      </c>
+      <c r="E26" s="17" t="n">
+        <f aca="false">E25*(1+Inputs!B19)</f>
+        <v>317059.036862006</v>
+      </c>
+      <c r="F26" s="17" t="n">
+        <f aca="false">MAX(0,F25*(1+Inputs!B19)-'Withdrawal Plan'!M17)</f>
+        <v>895471.4998383</v>
+      </c>
+      <c r="G26" s="17" t="n">
+        <f aca="false">MAX(0,G25*(1+Inputs!B19)-'Withdrawal Plan'!L17)</f>
+        <v>3170590.36862006</v>
+      </c>
+      <c r="H26" s="24" t="n">
+        <f aca="false">SUM(B26:G26)</f>
+        <v>10250074.1806457</v>
+      </c>
+      <c r="I26" s="25" t="n">
+        <f aca="false">H26+Inputs!B36</f>
+        <v>11050074.1806457</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="10" t="n">
+        <v>80</v>
+      </c>
+      <c r="B27" s="17" t="n">
+        <f aca="false">'Roth Conversion'!J18</f>
+        <v>932455.462898383</v>
+      </c>
+      <c r="C27" s="17" t="n">
+        <f aca="false">MAX(0,C26*(1+Inputs!B19)-'Withdrawal Plan'!K18)</f>
+        <v>5136356.39716449</v>
+      </c>
+      <c r="D27" s="17" t="n">
+        <f aca="false">D26*(1+Inputs!B19)</f>
+        <v>68484.7519621933</v>
+      </c>
+      <c r="E27" s="17" t="n">
+        <f aca="false">E26*(1+Inputs!B19)</f>
+        <v>342423.759810966</v>
+      </c>
+      <c r="F27" s="17" t="n">
+        <f aca="false">MAX(0,F26*(1+Inputs!B19)-'Withdrawal Plan'!M18)</f>
+        <v>962493.999267071</v>
+      </c>
+      <c r="G27" s="17" t="n">
+        <f aca="false">MAX(0,G26*(1+Inputs!B19)-'Withdrawal Plan'!L18)</f>
+        <v>3424237.59810966</v>
+      </c>
+      <c r="H27" s="24" t="n">
+        <f aca="false">SUM(B27:G27)</f>
+        <v>10866451.9692128</v>
+      </c>
+      <c r="I27" s="25" t="n">
+        <f aca="false">H27+Inputs!B36</f>
+        <v>11666451.9692128</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="10" t="n">
+        <v>81</v>
+      </c>
+      <c r="B28" s="17" t="n">
+        <f aca="false">'Roth Conversion'!J19</f>
+        <v>818651.249470843</v>
+      </c>
+      <c r="C28" s="17" t="n">
+        <f aca="false">MAX(0,C27*(1+Inputs!B19)-'Withdrawal Plan'!K19)</f>
+        <v>5547264.90893765</v>
+      </c>
+      <c r="D28" s="17" t="n">
+        <f aca="false">D27*(1+Inputs!B19)</f>
+        <v>73963.5321191687</v>
+      </c>
+      <c r="E28" s="17" t="n">
+        <f aca="false">E27*(1+Inputs!B19)</f>
+        <v>369817.660595844</v>
+      </c>
+      <c r="F28" s="17" t="n">
+        <f aca="false">MAX(0,F27*(1+Inputs!B19)-'Withdrawal Plan'!M19)</f>
+        <v>1034647.53762223</v>
+      </c>
+      <c r="G28" s="17" t="n">
+        <f aca="false">MAX(0,G27*(1+Inputs!B19)-'Withdrawal Plan'!L19)</f>
+        <v>3698176.60595844</v>
+      </c>
+      <c r="H28" s="24" t="n">
+        <f aca="false">SUM(B28:G28)</f>
+        <v>11542521.4947042</v>
+      </c>
+      <c r="I28" s="25" t="n">
+        <f aca="false">H28+Inputs!B36</f>
+        <v>12342521.4947042</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="10" t="n">
+        <v>82</v>
+      </c>
+      <c r="B29" s="17" t="n">
+        <f aca="false">'Roth Conversion'!J20</f>
+        <v>706278.180707614</v>
+      </c>
+      <c r="C29" s="17" t="n">
+        <f aca="false">MAX(0,C28*(1+Inputs!B19)-'Withdrawal Plan'!K20)</f>
+        <v>5991046.10165267</v>
+      </c>
+      <c r="D29" s="17" t="n">
+        <f aca="false">D28*(1+Inputs!B19)</f>
+        <v>79880.6146887023</v>
+      </c>
+      <c r="E29" s="17" t="n">
+        <f aca="false">E28*(1+Inputs!B19)</f>
+        <v>399403.073443511</v>
+      </c>
+      <c r="F29" s="17" t="n">
+        <f aca="false">MAX(0,F28*(1+Inputs!B19)-'Withdrawal Plan'!M20)</f>
+        <v>1112331.05996649</v>
+      </c>
+      <c r="G29" s="17" t="n">
+        <f aca="false">MAX(0,G28*(1+Inputs!B19)-'Withdrawal Plan'!L20)</f>
+        <v>3994030.73443511</v>
+      </c>
+      <c r="H29" s="24" t="n">
+        <f aca="false">SUM(B29:G29)</f>
+        <v>12282969.7648941</v>
+      </c>
+      <c r="I29" s="25" t="n">
+        <f aca="false">H29+Inputs!B36</f>
+        <v>13082969.7648941</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="10" t="n">
+        <v>83</v>
+      </c>
+      <c r="B30" s="17" t="n">
+        <f aca="false">'Roth Conversion'!J21</f>
+        <v>595372.035225304</v>
+      </c>
+      <c r="C30" s="17" t="n">
+        <f aca="false">MAX(0,C29*(1+Inputs!B19)-'Withdrawal Plan'!K21)</f>
+        <v>6470329.78978488</v>
+      </c>
+      <c r="D30" s="17" t="n">
+        <f aca="false">D29*(1+Inputs!B19)</f>
+        <v>86271.0638637984</v>
+      </c>
+      <c r="E30" s="17" t="n">
+        <f aca="false">E29*(1+Inputs!B19)</f>
+        <v>431355.319318992</v>
+      </c>
+      <c r="F30" s="17" t="n">
+        <f aca="false">MAX(0,F29*(1+Inputs!B19)-'Withdrawal Plan'!M21)</f>
+        <v>1195974.85006501</v>
+      </c>
+      <c r="G30" s="17" t="n">
+        <f aca="false">MAX(0,G29*(1+Inputs!B19)-'Withdrawal Plan'!L21)</f>
+        <v>4313553.19318992</v>
+      </c>
+      <c r="H30" s="24" t="n">
+        <f aca="false">SUM(B30:G30)</f>
+        <v>13092856.2514479</v>
+      </c>
+      <c r="I30" s="25" t="n">
+        <f aca="false">H30+Inputs!B36</f>
+        <v>13892856.2514479</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="10" t="n">
+        <v>84</v>
+      </c>
+      <c r="B31" s="17" t="n">
+        <f aca="false">'Roth Conversion'!J22</f>
+        <v>485969.486105936</v>
+      </c>
+      <c r="C31" s="17" t="n">
+        <f aca="false">MAX(0,C30*(1+Inputs!B19)-'Withdrawal Plan'!K22)</f>
+        <v>6987956.17296767</v>
+      </c>
+      <c r="D31" s="17" t="n">
+        <f aca="false">D30*(1+Inputs!B19)</f>
+        <v>93172.7489729023</v>
+      </c>
+      <c r="E31" s="17" t="n">
+        <f aca="false">E30*(1+Inputs!B19)</f>
+        <v>465863.744864511</v>
+      </c>
+      <c r="F31" s="17" t="n">
+        <f aca="false">MAX(0,F30*(1+Inputs!B19)-'Withdrawal Plan'!M22)</f>
+        <v>1286043.00863648</v>
+      </c>
+      <c r="G31" s="17" t="n">
+        <f aca="false">MAX(0,G30*(1+Inputs!B19)-'Withdrawal Plan'!L22)</f>
+        <v>4658637.44864512</v>
+      </c>
+      <c r="H31" s="24" t="n">
+        <f aca="false">SUM(B31:G31)</f>
+        <v>13977642.6101926</v>
+      </c>
+      <c r="I31" s="25" t="n">
+        <f aca="false">H31+Inputs!B36</f>
+        <v>14777642.6101926</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="10" t="n">
+        <v>85</v>
+      </c>
+      <c r="B32" s="17" t="n">
+        <f aca="false">'Roth Conversion'!J23</f>
+        <v>378108.123258585</v>
+      </c>
+      <c r="C32" s="17" t="n">
+        <f aca="false">MAX(0,C31*(1+Inputs!B19)-'Withdrawal Plan'!K23)</f>
+        <v>7546992.66680509</v>
+      </c>
+      <c r="D32" s="17" t="n">
+        <f aca="false">D31*(1+Inputs!B19)</f>
+        <v>100626.568890735</v>
+      </c>
+      <c r="E32" s="17" t="n">
+        <f aca="false">E31*(1+Inputs!B19)</f>
+        <v>503132.844453672</v>
+      </c>
+      <c r="F32" s="17" t="n">
+        <f aca="false">MAX(0,F31*(1+Inputs!B19)-'Withdrawal Plan'!M23)</f>
+        <v>1383036.12842198</v>
+      </c>
+      <c r="G32" s="17" t="n">
+        <f aca="false">MAX(0,G31*(1+Inputs!B19)-'Withdrawal Plan'!L23)</f>
+        <v>5031328.44453672</v>
+      </c>
+      <c r="H32" s="24" t="n">
+        <f aca="false">SUM(B32:G32)</f>
+        <v>14943224.7763668</v>
+      </c>
+      <c r="I32" s="25" t="n">
+        <f aca="false">H32+Inputs!B36</f>
+        <v>15743224.7763668</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="30" t="s">
+        <v>87</v>
+      </c>
+      <c r="B34" s="30"/>
+      <c r="C34" s="30"/>
+      <c r="D34" s="30"/>
+      <c r="E34" s="30"/>
+      <c r="F34" s="30"/>
+      <c r="G34" s="30"/>
+      <c r="H34" s="30"/>
+      <c r="I34" s="30"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A34:I34"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -4787,120 +5171,120 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B1" s="8"/>
       <c r="C1" s="8"/>
       <c r="D1" s="8"/>
     </row>
     <row r="2" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="26" t="s">
-        <v>88</v>
-      </c>
-      <c r="B2" s="26" t="s">
+      <c r="A2" s="31" t="s">
         <v>89</v>
       </c>
-      <c r="C2" s="26" t="s">
+      <c r="B2" s="31" t="s">
         <v>90</v>
       </c>
-      <c r="D2" s="26" t="s">
+      <c r="C2" s="31" t="s">
         <v>91</v>
       </c>
+      <c r="D2" s="31" t="s">
+        <v>92</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="27" t="s">
-        <v>92</v>
-      </c>
-      <c r="B3" s="28" t="n">
+      <c r="A3" s="32" t="s">
+        <v>93</v>
+      </c>
+      <c r="B3" s="33" t="n">
         <f aca="false">Inputs!B22</f>
         <v>3330</v>
       </c>
-      <c r="C3" s="28" t="n">
+      <c r="C3" s="33" t="n">
         <f aca="false">Inputs!B23</f>
         <v>3972</v>
       </c>
-      <c r="D3" s="28" t="n">
+      <c r="D3" s="33" t="n">
         <f aca="false">Inputs!B24</f>
         <v>5200</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="27" t="s">
-        <v>93</v>
-      </c>
-      <c r="B4" s="29" t="n">
+      <c r="A4" s="32" t="s">
+        <v>94</v>
+      </c>
+      <c r="B4" s="34" t="n">
         <f aca="false">Inputs!B22*12</f>
         <v>39960</v>
       </c>
-      <c r="C4" s="29" t="n">
+      <c r="C4" s="34" t="n">
         <f aca="false">Inputs!B23*12</f>
         <v>47664</v>
       </c>
-      <c r="D4" s="29" t="n">
+      <c r="D4" s="34" t="n">
         <f aca="false">Inputs!B24*12</f>
         <v>62400</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="27" t="s">
-        <v>94</v>
-      </c>
-      <c r="B5" s="30" t="n">
+      <c r="A5" s="32" t="s">
+        <v>95</v>
+      </c>
+      <c r="B5" s="35" t="n">
         <f aca="false">85-65</f>
         <v>20</v>
       </c>
-      <c r="C5" s="30" t="n">
+      <c r="C5" s="35" t="n">
         <f aca="false">85-67</f>
         <v>18</v>
       </c>
-      <c r="D5" s="30" t="n">
+      <c r="D5" s="35" t="n">
         <f aca="false">85-70</f>
         <v>15</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="27" t="s">
-        <v>95</v>
-      </c>
-      <c r="B6" s="29" t="n">
+      <c r="A6" s="32" t="s">
+        <v>96</v>
+      </c>
+      <c r="B6" s="34" t="n">
         <f aca="false">Inputs!B22*12*20</f>
         <v>799200</v>
       </c>
-      <c r="C6" s="29" t="n">
+      <c r="C6" s="34" t="n">
         <f aca="false">Inputs!B23*12*18</f>
         <v>857952</v>
       </c>
-      <c r="D6" s="29" t="n">
+      <c r="D6" s="34" t="n">
         <f aca="false">Inputs!B24*12*15</f>
         <v>936000</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="27" t="s">
-        <v>96</v>
-      </c>
-      <c r="B7" s="30" t="s">
+      <c r="A7" s="32" t="s">
         <v>97</v>
       </c>
-      <c r="C7" s="30" t="s">
+      <c r="B7" s="35" t="s">
         <v>98</v>
       </c>
-      <c r="D7" s="30" t="s">
+      <c r="C7" s="35" t="s">
         <v>99</v>
       </c>
+      <c r="D7" s="35" t="s">
+        <v>100</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="27" t="s">
-        <v>100</v>
-      </c>
-      <c r="B8" s="31" t="s">
+      <c r="A8" s="32" t="s">
         <v>101</v>
       </c>
-      <c r="C8" s="31" t="s">
+      <c r="B8" s="36" t="s">
         <v>102</v>
       </c>
-      <c r="D8" s="31" t="s">
+      <c r="C8" s="36" t="s">
         <v>103</v>
+      </c>
+      <c r="D8" s="36" t="s">
+        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -4932,96 +5316,96 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B1" s="8"/>
     </row>
     <row r="2" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="32" t="s">
-        <v>105</v>
-      </c>
-      <c r="B2" s="33" t="s">
+      <c r="A2" s="37" t="s">
         <v>106</v>
       </c>
+      <c r="B2" s="38" t="s">
+        <v>107</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="34" t="s">
-        <v>107</v>
-      </c>
-      <c r="B3" s="35" t="s">
+      <c r="A3" s="39" t="s">
         <v>108</v>
       </c>
+      <c r="B3" s="40" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="36" t="s">
-        <v>109</v>
-      </c>
-      <c r="B4" s="37" t="s">
+      <c r="A4" s="41" t="s">
         <v>110</v>
       </c>
+      <c r="B4" s="42" t="s">
+        <v>111</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="34" t="s">
-        <v>111</v>
-      </c>
-      <c r="B5" s="35" t="s">
+      <c r="A5" s="39" t="s">
         <v>112</v>
       </c>
+      <c r="B5" s="40" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="36" t="s">
-        <v>113</v>
-      </c>
-      <c r="B6" s="37" t="s">
+      <c r="A6" s="41" t="s">
         <v>114</v>
       </c>
+      <c r="B6" s="42" t="s">
+        <v>115</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="34" t="s">
-        <v>115</v>
-      </c>
-      <c r="B7" s="35" t="s">
+      <c r="A7" s="39" t="s">
         <v>116</v>
       </c>
+      <c r="B7" s="40" t="s">
+        <v>117</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="36" t="s">
-        <v>117</v>
-      </c>
-      <c r="B8" s="37" t="s">
+      <c r="A8" s="41" t="s">
         <v>118</v>
       </c>
+      <c r="B8" s="42" t="s">
+        <v>119</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="34" t="s">
-        <v>119</v>
-      </c>
-      <c r="B9" s="35" t="s">
+      <c r="A9" s="39" t="s">
         <v>120</v>
       </c>
+      <c r="B9" s="40" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="36" t="s">
-        <v>121</v>
-      </c>
-      <c r="B10" s="37" t="s">
+      <c r="A10" s="41" t="s">
         <v>122</v>
       </c>
+      <c r="B10" s="42" t="s">
+        <v>123</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="34" t="s">
-        <v>123</v>
-      </c>
-      <c r="B11" s="35" t="s">
+      <c r="A11" s="39" t="s">
         <v>124</v>
       </c>
+      <c r="B11" s="40" t="s">
+        <v>125</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="36" t="s">
-        <v>125</v>
-      </c>
-      <c r="B12" s="37" t="s">
+      <c r="A12" s="41" t="s">
         <v>126</v>
+      </c>
+      <c r="B12" s="42" t="s">
+        <v>127</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix charts 3 and 4 - use local data area in Charts sheet
</commit_message>
<xml_diff>
--- a/retirement_planner.xlsx
+++ b/retirement_planner.xlsx
@@ -730,7 +730,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="9">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="\$#,##0;&quot;($&quot;#,##0\);\-"/>
     <numFmt numFmtId="166" formatCode="0.0%;\(0.0%\);\-"/>
@@ -739,7 +739,6 @@
     <numFmt numFmtId="169" formatCode="0.0"/>
     <numFmt numFmtId="170" formatCode="0"/>
     <numFmt numFmtId="171" formatCode="0%"/>
-    <numFmt numFmtId="172" formatCode="\$#,##0"/>
   </numFmts>
   <fonts count="41">
     <font>
@@ -1205,7 +1204,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="88">
+  <cellXfs count="86">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1538,23 +1537,15 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="25" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="25" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="37" fillId="13" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="37" fillId="13" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1634,7 +1625,6 @@
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
-  <c:style val="10"/>
   <c:chart>
     <c:title>
       <c:tx>
@@ -1702,23 +1692,27 @@
           <c:invertIfNegative val="0"/>
           <c:dLbls>
             <c:txPr>
-              <a:bodyPr wrap="none"/>
+              <a:bodyPr wrap="square"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="ctr"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
-            <c:separator> </c:separator>
+            <c:separator>; </c:separator>
             <c:showLeaderLines val="1"/>
             <c:leaderLines>
               <c:spPr>
@@ -1960,23 +1954,27 @@
           <c:invertIfNegative val="0"/>
           <c:dLbls>
             <c:txPr>
-              <a:bodyPr wrap="none"/>
+              <a:bodyPr wrap="square"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="ctr"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
-            <c:separator> </c:separator>
+            <c:separator>; </c:separator>
             <c:showLeaderLines val="1"/>
             <c:leaderLines>
               <c:spPr>
@@ -2218,23 +2216,27 @@
           <c:invertIfNegative val="0"/>
           <c:dLbls>
             <c:txPr>
-              <a:bodyPr wrap="none"/>
+              <a:bodyPr wrap="square"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="ctr"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
-            <c:separator> </c:separator>
+            <c:separator>; </c:separator>
             <c:showLeaderLines val="1"/>
             <c:leaderLines>
               <c:spPr>
@@ -2476,23 +2478,27 @@
           <c:invertIfNegative val="0"/>
           <c:dLbls>
             <c:txPr>
-              <a:bodyPr wrap="none"/>
+              <a:bodyPr wrap="square"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="ctr"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
-            <c:separator> </c:separator>
+            <c:separator>; </c:separator>
             <c:showLeaderLines val="1"/>
             <c:leaderLines>
               <c:spPr>
@@ -2734,23 +2740,27 @@
           <c:invertIfNegative val="0"/>
           <c:dLbls>
             <c:txPr>
-              <a:bodyPr wrap="none"/>
+              <a:bodyPr wrap="square"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="ctr"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
-            <c:separator> </c:separator>
+            <c:separator>; </c:separator>
             <c:showLeaderLines val="1"/>
             <c:leaderLines>
               <c:spPr>
@@ -2992,23 +3002,27 @@
           <c:invertIfNegative val="0"/>
           <c:dLbls>
             <c:txPr>
-              <a:bodyPr wrap="none"/>
+              <a:bodyPr wrap="square"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="ctr"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
-            <c:separator> </c:separator>
+            <c:separator>; </c:separator>
             <c:showLeaderLines val="1"/>
             <c:leaderLines>
               <c:spPr>
@@ -3225,11 +3239,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="67194089"/>
-        <c:axId val="5062873"/>
+        <c:axId val="25963316"/>
+        <c:axId val="99463107"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="67194089"/>
+        <c:axId val="25963316"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3268,7 +3282,7 @@
             </a:ln>
           </c:spPr>
         </c:title>
-        <c:numFmt formatCode="0" sourceLinked="1"/>
+        <c:numFmt formatCode="0" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -3294,7 +3308,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="5062873"/>
+        <c:crossAx val="99463107"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3302,7 +3316,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="5062873"/>
+        <c:axId val="99463107"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3350,7 +3364,7 @@
             </a:ln>
           </c:spPr>
         </c:title>
-        <c:numFmt formatCode="\$#,##0" sourceLinked="1"/>
+        <c:numFmt formatCode="\$#,##0" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -3376,7 +3390,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="67194089"/>
+        <c:crossAx val="25963316"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3435,7 +3449,6 @@
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
-  <c:style val="10"/>
   <c:chart>
     <c:title>
       <c:tx>
@@ -3503,23 +3516,27 @@
           <c:invertIfNegative val="0"/>
           <c:dLbls>
             <c:txPr>
-              <a:bodyPr wrap="none"/>
+              <a:bodyPr wrap="square"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="ctr"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
-            <c:separator> </c:separator>
+            <c:separator>; </c:separator>
             <c:showLeaderLines val="1"/>
             <c:leaderLines>
               <c:spPr>
@@ -3707,23 +3724,27 @@
           <c:invertIfNegative val="0"/>
           <c:dLbls>
             <c:txPr>
-              <a:bodyPr wrap="none"/>
+              <a:bodyPr wrap="square"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="ctr"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
-            <c:separator> </c:separator>
+            <c:separator>; </c:separator>
             <c:showLeaderLines val="1"/>
             <c:leaderLines>
               <c:spPr>
@@ -3911,23 +3932,27 @@
           <c:invertIfNegative val="0"/>
           <c:dLbls>
             <c:txPr>
-              <a:bodyPr wrap="none"/>
+              <a:bodyPr wrap="square"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="ctr"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
-            <c:separator> </c:separator>
+            <c:separator>; </c:separator>
             <c:showLeaderLines val="1"/>
             <c:leaderLines>
               <c:spPr>
@@ -4115,23 +4140,27 @@
           <c:invertIfNegative val="0"/>
           <c:dLbls>
             <c:txPr>
-              <a:bodyPr wrap="none"/>
+              <a:bodyPr wrap="square"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="ctr"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
-            <c:separator> </c:separator>
+            <c:separator>; </c:separator>
             <c:showLeaderLines val="1"/>
             <c:leaderLines>
               <c:spPr>
@@ -4319,23 +4348,27 @@
           <c:invertIfNegative val="0"/>
           <c:dLbls>
             <c:txPr>
-              <a:bodyPr wrap="none"/>
+              <a:bodyPr wrap="square"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="ctr"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
-            <c:separator> </c:separator>
+            <c:separator>; </c:separator>
             <c:showLeaderLines val="1"/>
             <c:leaderLines>
               <c:spPr>
@@ -4498,11 +4531,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="8645488"/>
-        <c:axId val="91649147"/>
+        <c:axId val="94463532"/>
+        <c:axId val="24927322"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="8645488"/>
+        <c:axId val="94463532"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4541,7 +4574,7 @@
             </a:ln>
           </c:spPr>
         </c:title>
-        <c:numFmt formatCode="0" sourceLinked="1"/>
+        <c:numFmt formatCode="0" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -4567,7 +4600,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="91649147"/>
+        <c:crossAx val="24927322"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4575,7 +4608,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="91649147"/>
+        <c:axId val="24927322"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4623,7 +4656,7 @@
             </a:ln>
           </c:spPr>
         </c:title>
-        <c:numFmt formatCode="\$#,##0" sourceLinked="1"/>
+        <c:numFmt formatCode="\$#,##0" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -4649,7 +4682,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="8645488"/>
+        <c:crossAx val="94463532"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -5377,11 +5410,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="83039156"/>
-        <c:axId val="64966211"/>
+        <c:axId val="92312010"/>
+        <c:axId val="20534526"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="83039156"/>
+        <c:axId val="92312010"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5446,7 +5479,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="64966211"/>
+        <c:crossAx val="20534526"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5454,7 +5487,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="64966211"/>
+        <c:axId val="20534526"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5528,7 +5561,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="83039156"/>
+        <c:crossAx val="92312010"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -6050,11 +6083,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="64165522"/>
-        <c:axId val="66198551"/>
+        <c:axId val="40997645"/>
+        <c:axId val="34236095"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="64165522"/>
+        <c:axId val="40997645"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6119,7 +6152,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="66198551"/>
+        <c:crossAx val="34236095"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -6127,7 +6160,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="66198551"/>
+        <c:axId val="34236095"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6201,7 +6234,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="64165522"/>
+        <c:crossAx val="40997645"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -7131,9 +7164,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>21</xdr:col>
-      <xdr:colOff>551160</xdr:colOff>
+      <xdr:colOff>550800</xdr:colOff>
       <xdr:row>32</xdr:row>
-      <xdr:rowOff>44640</xdr:rowOff>
+      <xdr:rowOff>44280</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -7142,7 +7175,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="8881200" y="438120"/>
-        <a:ext cx="8639640" cy="5759640"/>
+        <a:ext cx="8639280" cy="5759280"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -7161,9 +7194,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>21</xdr:col>
-      <xdr:colOff>551160</xdr:colOff>
+      <xdr:colOff>550800</xdr:colOff>
       <xdr:row>64</xdr:row>
-      <xdr:rowOff>44640</xdr:rowOff>
+      <xdr:rowOff>44280</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -7172,7 +7205,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="8881200" y="6534000"/>
-        <a:ext cx="8639640" cy="5759640"/>
+        <a:ext cx="8639280" cy="5759280"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -8031,7 +8064,7 @@
   <dimension ref="A1:T79"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="1" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="1" style="1" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8058,7 +8091,7 @@
       <c r="S1" s="83"/>
       <c r="T1" s="83"/>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="84" t="s">
         <v>60</v>
       </c>
@@ -8084,1027 +8117,1027 @@
         <v>198</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="85" t="n">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="47" t="n">
         <f aca="false">Portfolio!A3</f>
         <v>56</v>
       </c>
-      <c r="B4" s="86" t="n">
+      <c r="B4" s="85" t="n">
         <f aca="false">Portfolio!B3</f>
         <v>3037518.75</v>
       </c>
-      <c r="C4" s="86" t="n">
+      <c r="C4" s="85" t="n">
         <f aca="false">Portfolio!C3</f>
         <v>810000</v>
       </c>
-      <c r="D4" s="86" t="n">
+      <c r="D4" s="85" t="n">
         <f aca="false">Portfolio!D3</f>
         <v>10800</v>
       </c>
-      <c r="E4" s="86" t="n">
+      <c r="E4" s="85" t="n">
         <f aca="false">Portfolio!E3</f>
         <v>54000</v>
       </c>
-      <c r="F4" s="86" t="n">
+      <c r="F4" s="85" t="n">
         <f aca="false">Portfolio!F3</f>
         <v>116640</v>
       </c>
-      <c r="G4" s="86" t="n">
+      <c r="G4" s="85" t="n">
         <f aca="false">Portfolio!G3</f>
         <v>540000</v>
       </c>
-      <c r="H4" s="86" t="n">
+      <c r="H4" s="85" t="n">
         <f aca="false">Portfolio!I3</f>
         <v>5368958.75</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="85" t="n">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="47" t="n">
         <f aca="false">Portfolio!A4</f>
         <v>57</v>
       </c>
-      <c r="B5" s="86" t="n">
+      <c r="B5" s="85" t="n">
         <f aca="false">Portfolio!B4</f>
         <v>3318039</v>
       </c>
-      <c r="C5" s="86" t="n">
+      <c r="C5" s="85" t="n">
         <f aca="false">Portfolio!C4</f>
         <v>874800</v>
       </c>
-      <c r="D5" s="86" t="n">
+      <c r="D5" s="85" t="n">
         <f aca="false">Portfolio!D4</f>
         <v>11664</v>
       </c>
-      <c r="E5" s="86" t="n">
+      <c r="E5" s="85" t="n">
         <f aca="false">Portfolio!E4</f>
         <v>58320</v>
       </c>
-      <c r="F5" s="86" t="n">
+      <c r="F5" s="85" t="n">
         <f aca="false">Portfolio!F4</f>
         <v>134611.2</v>
       </c>
-      <c r="G5" s="86" t="n">
+      <c r="G5" s="85" t="n">
         <f aca="false">Portfolio!G4</f>
         <v>583200</v>
       </c>
-      <c r="H5" s="86" t="n">
+      <c r="H5" s="85" t="n">
         <f aca="false">Portfolio!I4</f>
         <v>5816634.2</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="85" t="n">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="47" t="n">
         <f aca="false">Portfolio!A5</f>
         <v>58</v>
       </c>
-      <c r="B6" s="86" t="n">
+      <c r="B6" s="85" t="n">
         <f aca="false">Portfolio!B5</f>
         <v>3621000.87</v>
       </c>
-      <c r="C6" s="86" t="n">
+      <c r="C6" s="85" t="n">
         <f aca="false">Portfolio!C5</f>
         <v>944784</v>
       </c>
-      <c r="D6" s="86" t="n">
+      <c r="D6" s="85" t="n">
         <f aca="false">Portfolio!D5</f>
         <v>12597.12</v>
       </c>
-      <c r="E6" s="86" t="n">
+      <c r="E6" s="85" t="n">
         <f aca="false">Portfolio!E5</f>
         <v>62985.6</v>
       </c>
-      <c r="F6" s="86" t="n">
+      <c r="F6" s="85" t="n">
         <f aca="false">Portfolio!F5</f>
         <v>154020.096</v>
       </c>
-      <c r="G6" s="86" t="n">
+      <c r="G6" s="85" t="n">
         <f aca="false">Portfolio!G5</f>
         <v>629856</v>
       </c>
-      <c r="H6" s="86" t="n">
+      <c r="H6" s="85" t="n">
         <f aca="false">Portfolio!I5</f>
         <v>6298863.686</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="85" t="n">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="47" t="n">
         <f aca="false">Portfolio!A6</f>
         <v>59</v>
       </c>
-      <c r="B7" s="86" t="n">
+      <c r="B7" s="85" t="n">
         <f aca="false">Portfolio!B6</f>
         <v>3948199.6896</v>
       </c>
-      <c r="C7" s="86" t="n">
+      <c r="C7" s="85" t="n">
         <f aca="false">Portfolio!C6</f>
         <v>1020366.72</v>
       </c>
-      <c r="D7" s="86" t="n">
+      <c r="D7" s="85" t="n">
         <f aca="false">Portfolio!D6</f>
         <v>13604.8896</v>
       </c>
-      <c r="E7" s="86" t="n">
+      <c r="E7" s="85" t="n">
         <f aca="false">Portfolio!E6</f>
         <v>68024.448</v>
       </c>
-      <c r="F7" s="86" t="n">
+      <c r="F7" s="85" t="n">
         <f aca="false">Portfolio!F6</f>
         <v>174981.70368</v>
       </c>
-      <c r="G7" s="86" t="n">
+      <c r="G7" s="85" t="n">
         <f aca="false">Portfolio!G6</f>
         <v>680244.48</v>
       </c>
-      <c r="H7" s="86" t="n">
+      <c r="H7" s="85" t="n">
         <f aca="false">Portfolio!I6</f>
         <v>6818354.83088</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="85" t="n">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="47" t="n">
         <f aca="false">Portfolio!A7</f>
         <v>60</v>
       </c>
-      <c r="B8" s="86" t="n">
+      <c r="B8" s="85" t="n">
         <f aca="false">Portfolio!B7</f>
         <v>4301574.414768</v>
       </c>
-      <c r="C8" s="86" t="n">
+      <c r="C8" s="85" t="n">
         <f aca="false">Portfolio!C7</f>
         <v>1101996.0576</v>
       </c>
-      <c r="D8" s="86" t="n">
+      <c r="D8" s="85" t="n">
         <f aca="false">Portfolio!D7</f>
         <v>14693.280768</v>
       </c>
-      <c r="E8" s="86" t="n">
+      <c r="E8" s="85" t="n">
         <f aca="false">Portfolio!E7</f>
         <v>73466.40384</v>
       </c>
-      <c r="F8" s="86" t="n">
+      <c r="F8" s="85" t="n">
         <f aca="false">Portfolio!F7</f>
         <v>197620.2399744</v>
       </c>
-      <c r="G8" s="86" t="n">
+      <c r="G8" s="85" t="n">
         <f aca="false">Portfolio!G7</f>
         <v>734664.0384</v>
       </c>
-      <c r="H8" s="86" t="n">
+      <c r="H8" s="85" t="n">
         <f aca="false">Portfolio!I7</f>
         <v>7378029.3158504</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="85" t="n">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="47" t="n">
         <f aca="false">Portfolio!A8</f>
         <v>61</v>
       </c>
-      <c r="B9" s="86" t="n">
+      <c r="B9" s="85" t="n">
         <f aca="false">Portfolio!B8</f>
         <v>4683219.11794944</v>
       </c>
-      <c r="C9" s="86" t="n">
+      <c r="C9" s="85" t="n">
         <f aca="false">Portfolio!C8</f>
         <v>1190155.742208</v>
       </c>
-      <c r="D9" s="86" t="n">
+      <c r="D9" s="85" t="n">
         <f aca="false">Portfolio!D8</f>
         <v>15868.74322944</v>
       </c>
-      <c r="E9" s="86" t="n">
+      <c r="E9" s="85" t="n">
         <f aca="false">Portfolio!E8</f>
         <v>79343.7161472</v>
       </c>
-      <c r="F9" s="86" t="n">
+      <c r="F9" s="85" t="n">
         <f aca="false">Portfolio!F8</f>
         <v>222069.859172352</v>
       </c>
-      <c r="G9" s="86" t="n">
+      <c r="G9" s="85" t="n">
         <f aca="false">Portfolio!G8</f>
         <v>793437.161472</v>
       </c>
-      <c r="H9" s="86" t="n">
+      <c r="H9" s="85" t="n">
         <f aca="false">Portfolio!I8</f>
         <v>7981039.89030093</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="85" t="n">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="47" t="n">
         <f aca="false">Portfolio!A9</f>
         <v>62</v>
       </c>
-      <c r="B10" s="86" t="n">
+      <c r="B10" s="85" t="n">
         <f aca="false">Portfolio!B9</f>
         <v>5095395.3973854</v>
       </c>
-      <c r="C10" s="86" t="n">
+      <c r="C10" s="85" t="n">
         <f aca="false">Portfolio!C9</f>
         <v>1285368.20158464</v>
       </c>
-      <c r="D10" s="86" t="n">
+      <c r="D10" s="85" t="n">
         <f aca="false">Portfolio!D9</f>
         <v>17138.2426877952</v>
       </c>
-      <c r="E10" s="86" t="n">
+      <c r="E10" s="85" t="n">
         <f aca="false">Portfolio!E9</f>
         <v>85691.213438976</v>
       </c>
-      <c r="F10" s="86" t="n">
+      <c r="F10" s="85" t="n">
         <f aca="false">Portfolio!F9</f>
         <v>248475.44790614</v>
       </c>
-      <c r="G10" s="86" t="n">
+      <c r="G10" s="85" t="n">
         <f aca="false">Portfolio!G9</f>
         <v>856912.13438976</v>
       </c>
-      <c r="H10" s="86" t="n">
+      <c r="H10" s="85" t="n">
         <f aca="false">Portfolio!I9</f>
         <v>8630788.73727072</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="85" t="n">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="47" t="n">
         <f aca="false">Portfolio!A10</f>
         <v>63</v>
       </c>
-      <c r="B11" s="86" t="n">
+      <c r="B11" s="85" t="n">
         <f aca="false">Portfolio!B10</f>
         <v>5540545.77917623</v>
       </c>
-      <c r="C11" s="86" t="n">
+      <c r="C11" s="85" t="n">
         <f aca="false">Portfolio!C10</f>
         <v>1388197.65771141</v>
       </c>
-      <c r="D11" s="86" t="n">
+      <c r="D11" s="85" t="n">
         <f aca="false">Portfolio!D10</f>
         <v>18509.3021028188</v>
       </c>
-      <c r="E11" s="86" t="n">
+      <c r="E11" s="85" t="n">
         <f aca="false">Portfolio!E10</f>
         <v>92546.5105140941</v>
       </c>
-      <c r="F11" s="86" t="n">
+      <c r="F11" s="85" t="n">
         <f aca="false">Portfolio!F10</f>
         <v>276993.483738632</v>
       </c>
-      <c r="G11" s="86" t="n">
+      <c r="G11" s="85" t="n">
         <f aca="false">Portfolio!G10</f>
         <v>925465.105140941</v>
       </c>
-      <c r="H11" s="86" t="n">
+      <c r="H11" s="85" t="n">
         <f aca="false">Portfolio!I10</f>
         <v>9330947.30275665</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="85" t="n">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="47" t="n">
         <f aca="false">Portfolio!A11</f>
         <v>64</v>
       </c>
-      <c r="B12" s="86" t="n">
+      <c r="B12" s="85" t="n">
         <f aca="false">Portfolio!B11</f>
         <v>6021308.19151033</v>
       </c>
-      <c r="C12" s="86" t="n">
+      <c r="C12" s="85" t="n">
         <f aca="false">Portfolio!C11</f>
         <v>1499253.47032833</v>
       </c>
-      <c r="D12" s="86" t="n">
+      <c r="D12" s="85" t="n">
         <f aca="false">Portfolio!D11</f>
         <v>19990.0462710443</v>
       </c>
-      <c r="E12" s="86" t="n">
+      <c r="E12" s="85" t="n">
         <f aca="false">Portfolio!E11</f>
         <v>99950.2313552217</v>
       </c>
-      <c r="F12" s="86" t="n">
+      <c r="F12" s="85" t="n">
         <f aca="false">Portfolio!F11</f>
         <v>307792.962437722</v>
       </c>
-      <c r="G12" s="86" t="n">
+      <c r="G12" s="85" t="n">
         <f aca="false">Portfolio!G11</f>
         <v>999502.313552217</v>
       </c>
-      <c r="H12" s="86" t="n">
+      <c r="H12" s="85" t="n">
         <f aca="false">Portfolio!I11</f>
         <v>10085477.7057241</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="85" t="n">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="47" t="n">
         <f aca="false">Portfolio!A12</f>
         <v>65</v>
       </c>
-      <c r="B13" s="86" t="n">
+      <c r="B13" s="85" t="n">
         <f aca="false">Portfolio!B12</f>
         <v>2828950</v>
       </c>
-      <c r="C13" s="86" t="n">
+      <c r="C13" s="85" t="n">
         <f aca="false">Portfolio!C12</f>
         <v>1619193.74795459</v>
       </c>
-      <c r="D13" s="86" t="n">
+      <c r="D13" s="85" t="n">
         <f aca="false">Portfolio!D12</f>
         <v>21589.2499727279</v>
       </c>
-      <c r="E13" s="86" t="n">
+      <c r="E13" s="85" t="n">
         <f aca="false">Portfolio!E12</f>
         <v>107946.249863639</v>
       </c>
-      <c r="F13" s="86" t="n">
+      <c r="F13" s="85" t="n">
         <f aca="false">Portfolio!F12</f>
         <v>330196.39943274</v>
       </c>
-      <c r="G13" s="86" t="n">
+      <c r="G13" s="85" t="n">
         <f aca="false">Portfolio!G12</f>
         <v>1079462.49863639</v>
       </c>
-      <c r="H13" s="86" t="n">
+      <c r="H13" s="85" t="n">
         <f aca="false">Portfolio!I12</f>
         <v>7176214.2581915</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="85" t="n">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="47" t="n">
         <f aca="false">Portfolio!A13</f>
         <v>66</v>
       </c>
-      <c r="B14" s="86" t="n">
+      <c r="B14" s="85" t="n">
         <f aca="false">Portfolio!B13</f>
         <v>2657900</v>
       </c>
-      <c r="C14" s="86" t="n">
+      <c r="C14" s="85" t="n">
         <f aca="false">Portfolio!C13</f>
         <v>1748729.24779096</v>
       </c>
-      <c r="D14" s="86" t="n">
+      <c r="D14" s="85" t="n">
         <f aca="false">Portfolio!D13</f>
         <v>23316.3899705461</v>
       </c>
-      <c r="E14" s="86" t="n">
+      <c r="E14" s="85" t="n">
         <f aca="false">Portfolio!E13</f>
         <v>116581.949852731</v>
       </c>
-      <c r="F14" s="86" t="n">
+      <c r="F14" s="85" t="n">
         <f aca="false">Portfolio!F13</f>
         <v>354281.111387359</v>
       </c>
-      <c r="G14" s="86" t="n">
+      <c r="G14" s="85" t="n">
         <f aca="false">Portfolio!G13</f>
         <v>1165819.49852731</v>
       </c>
-      <c r="H14" s="86" t="n">
+      <c r="H14" s="85" t="n">
         <f aca="false">Portfolio!I13</f>
         <v>7309003.73491522</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="85" t="n">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="47" t="n">
         <f aca="false">Portfolio!A14</f>
         <v>67</v>
       </c>
-      <c r="B15" s="86" t="n">
+      <c r="B15" s="85" t="n">
         <f aca="false">Portfolio!B14</f>
         <v>2527364.4</v>
       </c>
-      <c r="C15" s="86" t="n">
+      <c r="C15" s="85" t="n">
         <f aca="false">Portfolio!C14</f>
         <v>1888627.58761424</v>
       </c>
-      <c r="D15" s="86" t="n">
+      <c r="D15" s="85" t="n">
         <f aca="false">Portfolio!D14</f>
         <v>25181.7011681898</v>
       </c>
-      <c r="E15" s="86" t="n">
+      <c r="E15" s="85" t="n">
         <f aca="false">Portfolio!E14</f>
         <v>125908.505840949</v>
       </c>
-      <c r="F15" s="86" t="n">
+      <c r="F15" s="85" t="n">
         <f aca="false">Portfolio!F14</f>
         <v>380176.050298348</v>
       </c>
-      <c r="G15" s="86" t="n">
+      <c r="G15" s="85" t="n">
         <f aca="false">Portfolio!G14</f>
         <v>1259085.05840949</v>
       </c>
-      <c r="H15" s="86" t="n">
+      <c r="H15" s="85" t="n">
         <f aca="false">Portfolio!I14</f>
         <v>7504625.73989991</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="85" t="n">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="47" t="n">
         <f aca="false">Portfolio!A15</f>
         <v>68</v>
       </c>
-      <c r="B16" s="86" t="n">
+      <c r="B16" s="85" t="n">
         <f aca="false">Portfolio!B15</f>
         <v>2397841.66</v>
       </c>
-      <c r="C16" s="86" t="n">
+      <c r="C16" s="85" t="n">
         <f aca="false">Portfolio!C15</f>
         <v>2039717.79462337</v>
       </c>
-      <c r="D16" s="86" t="n">
+      <c r="D16" s="85" t="n">
         <f aca="false">Portfolio!D15</f>
         <v>27196.237261645</v>
       </c>
-      <c r="E16" s="86" t="n">
+      <c r="E16" s="85" t="n">
         <f aca="false">Portfolio!E15</f>
         <v>135981.186308225</v>
       </c>
-      <c r="F16" s="86" t="n">
+      <c r="F16" s="85" t="n">
         <f aca="false">Portfolio!F15</f>
         <v>408020.206822216</v>
       </c>
-      <c r="G16" s="86" t="n">
+      <c r="G16" s="85" t="n">
         <f aca="false">Portfolio!G15</f>
         <v>1359811.86308225</v>
       </c>
-      <c r="H16" s="86" t="n">
+      <c r="H16" s="85" t="n">
         <f aca="false">Portfolio!I15</f>
         <v>7725274.094312</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="85" t="n">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="47" t="n">
         <f aca="false">Portfolio!A16</f>
         <v>69</v>
       </c>
-      <c r="B17" s="86" t="n">
+      <c r="B17" s="85" t="n">
         <f aca="false">Portfolio!B16</f>
         <v>2269357.1015</v>
       </c>
-      <c r="C17" s="86" t="n">
+      <c r="C17" s="85" t="n">
         <f aca="false">Portfolio!C16</f>
         <v>2202895.21819324</v>
       </c>
-      <c r="D17" s="86" t="n">
+      <c r="D17" s="85" t="n">
         <f aca="false">Portfolio!D16</f>
         <v>29371.9362425766</v>
       </c>
-      <c r="E17" s="86" t="n">
+      <c r="E17" s="85" t="n">
         <f aca="false">Portfolio!E16</f>
         <v>146859.681212883</v>
       </c>
-      <c r="F17" s="86" t="n">
+      <c r="F17" s="85" t="n">
         <f aca="false">Portfolio!F16</f>
         <v>437963.399492993</v>
       </c>
-      <c r="G17" s="86" t="n">
+      <c r="G17" s="85" t="n">
         <f aca="false">Portfolio!G16</f>
         <v>1468596.81212883</v>
       </c>
-      <c r="H17" s="86" t="n">
+      <c r="H17" s="85" t="n">
         <f aca="false">Portfolio!I16</f>
         <v>7972801.02656446</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="85" t="n">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="47" t="n">
         <f aca="false">Portfolio!A17</f>
         <v>70</v>
       </c>
-      <c r="B18" s="86" t="n">
+      <c r="B18" s="85" t="n">
         <f aca="false">Portfolio!B17</f>
         <v>2141936.6790375</v>
       </c>
-      <c r="C18" s="86" t="n">
+      <c r="C18" s="85" t="n">
         <f aca="false">Portfolio!C17</f>
         <v>2379126.8356487</v>
       </c>
-      <c r="D18" s="86" t="n">
+      <c r="D18" s="85" t="n">
         <f aca="false">Portfolio!D17</f>
         <v>31721.6911419827</v>
       </c>
-      <c r="E18" s="86" t="n">
+      <c r="E18" s="85" t="n">
         <f aca="false">Portfolio!E17</f>
         <v>158608.455709914</v>
       </c>
-      <c r="F18" s="86" t="n">
+      <c r="F18" s="85" t="n">
         <f aca="false">Portfolio!F17</f>
         <v>470167.126383683</v>
       </c>
-      <c r="G18" s="86" t="n">
+      <c r="G18" s="85" t="n">
         <f aca="false">Portfolio!G17</f>
         <v>1586084.55709914</v>
       </c>
-      <c r="H18" s="86" t="n">
+      <c r="H18" s="85" t="n">
         <f aca="false">Portfolio!I17</f>
         <v>8249201.28231558</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="85" t="n">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="47" t="n">
         <f aca="false">Portfolio!A18</f>
         <v>71</v>
       </c>
-      <c r="B19" s="86" t="n">
+      <c r="B19" s="85" t="n">
         <f aca="false">Portfolio!B18</f>
         <v>2015606.99601344</v>
       </c>
-      <c r="C19" s="86" t="n">
+      <c r="C19" s="85" t="n">
         <f aca="false">Portfolio!C18</f>
         <v>2569456.9825006</v>
       </c>
-      <c r="D19" s="86" t="n">
+      <c r="D19" s="85" t="n">
         <f aca="false">Portfolio!D18</f>
         <v>34259.4264333413</v>
       </c>
-      <c r="E19" s="86" t="n">
+      <c r="E19" s="85" t="n">
         <f aca="false">Portfolio!E18</f>
         <v>171297.132166707</v>
       </c>
-      <c r="F19" s="86" t="n">
+      <c r="F19" s="85" t="n">
         <f aca="false">Portfolio!F18</f>
         <v>504805.48417219</v>
       </c>
-      <c r="G19" s="86" t="n">
+      <c r="G19" s="85" t="n">
         <f aca="false">Portfolio!G18</f>
         <v>1712971.32166707</v>
       </c>
-      <c r="H19" s="86" t="n">
+      <c r="H19" s="85" t="n">
         <f aca="false">Portfolio!I18</f>
         <v>8556623.29742627</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="85" t="n">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="47" t="n">
         <f aca="false">Portfolio!A19</f>
         <v>72</v>
       </c>
-      <c r="B20" s="86" t="n">
+      <c r="B20" s="85" t="n">
         <f aca="false">Portfolio!B19</f>
         <v>1890395.32091377</v>
       </c>
-      <c r="C20" s="86" t="n">
+      <c r="C20" s="85" t="n">
         <f aca="false">Portfolio!C19</f>
         <v>2775013.54110065</v>
       </c>
-      <c r="D20" s="86" t="n">
+      <c r="D20" s="85" t="n">
         <f aca="false">Portfolio!D19</f>
         <v>37000.1805480087</v>
       </c>
-      <c r="E20" s="86" t="n">
+      <c r="E20" s="85" t="n">
         <f aca="false">Portfolio!E19</f>
         <v>185000.902740043</v>
       </c>
-      <c r="F20" s="86" t="n">
+      <c r="F20" s="85" t="n">
         <f aca="false">Portfolio!F19</f>
         <v>542066.159967668</v>
       </c>
-      <c r="G20" s="86" t="n">
+      <c r="G20" s="85" t="n">
         <f aca="false">Portfolio!G19</f>
         <v>1850009.02740043</v>
       </c>
-      <c r="H20" s="86" t="n">
+      <c r="H20" s="85" t="n">
         <f aca="false">Portfolio!I19</f>
         <v>8897381.25509478</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="85" t="n">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="47" t="n">
         <f aca="false">Portfolio!A20</f>
         <v>73</v>
       </c>
-      <c r="B21" s="86" t="n">
+      <c r="B21" s="85" t="n">
         <f aca="false">Portfolio!B20</f>
         <v>1766329.60393662</v>
       </c>
-      <c r="C21" s="86" t="n">
+      <c r="C21" s="85" t="n">
         <f aca="false">Portfolio!C20</f>
         <v>2997014.6243887</v>
       </c>
-      <c r="D21" s="86" t="n">
+      <c r="D21" s="85" t="n">
         <f aca="false">Portfolio!D20</f>
         <v>39960.1949918494</v>
       </c>
-      <c r="E21" s="86" t="n">
+      <c r="E21" s="85" t="n">
         <f aca="false">Portfolio!E20</f>
         <v>199800.974959247</v>
       </c>
-      <c r="F21" s="86" t="n">
+      <c r="F21" s="85" t="n">
         <f aca="false">Portfolio!F20</f>
         <v>582151.50167987</v>
       </c>
-      <c r="G21" s="86" t="n">
+      <c r="G21" s="85" t="n">
         <f aca="false">Portfolio!G20</f>
         <v>1998009.74959247</v>
       </c>
-      <c r="H21" s="86" t="n">
+      <c r="H21" s="85" t="n">
         <f aca="false">Portfolio!I20</f>
         <v>9273968.09748204</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="85" t="n">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="47" t="n">
         <f aca="false">Portfolio!A21</f>
         <v>74</v>
       </c>
-      <c r="B22" s="86" t="n">
+      <c r="B22" s="85" t="n">
         <f aca="false">Portfolio!B21</f>
         <v>1643438.49403503</v>
       </c>
-      <c r="C22" s="86" t="n">
+      <c r="C22" s="85" t="n">
         <f aca="false">Portfolio!C21</f>
         <v>3236775.7943398</v>
       </c>
-      <c r="D22" s="86" t="n">
+      <c r="D22" s="85" t="n">
         <f aca="false">Portfolio!D21</f>
         <v>43157.0105911973</v>
       </c>
-      <c r="E22" s="86" t="n">
+      <c r="E22" s="85" t="n">
         <f aca="false">Portfolio!E21</f>
         <v>215785.052955986</v>
       </c>
-      <c r="F22" s="86" t="n">
+      <c r="F22" s="85" t="n">
         <f aca="false">Portfolio!F21</f>
         <v>625279.673174787</v>
       </c>
-      <c r="G22" s="86" t="n">
+      <c r="G22" s="85" t="n">
         <f aca="false">Portfolio!G21</f>
         <v>2157850.52955986</v>
       </c>
-      <c r="H22" s="86" t="n">
+      <c r="H22" s="85" t="n">
         <f aca="false">Portfolio!I21</f>
         <v>9689069.56774696</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="85" t="n">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="47" t="n">
         <f aca="false">Portfolio!A22</f>
         <v>75</v>
       </c>
-      <c r="B23" s="86" t="n">
+      <c r="B23" s="85" t="n">
         <f aca="false">Portfolio!B22</f>
         <v>1521751.35638591</v>
       </c>
-      <c r="C23" s="86" t="n">
+      <c r="C23" s="85" t="n">
         <f aca="false">Portfolio!C22</f>
         <v>3495717.85788698</v>
       </c>
-      <c r="D23" s="86" t="n">
+      <c r="D23" s="85" t="n">
         <f aca="false">Portfolio!D22</f>
         <v>46609.5714384931</v>
       </c>
-      <c r="E23" s="86" t="n">
+      <c r="E23" s="85" t="n">
         <f aca="false">Portfolio!E22</f>
         <v>233047.857192465</v>
       </c>
-      <c r="F23" s="86" t="n">
+      <c r="F23" s="85" t="n">
         <f aca="false">Portfolio!F22</f>
         <v>671685.900957324</v>
       </c>
-      <c r="G23" s="86" t="n">
+      <c r="G23" s="85" t="n">
         <f aca="false">Portfolio!G22</f>
         <v>2330478.57192465</v>
       </c>
-      <c r="H23" s="86" t="n">
+      <c r="H23" s="85" t="n">
         <f aca="false">Portfolio!I22</f>
         <v>10145579.3644652</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="85" t="n">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="47" t="n">
         <f aca="false">Portfolio!A23</f>
         <v>76</v>
       </c>
-      <c r="B24" s="86" t="n">
+      <c r="B24" s="85" t="n">
         <f aca="false">Portfolio!B23</f>
         <v>1401298.29029556</v>
       </c>
-      <c r="C24" s="86" t="n">
+      <c r="C24" s="85" t="n">
         <f aca="false">Portfolio!C23</f>
         <v>3775375.28651794</v>
       </c>
-      <c r="D24" s="86" t="n">
+      <c r="D24" s="85" t="n">
         <f aca="false">Portfolio!D23</f>
         <v>50338.3371535725</v>
       </c>
-      <c r="E24" s="86" t="n">
+      <c r="E24" s="85" t="n">
         <f aca="false">Portfolio!E23</f>
         <v>251691.685767863</v>
       </c>
-      <c r="F24" s="86" t="n">
+      <c r="F24" s="85" t="n">
         <f aca="false">Portfolio!F23</f>
         <v>721623.819658892</v>
       </c>
-      <c r="G24" s="86" t="n">
+      <c r="G24" s="85" t="n">
         <f aca="false">Portfolio!G23</f>
         <v>2516916.85767863</v>
       </c>
-      <c r="H24" s="86" t="n">
+      <c r="H24" s="85" t="n">
         <f aca="false">Portfolio!I23</f>
         <v>10646615.4969424</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="85" t="n">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="47" t="n">
         <f aca="false">Portfolio!A24</f>
         <v>77</v>
       </c>
-      <c r="B25" s="86" t="n">
+      <c r="B25" s="85" t="n">
         <f aca="false">Portfolio!B24</f>
         <v>1282110.14755295</v>
       </c>
-      <c r="C25" s="86" t="n">
+      <c r="C25" s="85" t="n">
         <f aca="false">Portfolio!C24</f>
         <v>4077405.30943937</v>
       </c>
-      <c r="D25" s="86" t="n">
+      <c r="D25" s="85" t="n">
         <f aca="false">Portfolio!D24</f>
         <v>54365.4041258583</v>
       </c>
-      <c r="E25" s="86" t="n">
+      <c r="E25" s="85" t="n">
         <f aca="false">Portfolio!E24</f>
         <v>271827.020629292</v>
       </c>
-      <c r="F25" s="86" t="n">
+      <c r="F25" s="85" t="n">
         <f aca="false">Portfolio!F24</f>
         <v>775366.924187834</v>
       </c>
-      <c r="G25" s="86" t="n">
+      <c r="G25" s="85" t="n">
         <f aca="false">Portfolio!G24</f>
         <v>2718270.20629292</v>
       </c>
-      <c r="H25" s="86" t="n">
+      <c r="H25" s="85" t="n">
         <f aca="false">Portfolio!I24</f>
         <v>11195537.9369923</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="85" t="n">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="47" t="n">
         <f aca="false">Portfolio!A25</f>
         <v>78</v>
       </c>
-      <c r="B26" s="86" t="n">
+      <c r="B26" s="85" t="n">
         <f aca="false">Portfolio!B25</f>
         <v>1164218.55124177</v>
       </c>
-      <c r="C26" s="86" t="n">
+      <c r="C26" s="85" t="n">
         <f aca="false">Portfolio!C25</f>
         <v>4403597.73419453</v>
       </c>
-      <c r="D26" s="86" t="n">
+      <c r="D26" s="85" t="n">
         <f aca="false">Portfolio!D25</f>
         <v>58714.636455927</v>
       </c>
-      <c r="E26" s="86" t="n">
+      <c r="E26" s="85" t="n">
         <f aca="false">Portfolio!E25</f>
         <v>293573.182279635</v>
       </c>
-      <c r="F26" s="86" t="n">
+      <c r="F26" s="85" t="n">
         <f aca="false">Portfolio!F25</f>
         <v>833210.137026903</v>
       </c>
-      <c r="G26" s="86" t="n">
+      <c r="G26" s="85" t="n">
         <f aca="false">Portfolio!G25</f>
         <v>2935731.82279635</v>
       </c>
-      <c r="H26" s="86" t="n">
+      <c r="H26" s="85" t="n">
         <f aca="false">Portfolio!I25</f>
         <v>11795967.6703736</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="85" t="n">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="47" t="n">
         <f aca="false">Portfolio!A26</f>
         <v>79</v>
       </c>
-      <c r="B27" s="86" t="n">
+      <c r="B27" s="85" t="n">
         <f aca="false">Portfolio!B26</f>
         <v>1047655.91502281</v>
       </c>
-      <c r="C27" s="86" t="n">
+      <c r="C27" s="85" t="n">
         <f aca="false">Portfolio!C26</f>
         <v>4755885.55293009</v>
       </c>
-      <c r="D27" s="86" t="n">
+      <c r="D27" s="85" t="n">
         <f aca="false">Portfolio!D26</f>
         <v>63411.8073724012</v>
       </c>
-      <c r="E27" s="86" t="n">
+      <c r="E27" s="85" t="n">
         <f aca="false">Portfolio!E26</f>
         <v>317059.036862006</v>
       </c>
-      <c r="F27" s="86" t="n">
+      <c r="F27" s="85" t="n">
         <f aca="false">Portfolio!F26</f>
         <v>895471.4998383</v>
       </c>
-      <c r="G27" s="86" t="n">
+      <c r="G27" s="85" t="n">
         <f aca="false">Portfolio!G26</f>
         <v>3170590.36862006</v>
       </c>
-      <c r="H27" s="86" t="n">
+      <c r="H27" s="85" t="n">
         <f aca="false">Portfolio!I26</f>
         <v>12451807.2593111</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="85" t="n">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="47" t="n">
         <f aca="false">Portfolio!A27</f>
         <v>80</v>
       </c>
-      <c r="B28" s="86" t="n">
+      <c r="B28" s="85" t="n">
         <f aca="false">Portfolio!B27</f>
         <v>932455.462898383</v>
       </c>
-      <c r="C28" s="86" t="n">
+      <c r="C28" s="85" t="n">
         <f aca="false">Portfolio!C27</f>
         <v>5136356.39716449</v>
       </c>
-      <c r="D28" s="86" t="n">
+      <c r="D28" s="85" t="n">
         <f aca="false">Portfolio!D27</f>
         <v>68484.7519621933</v>
       </c>
-      <c r="E28" s="86" t="n">
+      <c r="E28" s="85" t="n">
         <f aca="false">Portfolio!E27</f>
         <v>342423.759810966</v>
       </c>
-      <c r="F28" s="86" t="n">
+      <c r="F28" s="85" t="n">
         <f aca="false">Portfolio!F27</f>
         <v>962493.999267071</v>
       </c>
-      <c r="G28" s="86" t="n">
+      <c r="G28" s="85" t="n">
         <f aca="false">Portfolio!G27</f>
         <v>3424237.59810966</v>
       </c>
-      <c r="H28" s="86" t="n">
+      <c r="H28" s="85" t="n">
         <f aca="false">Portfolio!I27</f>
         <v>13167263.0364182</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="85" t="n">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="47" t="n">
         <f aca="false">Portfolio!A28</f>
         <v>81</v>
       </c>
-      <c r="B29" s="86" t="n">
+      <c r="B29" s="85" t="n">
         <f aca="false">Portfolio!B28</f>
         <v>818651.249470843</v>
       </c>
-      <c r="C29" s="86" t="n">
+      <c r="C29" s="85" t="n">
         <f aca="false">Portfolio!C28</f>
         <v>5547264.90893765</v>
       </c>
-      <c r="D29" s="86" t="n">
+      <c r="D29" s="85" t="n">
         <f aca="false">Portfolio!D28</f>
         <v>73963.5321191687</v>
       </c>
-      <c r="E29" s="86" t="n">
+      <c r="E29" s="85" t="n">
         <f aca="false">Portfolio!E28</f>
         <v>369817.660595844</v>
       </c>
-      <c r="F29" s="86" t="n">
+      <c r="F29" s="85" t="n">
         <f aca="false">Portfolio!F28</f>
         <v>1034647.53762223</v>
       </c>
-      <c r="G29" s="86" t="n">
+      <c r="G29" s="85" t="n">
         <f aca="false">Portfolio!G28</f>
         <v>3698176.60595844</v>
       </c>
-      <c r="H29" s="86" t="n">
+      <c r="H29" s="85" t="n">
         <f aca="false">Portfolio!I28</f>
         <v>13946869.0599338</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="85" t="n">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="47" t="n">
         <f aca="false">Portfolio!A29</f>
         <v>82</v>
       </c>
-      <c r="B30" s="86" t="n">
+      <c r="B30" s="85" t="n">
         <f aca="false">Portfolio!B29</f>
         <v>706278.180707614</v>
       </c>
-      <c r="C30" s="86" t="n">
+      <c r="C30" s="85" t="n">
         <f aca="false">Portfolio!C29</f>
         <v>5991046.10165267</v>
       </c>
-      <c r="D30" s="86" t="n">
+      <c r="D30" s="85" t="n">
         <f aca="false">Portfolio!D29</f>
         <v>79880.6146887023</v>
       </c>
-      <c r="E30" s="86" t="n">
+      <c r="E30" s="85" t="n">
         <f aca="false">Portfolio!E29</f>
         <v>399403.073443511</v>
       </c>
-      <c r="F30" s="86" t="n">
+      <c r="F30" s="85" t="n">
         <f aca="false">Portfolio!F29</f>
         <v>1112331.05996649</v>
       </c>
-      <c r="G30" s="86" t="n">
+      <c r="G30" s="85" t="n">
         <f aca="false">Portfolio!G29</f>
         <v>3994030.73443511</v>
       </c>
-      <c r="H30" s="86" t="n">
+      <c r="H30" s="85" t="n">
         <f aca="false">Portfolio!I29</f>
         <v>14795512.9705591</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="85" t="n">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="47" t="n">
         <f aca="false">Portfolio!A30</f>
         <v>83</v>
       </c>
-      <c r="B31" s="86" t="n">
+      <c r="B31" s="85" t="n">
         <f aca="false">Portfolio!B30</f>
         <v>595372.035225304</v>
       </c>
-      <c r="C31" s="86" t="n">
+      <c r="C31" s="85" t="n">
         <f aca="false">Portfolio!C30</f>
         <v>6470329.78978488</v>
       </c>
-      <c r="D31" s="86" t="n">
+      <c r="D31" s="85" t="n">
         <f aca="false">Portfolio!D30</f>
         <v>86271.0638637984</v>
       </c>
-      <c r="E31" s="86" t="n">
+      <c r="E31" s="85" t="n">
         <f aca="false">Portfolio!E30</f>
         <v>431355.319318992</v>
       </c>
-      <c r="F31" s="86" t="n">
+      <c r="F31" s="85" t="n">
         <f aca="false">Portfolio!F30</f>
         <v>1195974.85006501</v>
       </c>
-      <c r="G31" s="86" t="n">
+      <c r="G31" s="85" t="n">
         <f aca="false">Portfolio!G30</f>
         <v>4313553.19318992</v>
       </c>
-      <c r="H31" s="86" t="n">
+      <c r="H31" s="85" t="n">
         <f aca="false">Portfolio!I30</f>
         <v>15718463.9013678</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="85" t="n">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="47" t="n">
         <f aca="false">Portfolio!A31</f>
         <v>84</v>
       </c>
-      <c r="B32" s="86" t="n">
+      <c r="B32" s="85" t="n">
         <f aca="false">Portfolio!B31</f>
         <v>485969.486105936</v>
       </c>
-      <c r="C32" s="86" t="n">
+      <c r="C32" s="85" t="n">
         <f aca="false">Portfolio!C31</f>
         <v>6987956.17296767</v>
       </c>
-      <c r="D32" s="86" t="n">
+      <c r="D32" s="85" t="n">
         <f aca="false">Portfolio!D31</f>
         <v>93172.7489729023</v>
       </c>
-      <c r="E32" s="86" t="n">
+      <c r="E32" s="85" t="n">
         <f aca="false">Portfolio!E31</f>
         <v>465863.744864511</v>
       </c>
-      <c r="F32" s="86" t="n">
+      <c r="F32" s="85" t="n">
         <f aca="false">Portfolio!F31</f>
         <v>1286043.00863648</v>
       </c>
-      <c r="G32" s="86" t="n">
+      <c r="G32" s="85" t="n">
         <f aca="false">Portfolio!G31</f>
         <v>4658637.44864512</v>
       </c>
-      <c r="H32" s="86" t="n">
+      <c r="H32" s="85" t="n">
         <f aca="false">Portfolio!I31</f>
         <v>16721402.604359</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="85" t="n">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="47" t="n">
         <f aca="false">Portfolio!A32</f>
         <v>85</v>
       </c>
-      <c r="B33" s="86" t="n">
+      <c r="B33" s="85" t="n">
         <f aca="false">Portfolio!B32</f>
         <v>378108.123258585</v>
       </c>
-      <c r="C33" s="86" t="n">
+      <c r="C33" s="85" t="n">
         <f aca="false">Portfolio!C32</f>
         <v>7546992.66680509</v>
       </c>
-      <c r="D33" s="86" t="n">
+      <c r="D33" s="85" t="n">
         <f aca="false">Portfolio!D32</f>
         <v>100626.568890735</v>
       </c>
-      <c r="E33" s="86" t="n">
+      <c r="E33" s="85" t="n">
         <f aca="false">Portfolio!E32</f>
         <v>503132.844453672</v>
       </c>
-      <c r="F33" s="86" t="n">
+      <c r="F33" s="85" t="n">
         <f aca="false">Portfolio!F32</f>
         <v>1383036.12842198</v>
       </c>
-      <c r="G33" s="86" t="n">
+      <c r="G33" s="85" t="n">
         <f aca="false">Portfolio!G32</f>
         <v>5031328.44453672</v>
       </c>
-      <c r="H33" s="86" t="n">
+      <c r="H33" s="85" t="n">
         <f aca="false">Portfolio!I32</f>
         <v>17810453.9702706</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="84" t="s">
         <v>60</v>
       </c>
@@ -9139,973 +9172,973 @@
         <v>208</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="85" t="n">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="47" t="n">
         <f aca="false">'Withdrawal Plan'!A3</f>
         <v>65</v>
       </c>
-      <c r="B36" s="86" t="n">
+      <c r="B36" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!H3</f>
         <v>0</v>
       </c>
-      <c r="C36" s="86" t="n">
+      <c r="C36" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!I3</f>
         <v>0</v>
       </c>
-      <c r="D36" s="86" t="n">
+      <c r="D36" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!J3</f>
         <v>171050</v>
       </c>
-      <c r="E36" s="86" t="n">
+      <c r="E36" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!K3</f>
         <v>0</v>
       </c>
-      <c r="F36" s="86" t="n">
+      <c r="F36" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!L3</f>
         <v>0</v>
       </c>
-      <c r="G36" s="86" t="n">
+      <c r="G36" s="85" t="n">
         <f aca="false">B36+C36+D36+E36+F36</f>
         <v>171050</v>
       </c>
-      <c r="H36" s="86" t="n">
+      <c r="H36" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!G3</f>
         <v>148320</v>
       </c>
-      <c r="I36" s="86" t="n">
+      <c r="I36" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!N3</f>
         <v>27737</v>
       </c>
-      <c r="J36" s="86" t="n">
+      <c r="J36" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!O3</f>
         <v>10895.885</v>
       </c>
-      <c r="K36" s="86" t="n">
+      <c r="K36" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!P3</f>
         <v>-15902.885</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="85" t="n">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="47" t="n">
         <f aca="false">'Withdrawal Plan'!A4</f>
         <v>66</v>
       </c>
-      <c r="B37" s="86" t="n">
+      <c r="B37" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!H4</f>
         <v>0</v>
       </c>
-      <c r="C37" s="86" t="n">
+      <c r="C37" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!I4</f>
         <v>0</v>
       </c>
-      <c r="D37" s="86" t="n">
+      <c r="D37" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!J4</f>
         <v>171050</v>
       </c>
-      <c r="E37" s="86" t="n">
+      <c r="E37" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!K4</f>
         <v>0</v>
       </c>
-      <c r="F37" s="86" t="n">
+      <c r="F37" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!L4</f>
         <v>0</v>
       </c>
-      <c r="G37" s="86" t="n">
+      <c r="G37" s="85" t="n">
         <f aca="false">B37+C37+D37+E37+F37</f>
         <v>171050</v>
       </c>
-      <c r="H37" s="86" t="n">
+      <c r="H37" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!G4</f>
         <v>150951</v>
       </c>
-      <c r="I37" s="86" t="n">
+      <c r="I37" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!N4</f>
         <v>27737</v>
       </c>
-      <c r="J37" s="86" t="n">
+      <c r="J37" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!O4</f>
         <v>10895.885</v>
       </c>
-      <c r="K37" s="86" t="n">
+      <c r="K37" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!P4</f>
         <v>-18533.885</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="85" t="n">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="47" t="n">
         <f aca="false">'Withdrawal Plan'!A5</f>
         <v>67</v>
       </c>
-      <c r="B38" s="86" t="n">
+      <c r="B38" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!H5</f>
         <v>47664</v>
       </c>
-      <c r="C38" s="86" t="n">
+      <c r="C38" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!I5</f>
         <v>0</v>
       </c>
-      <c r="D38" s="86" t="n">
+      <c r="D38" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!J5</f>
         <v>130535.6</v>
       </c>
-      <c r="E38" s="86" t="n">
+      <c r="E38" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!K5</f>
         <v>0</v>
       </c>
-      <c r="F38" s="86" t="n">
+      <c r="F38" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!L5</f>
         <v>0</v>
       </c>
-      <c r="G38" s="86" t="n">
+      <c r="G38" s="85" t="n">
         <f aca="false">B38+C38+D38+E38+F38</f>
         <v>178199.6</v>
       </c>
-      <c r="H38" s="86" t="n">
+      <c r="H38" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!G5</f>
         <v>153663.15</v>
       </c>
-      <c r="I38" s="86" t="n">
+      <c r="I38" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!N5</f>
         <v>27737</v>
       </c>
-      <c r="J38" s="86" t="n">
+      <c r="J38" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!O5</f>
         <v>8315.11772</v>
       </c>
-      <c r="K38" s="86" t="n">
+      <c r="K38" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!P5</f>
         <v>-11515.66772</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="85" t="n">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="47" t="n">
         <f aca="false">'Withdrawal Plan'!A6</f>
         <v>68</v>
       </c>
-      <c r="B39" s="86" t="n">
+      <c r="B39" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!H6</f>
         <v>48855.6</v>
       </c>
-      <c r="C39" s="86" t="n">
+      <c r="C39" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!I6</f>
         <v>0</v>
       </c>
-      <c r="D39" s="86" t="n">
+      <c r="D39" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!J6</f>
         <v>129522.74</v>
       </c>
-      <c r="E39" s="86" t="n">
+      <c r="E39" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!K6</f>
         <v>0</v>
       </c>
-      <c r="F39" s="86" t="n">
+      <c r="F39" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!L6</f>
         <v>0</v>
       </c>
-      <c r="G39" s="86" t="n">
+      <c r="G39" s="85" t="n">
         <f aca="false">B39+C39+D39+E39+F39</f>
         <v>178378.34</v>
       </c>
-      <c r="H39" s="86" t="n">
+      <c r="H39" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!G6</f>
         <v>156458.9955</v>
       </c>
-      <c r="I39" s="86" t="n">
+      <c r="I39" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!N6</f>
         <v>27737</v>
       </c>
-      <c r="J39" s="86" t="n">
+      <c r="J39" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!O6</f>
         <v>8250.598538</v>
       </c>
-      <c r="K39" s="86" t="n">
+      <c r="K39" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!P6</f>
         <v>-14068.254038</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="85" t="n">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="47" t="n">
         <f aca="false">'Withdrawal Plan'!A7</f>
         <v>69</v>
       </c>
-      <c r="B40" s="86" t="n">
+      <c r="B40" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!H7</f>
         <v>50076.99</v>
       </c>
-      <c r="C40" s="86" t="n">
+      <c r="C40" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!I7</f>
         <v>0</v>
       </c>
-      <c r="D40" s="86" t="n">
+      <c r="D40" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!J7</f>
         <v>128484.5585</v>
       </c>
-      <c r="E40" s="86" t="n">
+      <c r="E40" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!K7</f>
         <v>0</v>
       </c>
-      <c r="F40" s="86" t="n">
+      <c r="F40" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!L7</f>
         <v>0</v>
       </c>
-      <c r="G40" s="86" t="n">
+      <c r="G40" s="85" t="n">
         <f aca="false">B40+C40+D40+E40+F40</f>
         <v>178561.5485</v>
       </c>
-      <c r="H40" s="86" t="n">
+      <c r="H40" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!G7</f>
         <v>159341.163915</v>
       </c>
-      <c r="I40" s="86" t="n">
+      <c r="I40" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!N7</f>
         <v>27737</v>
       </c>
-      <c r="J40" s="86" t="n">
+      <c r="J40" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!O7</f>
         <v>8184.46637645</v>
       </c>
-      <c r="K40" s="86" t="n">
+      <c r="K40" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!P7</f>
         <v>-16701.08179145</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="85" t="n">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="47" t="n">
         <f aca="false">'Withdrawal Plan'!A8</f>
         <v>70</v>
       </c>
-      <c r="B41" s="86" t="n">
+      <c r="B41" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!H8</f>
         <v>51328.91475</v>
       </c>
-      <c r="C41" s="86" t="n">
+      <c r="C41" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!I8</f>
         <v>23832</v>
       </c>
-      <c r="D41" s="86" t="n">
+      <c r="D41" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!J8</f>
         <v>127420.4224625</v>
       </c>
-      <c r="E41" s="86" t="n">
+      <c r="E41" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!K8</f>
         <v>0</v>
       </c>
-      <c r="F41" s="86" t="n">
+      <c r="F41" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!L8</f>
         <v>0</v>
       </c>
-      <c r="G41" s="86" t="n">
+      <c r="G41" s="85" t="n">
         <f aca="false">B41+C41+D41+E41+F41</f>
         <v>202581.3372125</v>
       </c>
-      <c r="H41" s="86" t="n">
+      <c r="H41" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!G8</f>
         <v>152712.36730995</v>
       </c>
-      <c r="I41" s="86" t="n">
+      <c r="I41" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!N8</f>
         <v>27737</v>
       </c>
-      <c r="J41" s="86" t="n">
+      <c r="J41" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!O8</f>
         <v>8116.68091086125</v>
       </c>
-      <c r="K41" s="86" t="n">
+      <c r="K41" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!P8</f>
         <v>14015.2889916887</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="85" t="n">
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="47" t="n">
         <f aca="false">'Withdrawal Plan'!A9</f>
         <v>71</v>
       </c>
-      <c r="B42" s="86" t="n">
+      <c r="B42" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!H9</f>
         <v>52612.13761875</v>
       </c>
-      <c r="C42" s="86" t="n">
+      <c r="C42" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!I9</f>
         <v>24427.8</v>
       </c>
-      <c r="D42" s="86" t="n">
+      <c r="D42" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!J9</f>
         <v>126329.683024063</v>
       </c>
-      <c r="E42" s="86" t="n">
+      <c r="E42" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!K9</f>
         <v>0</v>
       </c>
-      <c r="F42" s="86" t="n">
+      <c r="F42" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!L9</f>
         <v>0</v>
       </c>
-      <c r="G42" s="86" t="n">
+      <c r="G42" s="85" t="n">
         <f aca="false">B42+C42+D42+E42+F42</f>
         <v>203369.620642813</v>
       </c>
-      <c r="H42" s="86" t="n">
+      <c r="H42" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!G9</f>
         <v>155775.405230624</v>
       </c>
-      <c r="I42" s="86" t="n">
+      <c r="I42" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!N9</f>
         <v>27737</v>
       </c>
-      <c r="J42" s="86" t="n">
+      <c r="J42" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!O9</f>
         <v>8047.20080863278</v>
       </c>
-      <c r="K42" s="86" t="n">
+      <c r="K42" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!P9</f>
         <v>11810.0146035562</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="85" t="n">
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="47" t="n">
         <f aca="false">'Withdrawal Plan'!A10</f>
         <v>72</v>
       </c>
-      <c r="B43" s="86" t="n">
+      <c r="B43" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!H10</f>
         <v>53927.4410592187</v>
       </c>
-      <c r="C43" s="86" t="n">
+      <c r="C43" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!I10</f>
         <v>25038.495</v>
       </c>
-      <c r="D43" s="86" t="n">
+      <c r="D43" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!J10</f>
         <v>125211.675099664</v>
       </c>
-      <c r="E43" s="86" t="n">
+      <c r="E43" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!K10</f>
         <v>0</v>
       </c>
-      <c r="F43" s="86" t="n">
+      <c r="F43" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!L10</f>
         <v>0</v>
       </c>
-      <c r="G43" s="86" t="n">
+      <c r="G43" s="85" t="n">
         <f aca="false">B43+C43+D43+E43+F43</f>
         <v>204177.611158883</v>
       </c>
-      <c r="H43" s="86" t="n">
+      <c r="H43" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!G10</f>
         <v>158933.167633986</v>
       </c>
-      <c r="I43" s="86" t="n">
+      <c r="I43" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!N10</f>
         <v>27737</v>
       </c>
-      <c r="J43" s="86" t="n">
+      <c r="J43" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!O10</f>
         <v>7975.9837038486</v>
       </c>
-      <c r="K43" s="86" t="n">
+      <c r="K43" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!P10</f>
         <v>9531.45982104821</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="85" t="n">
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="47" t="n">
         <f aca="false">'Withdrawal Plan'!A11</f>
         <v>73</v>
       </c>
-      <c r="B44" s="86" t="n">
+      <c r="B44" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!H11</f>
         <v>55275.6270856992</v>
       </c>
-      <c r="C44" s="86" t="n">
+      <c r="C44" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!I11</f>
         <v>25664.457375</v>
       </c>
-      <c r="D44" s="86" t="n">
+      <c r="D44" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!J11</f>
         <v>124065.716977156</v>
       </c>
-      <c r="E44" s="86" t="n">
+      <c r="E44" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!K11</f>
         <v>0</v>
       </c>
-      <c r="F44" s="86" t="n">
+      <c r="F44" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!L11</f>
         <v>0</v>
       </c>
-      <c r="G44" s="86" t="n">
+      <c r="G44" s="85" t="n">
         <f aca="false">B44+C44+D44+E44+F44</f>
         <v>205005.801437855</v>
       </c>
-      <c r="H44" s="86" t="n">
+      <c r="H44" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!G11</f>
         <v>162188.637921772</v>
       </c>
-      <c r="I44" s="86" t="n">
+      <c r="I44" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!N11</f>
         <v>27737</v>
       </c>
-      <c r="J44" s="86" t="n">
+      <c r="J44" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!O11</f>
         <v>7902.98617144482</v>
       </c>
-      <c r="K44" s="86" t="n">
+      <c r="K44" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!P11</f>
         <v>7177.17734463854</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="85" t="n">
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="47" t="n">
         <f aca="false">'Withdrawal Plan'!A12</f>
         <v>74</v>
       </c>
-      <c r="B45" s="86" t="n">
+      <c r="B45" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!H12</f>
         <v>56657.5177628417</v>
       </c>
-      <c r="C45" s="86" t="n">
+      <c r="C45" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!I12</f>
         <v>26306.068809375</v>
       </c>
-      <c r="D45" s="86" t="n">
+      <c r="D45" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!J12</f>
         <v>122891.109901585</v>
       </c>
-      <c r="E45" s="86" t="n">
+      <c r="E45" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!K12</f>
         <v>0</v>
       </c>
-      <c r="F45" s="86" t="n">
+      <c r="F45" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!L12</f>
         <v>0</v>
       </c>
-      <c r="G45" s="86" t="n">
+      <c r="G45" s="85" t="n">
         <f aca="false">B45+C45+D45+E45+F45</f>
         <v>205854.696473801</v>
       </c>
-      <c r="H45" s="86" t="n">
+      <c r="H45" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!G12</f>
         <v>165544.896081129</v>
       </c>
-      <c r="I45" s="86" t="n">
+      <c r="I45" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!N12</f>
         <v>27737</v>
       </c>
-      <c r="J45" s="86" t="n">
+      <c r="J45" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!O12</f>
         <v>7828.16370073094</v>
       </c>
-      <c r="K45" s="86" t="n">
+      <c r="K45" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!P12</f>
         <v>4744.63669194142</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="85" t="n">
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="47" t="n">
         <f aca="false">'Withdrawal Plan'!A13</f>
         <v>75</v>
       </c>
-      <c r="B46" s="86" t="n">
+      <c r="B46" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!H13</f>
         <v>58073.9557069127</v>
       </c>
-      <c r="C46" s="86" t="n">
+      <c r="C46" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!I13</f>
         <v>26963.7205296094</v>
       </c>
-      <c r="D46" s="86" t="n">
+      <c r="D46" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!J13</f>
         <v>121687.137649124</v>
       </c>
-      <c r="E46" s="86" t="n">
+      <c r="E46" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!K13</f>
         <v>0</v>
       </c>
-      <c r="F46" s="86" t="n">
+      <c r="F46" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!L13</f>
         <v>0</v>
       </c>
-      <c r="G46" s="86" t="n">
+      <c r="G46" s="85" t="n">
         <f aca="false">B46+C46+D46+E46+F46</f>
         <v>206724.813885646</v>
       </c>
-      <c r="H46" s="86" t="n">
+      <c r="H46" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!G13</f>
         <v>169005.121936352</v>
       </c>
-      <c r="I46" s="86" t="n">
+      <c r="I46" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!N13</f>
         <v>27737</v>
       </c>
-      <c r="J46" s="86" t="n">
+      <c r="J46" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!O13</f>
         <v>7751.47066824921</v>
       </c>
-      <c r="K46" s="86" t="n">
+      <c r="K46" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!P13</f>
         <v>2231.22128104485</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="85" t="n">
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="47" t="n">
         <f aca="false">'Withdrawal Plan'!A14</f>
         <v>76</v>
       </c>
-      <c r="B47" s="86" t="n">
+      <c r="B47" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!H14</f>
         <v>59525.8045995855</v>
       </c>
-      <c r="C47" s="86" t="n">
+      <c r="C47" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!I14</f>
         <v>27637.8135428496</v>
       </c>
-      <c r="D47" s="86" t="n">
+      <c r="D47" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!J14</f>
         <v>120453.066090352</v>
       </c>
-      <c r="E47" s="86" t="n">
+      <c r="E47" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!K14</f>
         <v>0</v>
       </c>
-      <c r="F47" s="86" t="n">
+      <c r="F47" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!L14</f>
         <v>0</v>
       </c>
-      <c r="G47" s="86" t="n">
+      <c r="G47" s="85" t="n">
         <f aca="false">B47+C47+D47+E47+F47</f>
         <v>207616.684232787</v>
       </c>
-      <c r="H47" s="86" t="n">
+      <c r="H47" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!G14</f>
         <v>172572.598515872</v>
       </c>
-      <c r="I47" s="86" t="n">
+      <c r="I47" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!N14</f>
         <v>27737</v>
       </c>
-      <c r="J47" s="86" t="n">
+      <c r="J47" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!O14</f>
         <v>7672.86030995544</v>
       </c>
-      <c r="K47" s="86" t="n">
+      <c r="K47" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!P14</f>
         <v>-365.774593039748</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="85" t="n">
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="47" t="n">
         <f aca="false">'Withdrawal Plan'!A15</f>
         <v>77</v>
       </c>
-      <c r="B48" s="86" t="n">
+      <c r="B48" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!H15</f>
         <v>61013.9497145751</v>
       </c>
-      <c r="C48" s="86" t="n">
+      <c r="C48" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!I15</f>
         <v>28328.7588814208</v>
       </c>
-      <c r="D48" s="86" t="n">
+      <c r="D48" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!J15</f>
         <v>119188.142742611</v>
       </c>
-      <c r="E48" s="86" t="n">
+      <c r="E48" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!K15</f>
         <v>0</v>
       </c>
-      <c r="F48" s="86" t="n">
+      <c r="F48" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!L15</f>
         <v>0</v>
       </c>
-      <c r="G48" s="86" t="n">
+      <c r="G48" s="85" t="n">
         <f aca="false">B48+C48+D48+E48+F48</f>
         <v>208530.851338607</v>
       </c>
-      <c r="H48" s="86" t="n">
+      <c r="H48" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!G15</f>
         <v>176250.715538848</v>
       </c>
-      <c r="I48" s="86" t="n">
+      <c r="I48" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!N15</f>
         <v>27737</v>
       </c>
-      <c r="J48" s="86" t="n">
+      <c r="J48" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!O15</f>
         <v>7592.28469270433</v>
       </c>
-      <c r="K48" s="86" t="n">
+      <c r="K48" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!P15</f>
         <v>-3049.14889294547</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="85" t="n">
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="47" t="n">
         <f aca="false">'Withdrawal Plan'!A16</f>
         <v>78</v>
       </c>
-      <c r="B49" s="86" t="n">
+      <c r="B49" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!H16</f>
         <v>62539.2984574395</v>
       </c>
-      <c r="C49" s="86" t="n">
+      <c r="C49" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!I16</f>
         <v>29036.9778534564</v>
       </c>
-      <c r="D49" s="86" t="n">
+      <c r="D49" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!J16</f>
         <v>117891.596311176</v>
       </c>
-      <c r="E49" s="86" t="n">
+      <c r="E49" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!K16</f>
         <v>0</v>
       </c>
-      <c r="F49" s="86" t="n">
+      <c r="F49" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!L16</f>
         <v>0</v>
       </c>
-      <c r="G49" s="86" t="n">
+      <c r="G49" s="85" t="n">
         <f aca="false">B49+C49+D49+E49+F49</f>
         <v>209467.872622072</v>
       </c>
-      <c r="H49" s="86" t="n">
+      <c r="H49" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!G16</f>
         <v>144042.973025889</v>
       </c>
-      <c r="I49" s="86" t="n">
+      <c r="I49" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!N16</f>
         <v>27737</v>
       </c>
-      <c r="J49" s="86" t="n">
+      <c r="J49" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!O16</f>
         <v>7509.69468502194</v>
       </c>
-      <c r="K49" s="86" t="n">
+      <c r="K49" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!P16</f>
         <v>30178.2049111613</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="85" t="n">
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="47" t="n">
         <f aca="false">'Withdrawal Plan'!A17</f>
         <v>79</v>
       </c>
-      <c r="B50" s="86" t="n">
+      <c r="B50" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!H17</f>
         <v>64102.7809188755</v>
       </c>
-      <c r="C50" s="86" t="n">
+      <c r="C50" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!I17</f>
         <v>29762.9022997928</v>
       </c>
-      <c r="D50" s="86" t="n">
+      <c r="D50" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!J17</f>
         <v>116562.636218956</v>
       </c>
-      <c r="E50" s="86" t="n">
+      <c r="E50" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!K17</f>
         <v>0</v>
       </c>
-      <c r="F50" s="86" t="n">
+      <c r="F50" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!L17</f>
         <v>0</v>
       </c>
-      <c r="G50" s="86" t="n">
+      <c r="G50" s="85" t="n">
         <f aca="false">B50+C50+D50+E50+F50</f>
         <v>210428.319437624</v>
       </c>
-      <c r="H50" s="86" t="n">
+      <c r="H50" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!G17</f>
         <v>147952.985038585</v>
       </c>
-      <c r="I50" s="86" t="n">
+      <c r="I50" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!N17</f>
         <v>27737</v>
       </c>
-      <c r="J50" s="86" t="n">
+      <c r="J50" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!O17</f>
         <v>7425.03992714749</v>
       </c>
-      <c r="K50" s="86" t="n">
+      <c r="K50" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!P17</f>
         <v>27313.2944718917</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="85" t="n">
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="47" t="n">
         <f aca="false">'Withdrawal Plan'!A18</f>
         <v>80</v>
       </c>
-      <c r="B51" s="86" t="n">
+      <c r="B51" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!H18</f>
         <v>65705.3504418474</v>
       </c>
-      <c r="C51" s="86" t="n">
+      <c r="C51" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!I18</f>
         <v>30506.9748572876</v>
       </c>
-      <c r="D51" s="86" t="n">
+      <c r="D51" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!J18</f>
         <v>115200.45212443</v>
       </c>
-      <c r="E51" s="86" t="n">
+      <c r="E51" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!K18</f>
         <v>0</v>
       </c>
-      <c r="F51" s="86" t="n">
+      <c r="F51" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!L18</f>
         <v>0</v>
       </c>
-      <c r="G51" s="86" t="n">
+      <c r="G51" s="85" t="n">
         <f aca="false">B51+C51+D51+E51+F51</f>
         <v>211412.777423565</v>
       </c>
-      <c r="H51" s="86" t="n">
+      <c r="H51" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!G18</f>
         <v>151984.483552758</v>
       </c>
-      <c r="I51" s="86" t="n">
+      <c r="I51" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!N18</f>
         <v>27737</v>
       </c>
-      <c r="J51" s="86" t="n">
+      <c r="J51" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!O18</f>
         <v>7338.26880032618</v>
       </c>
-      <c r="K51" s="86" t="n">
+      <c r="K51" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!P18</f>
         <v>24353.025070481</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="85" t="n">
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="47" t="n">
         <f aca="false">'Withdrawal Plan'!A19</f>
         <v>81</v>
       </c>
-      <c r="B52" s="86" t="n">
+      <c r="B52" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!H19</f>
         <v>67347.9842028936</v>
       </c>
-      <c r="C52" s="86" t="n">
+      <c r="C52" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!I19</f>
         <v>31269.6492287198</v>
       </c>
-      <c r="D52" s="86" t="n">
+      <c r="D52" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!J19</f>
         <v>113804.21342754</v>
       </c>
-      <c r="E52" s="86" t="n">
+      <c r="E52" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!K19</f>
         <v>0</v>
       </c>
-      <c r="F52" s="86" t="n">
+      <c r="F52" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!L19</f>
         <v>0</v>
       </c>
-      <c r="G52" s="86" t="n">
+      <c r="G52" s="85" t="n">
         <f aca="false">B52+C52+D52+E52+F52</f>
         <v>212421.846859154</v>
       </c>
-      <c r="H52" s="86" t="n">
+      <c r="H52" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!G19</f>
         <v>156141.322470506</v>
       </c>
-      <c r="I52" s="86" t="n">
+      <c r="I52" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!N19</f>
         <v>27737</v>
       </c>
-      <c r="J52" s="86" t="n">
+      <c r="J52" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!O19</f>
         <v>7249.32839533433</v>
       </c>
-      <c r="K52" s="86" t="n">
+      <c r="K52" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!P19</f>
         <v>21294.1959933134</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="85" t="n">
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="47" t="n">
         <f aca="false">'Withdrawal Plan'!A20</f>
         <v>82</v>
       </c>
-      <c r="B53" s="86" t="n">
+      <c r="B53" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!H20</f>
         <v>69031.6838079659</v>
       </c>
-      <c r="C53" s="86" t="n">
+      <c r="C53" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!I20</f>
         <v>32051.3904594378</v>
       </c>
-      <c r="D53" s="86" t="n">
+      <c r="D53" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!J20</f>
         <v>112373.068763229</v>
       </c>
-      <c r="E53" s="86" t="n">
+      <c r="E53" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!K20</f>
         <v>0</v>
       </c>
-      <c r="F53" s="86" t="n">
+      <c r="F53" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!L20</f>
         <v>0</v>
       </c>
-      <c r="G53" s="86" t="n">
+      <c r="G53" s="85" t="n">
         <f aca="false">B53+C53+D53+E53+F53</f>
         <v>213456.143030633</v>
       </c>
-      <c r="H53" s="86" t="n">
+      <c r="H53" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!G20</f>
         <v>160427.481776345</v>
       </c>
-      <c r="I53" s="86" t="n">
+      <c r="I53" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!N20</f>
         <v>27737</v>
       </c>
-      <c r="J53" s="86" t="n">
+      <c r="J53" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!O20</f>
         <v>7158.16448021769</v>
       </c>
-      <c r="K53" s="86" t="n">
+      <c r="K53" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!P20</f>
         <v>18133.4967740695</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="85" t="n">
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="47" t="n">
         <f aca="false">'Withdrawal Plan'!A21</f>
         <v>83</v>
       </c>
-      <c r="B54" s="86" t="n">
+      <c r="B54" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!H21</f>
         <v>70757.475903165</v>
       </c>
-      <c r="C54" s="86" t="n">
+      <c r="C54" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!I21</f>
         <v>32852.6752209237</v>
       </c>
-      <c r="D54" s="86" t="n">
+      <c r="D54" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!J21</f>
         <v>110906.14548231</v>
       </c>
-      <c r="E54" s="86" t="n">
+      <c r="E54" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!K21</f>
         <v>0</v>
       </c>
-      <c r="F54" s="86" t="n">
+      <c r="F54" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!L21</f>
         <v>0</v>
       </c>
-      <c r="G54" s="86" t="n">
+      <c r="G54" s="85" t="n">
         <f aca="false">B54+C54+D54+E54+F54</f>
         <v>214516.296606398</v>
       </c>
-      <c r="H54" s="86" t="n">
+      <c r="H54" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!G21</f>
         <v>164847.071842946</v>
       </c>
-      <c r="I54" s="86" t="n">
+      <c r="I54" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!N21</f>
         <v>27737</v>
       </c>
-      <c r="J54" s="86" t="n">
+      <c r="J54" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!O21</f>
         <v>7064.72146722313</v>
       </c>
-      <c r="K54" s="86" t="n">
+      <c r="K54" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!P21</f>
         <v>14867.5032962291</v>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="85" t="n">
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="47" t="n">
         <f aca="false">'Withdrawal Plan'!A22</f>
         <v>84</v>
       </c>
-      <c r="B55" s="86" t="n">
+      <c r="B55" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!H22</f>
         <v>72526.4128007442</v>
       </c>
-      <c r="C55" s="86" t="n">
+      <c r="C55" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!I22</f>
         <v>33673.9921014468</v>
       </c>
-      <c r="D55" s="86" t="n">
+      <c r="D55" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!J22</f>
         <v>109402.549119367</v>
       </c>
-      <c r="E55" s="86" t="n">
+      <c r="E55" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!K22</f>
         <v>0</v>
       </c>
-      <c r="F55" s="86" t="n">
+      <c r="F55" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!L22</f>
         <v>0</v>
       </c>
-      <c r="G55" s="86" t="n">
+      <c r="G55" s="85" t="n">
         <f aca="false">B55+C55+D55+E55+F55</f>
         <v>215602.954021558</v>
       </c>
-      <c r="H55" s="86" t="n">
+      <c r="H55" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!G22</f>
         <v>169404.33789221</v>
       </c>
-      <c r="I55" s="86" t="n">
+      <c r="I55" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!N22</f>
         <v>27737</v>
       </c>
-      <c r="J55" s="86" t="n">
+      <c r="J55" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!O22</f>
         <v>6968.94237890371</v>
       </c>
-      <c r="K55" s="86" t="n">
+      <c r="K55" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!P22</f>
         <v>11492.6737504442</v>
       </c>
     </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="85" t="n">
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="47" t="n">
         <f aca="false">'Withdrawal Plan'!A23</f>
         <v>85</v>
       </c>
-      <c r="B56" s="86" t="n">
+      <c r="B56" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!H23</f>
         <v>74339.5731207628</v>
       </c>
-      <c r="C56" s="86" t="n">
+      <c r="C56" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!I23</f>
         <v>34515.8419039829</v>
       </c>
-      <c r="D56" s="86" t="n">
+      <c r="D56" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!J23</f>
         <v>107861.362847352</v>
       </c>
-      <c r="E56" s="86" t="n">
+      <c r="E56" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!K23</f>
         <v>0</v>
       </c>
-      <c r="F56" s="86" t="n">
+      <c r="F56" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!L23</f>
         <v>0</v>
       </c>
-      <c r="G56" s="86" t="n">
+      <c r="G56" s="85" t="n">
         <f aca="false">B56+C56+D56+E56+F56</f>
         <v>216716.777872097</v>
       </c>
-      <c r="H56" s="86" t="n">
+      <c r="H56" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!G23</f>
         <v>174103.664617651</v>
       </c>
-      <c r="I56" s="86" t="n">
+      <c r="I56" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!N23</f>
         <v>27737</v>
       </c>
-      <c r="J56" s="86" t="n">
+      <c r="J56" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!O23</f>
         <v>6870.7688133763</v>
       </c>
-      <c r="K56" s="86" t="n">
+      <c r="K56" s="85" t="n">
         <f aca="false">'Withdrawal Plan'!P23</f>
         <v>8005.34444106957</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="84" t="s">
         <v>60</v>
       </c>
@@ -10125,528 +10158,528 @@
         <v>210</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="85" t="n">
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="47" t="n">
         <f aca="false">'Stress Test'!A4</f>
         <v>65</v>
       </c>
-      <c r="B59" s="86" t="n">
+      <c r="B59" s="85" t="n">
         <f aca="false">'Stress Test'!C4</f>
         <v>9132439.10407305</v>
       </c>
-      <c r="C59" s="86" t="n">
+      <c r="C59" s="85" t="n">
         <f aca="false">'Stress Test'!E4</f>
         <v>9490350.99269125</v>
       </c>
-      <c r="D59" s="86" t="n">
+      <c r="D59" s="85" t="n">
         <f aca="false">'Stress Test'!F4</f>
         <v>9669306.93700034</v>
       </c>
-      <c r="E59" s="87" t="n">
+      <c r="E59" s="48" t="n">
         <f aca="false">IFERROR(('Withdrawal Plan'!J3+'Withdrawal Plan'!K3+'Withdrawal Plan'!L3+'Withdrawal Plan'!M3)/Portfolio!H12*100,0)</f>
         <v>2.89394044196095</v>
       </c>
-      <c r="F59" s="87" t="n">
+      <c r="F59" s="48" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="85" t="n">
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="47" t="n">
         <f aca="false">'Stress Test'!A5</f>
         <v>66</v>
       </c>
-      <c r="B60" s="86" t="n">
+      <c r="B60" s="85" t="n">
         <f aca="false">'Stress Test'!C5</f>
         <v>9324355.66823597</v>
       </c>
-      <c r="C60" s="86" t="n">
+      <c r="C60" s="85" t="n">
         <f aca="false">'Stress Test'!E5</f>
         <v>10076198.0721065</v>
       </c>
-      <c r="D60" s="86" t="n">
+      <c r="D60" s="85" t="n">
         <f aca="false">'Stress Test'!F5</f>
         <v>10462856.6307004</v>
       </c>
-      <c r="E60" s="87" t="n">
+      <c r="E60" s="48" t="n">
         <f aca="false">IFERROR(('Withdrawal Plan'!J4+'Withdrawal Plan'!K4+'Withdrawal Plan'!L4+'Withdrawal Plan'!M4)/Portfolio!H13*100,0)</f>
         <v>2.85794669385908</v>
       </c>
-      <c r="F60" s="87" t="n">
+      <c r="F60" s="48" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="85" t="n">
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="47" t="n">
         <f aca="false">'Stress Test'!A6</f>
         <v>67</v>
       </c>
-      <c r="B61" s="86" t="n">
+      <c r="B61" s="85" t="n">
         <f aca="false">'Stress Test'!C6</f>
         <v>9564346.74496541</v>
       </c>
-      <c r="C61" s="86" t="n">
+      <c r="C61" s="85" t="n">
         <f aca="false">'Stress Test'!E6</f>
         <v>10749310.7678751</v>
       </c>
-      <c r="D61" s="86" t="n">
+      <c r="D61" s="85" t="n">
         <f aca="false">'Stress Test'!F6</f>
         <v>11376159.1437704</v>
       </c>
-      <c r="E61" s="87" t="n">
+      <c r="E61" s="48" t="n">
         <f aca="false">IFERROR(('Withdrawal Plan'!J5+'Withdrawal Plan'!K5+'Withdrawal Plan'!L5+'Withdrawal Plan'!M5)/Portfolio!H14*100,0)</f>
         <v>2.14269729372886</v>
       </c>
-      <c r="F61" s="87" t="n">
+      <c r="F61" s="48" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="85" t="n">
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A62" s="47" t="n">
         <f aca="false">'Stress Test'!A7</f>
         <v>68</v>
       </c>
-      <c r="B62" s="86" t="n">
+      <c r="B62" s="85" t="n">
         <f aca="false">'Stress Test'!C7</f>
         <v>9814827.94726403</v>
       </c>
-      <c r="C62" s="86" t="n">
+      <c r="C62" s="85" t="n">
         <f aca="false">'Stress Test'!E7</f>
         <v>11477162.9618051</v>
       </c>
-      <c r="D62" s="86" t="n">
+      <c r="D62" s="85" t="n">
         <f aca="false">'Stress Test'!F7</f>
         <v>12381682.3906475</v>
       </c>
-      <c r="E62" s="87" t="n">
+      <c r="E62" s="48" t="n">
         <f aca="false">IFERROR(('Withdrawal Plan'!J6+'Withdrawal Plan'!K6+'Withdrawal Plan'!L6+'Withdrawal Plan'!M6)/Portfolio!H15*100,0)</f>
         <v>2.07413421408362</v>
       </c>
-      <c r="F62" s="87" t="n">
+      <c r="F62" s="48" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="85" t="n">
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A63" s="47" t="n">
         <f aca="false">'Stress Test'!A8</f>
         <v>69</v>
       </c>
-      <c r="B63" s="86" t="n">
+      <c r="B63" s="85" t="n">
         <f aca="false">'Stress Test'!C8</f>
         <v>10076238.0827796</v>
       </c>
-      <c r="C63" s="86" t="n">
+      <c r="C63" s="85" t="n">
         <f aca="false">'Stress Test'!E8</f>
         <v>12264153.0163745</v>
       </c>
-      <c r="D63" s="86" t="n">
+      <c r="D63" s="85" t="n">
         <f aca="false">'Stress Test'!F8</f>
         <v>13488667.6473372</v>
       </c>
-      <c r="E63" s="87" t="n">
+      <c r="E63" s="48" t="n">
         <f aca="false">IFERROR(('Withdrawal Plan'!J7+'Withdrawal Plan'!K7+'Withdrawal Plan'!L7+'Withdrawal Plan'!M7)/Portfolio!H16*100,0)</f>
         <v>2.00125246142858</v>
       </c>
-      <c r="F63" s="87" t="n">
+      <c r="F63" s="48" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="85" t="n">
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="47" t="n">
         <f aca="false">'Stress Test'!A9</f>
         <v>70</v>
       </c>
-      <c r="B64" s="86" t="n">
+      <c r="B64" s="85" t="n">
         <f aca="false">'Stress Test'!C9</f>
         <v>10349033.8385595</v>
       </c>
-      <c r="C64" s="86" t="n">
+      <c r="C64" s="85" t="n">
         <f aca="false">'Stress Test'!E9</f>
         <v>13115031.4901532</v>
       </c>
-      <c r="D64" s="86" t="n">
+      <c r="D64" s="85" t="n">
         <f aca="false">'Stress Test'!F9</f>
         <v>14707280.6445397</v>
       </c>
-      <c r="E64" s="87" t="n">
+      <c r="E64" s="48" t="n">
         <f aca="false">IFERROR(('Withdrawal Plan'!J8+'Withdrawal Plan'!K8+'Withdrawal Plan'!L8+'Withdrawal Plan'!M8)/Portfolio!H17*100,0)</f>
         <v>1.92465415799426</v>
       </c>
-      <c r="F64" s="87" t="n">
+      <c r="F64" s="48" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="85" t="n">
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="47" t="n">
         <f aca="false">'Stress Test'!A10</f>
         <v>71</v>
       </c>
-      <c r="B65" s="86" t="n">
+      <c r="B65" s="85" t="n">
         <f aca="false">'Stress Test'!C10</f>
         <v>10633690.4967557</v>
       </c>
-      <c r="C65" s="86" t="n">
+      <c r="C65" s="85" t="n">
         <f aca="false">'Stress Test'!E10</f>
         <v>14034929.3140192</v>
       </c>
-      <c r="D65" s="86" t="n">
+      <c r="D65" s="85" t="n">
         <f aca="false">'Stress Test'!F10</f>
         <v>16048704.0136474</v>
       </c>
-      <c r="E65" s="87" t="n">
+      <c r="E65" s="48" t="n">
         <f aca="false">IFERROR(('Withdrawal Plan'!J9+'Withdrawal Plan'!K9+'Withdrawal Plan'!L9+'Withdrawal Plan'!M9)/Portfolio!H18*100,0)</f>
         <v>1.84499663787272</v>
       </c>
-      <c r="F65" s="87" t="n">
+      <c r="F65" s="48" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="85" t="n">
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A66" s="47" t="n">
         <f aca="false">'Stress Test'!A11</f>
         <v>72</v>
       </c>
-      <c r="B66" s="86" t="n">
+      <c r="B66" s="85" t="n">
         <f aca="false">'Stress Test'!C11</f>
         <v>10930702.6785879</v>
       </c>
-      <c r="C66" s="86" t="n">
+      <c r="C66" s="85" t="n">
         <f aca="false">'Stress Test'!E11</f>
         <v>15029388.2211028</v>
       </c>
-      <c r="D66" s="86" t="n">
+      <c r="D66" s="85" t="n">
         <f aca="false">'Stress Test'!F11</f>
         <v>17525238.9769742</v>
       </c>
-      <c r="E66" s="87" t="n">
+      <c r="E66" s="48" t="n">
         <f aca="false">IFERROR(('Withdrawal Plan'!J10+'Withdrawal Plan'!K10+'Withdrawal Plan'!L10+'Withdrawal Plan'!M10)/Portfolio!H19*100,0)</f>
         <v>1.76297410735805</v>
       </c>
-      <c r="F66" s="87" t="n">
+      <c r="F66" s="48" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="85" t="n">
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="47" t="n">
         <f aca="false">'Stress Test'!A12</f>
         <v>73</v>
       </c>
-      <c r="B67" s="86" t="n">
+      <c r="B67" s="85" t="n">
         <f aca="false">'Stress Test'!C12</f>
         <v>11240585.1176691</v>
       </c>
-      <c r="C67" s="86" t="n">
+      <c r="C67" s="85" t="n">
         <f aca="false">'Stress Test'!E12</f>
         <v>16104393.6107286</v>
       </c>
-      <c r="D67" s="86" t="n">
+      <c r="D67" s="85" t="n">
         <f aca="false">'Stress Test'!F12</f>
         <v>19150417.2066092</v>
       </c>
-      <c r="E67" s="87" t="n">
+      <c r="E67" s="48" t="n">
         <f aca="false">IFERROR(('Withdrawal Plan'!J11+'Withdrawal Plan'!K11+'Withdrawal Plan'!L11+'Withdrawal Plan'!M11)/Portfolio!H20*100,0)</f>
         <v>1.67929830174105</v>
       </c>
-      <c r="F67" s="87" t="n">
+      <c r="F67" s="48" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="85" t="n">
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="47" t="n">
         <f aca="false">'Stress Test'!A13</f>
         <v>74</v>
       </c>
-      <c r="B68" s="86" t="n">
+      <c r="B68" s="85" t="n">
         <f aca="false">'Stress Test'!C13</f>
         <v>11563873.4638348</v>
       </c>
-      <c r="C68" s="86" t="n">
+      <c r="C68" s="85" t="n">
         <f aca="false">'Stress Test'!E13</f>
         <v>17266410.0410459</v>
       </c>
-      <c r="D68" s="86" t="n">
+      <c r="D68" s="85" t="n">
         <f aca="false">'Stress Test'!F13</f>
         <v>20939123.8687291</v>
       </c>
-      <c r="E68" s="87" t="n">
+      <c r="E68" s="48" t="n">
         <f aca="false">IFERROR(('Withdrawal Plan'!J12+'Withdrawal Plan'!K12+'Withdrawal Plan'!L12+'Withdrawal Plan'!M12)/Portfolio!H21*100,0)</f>
         <v>1.59467923394917</v>
       </c>
-      <c r="F68" s="87" t="n">
+      <c r="F68" s="48" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="85" t="n">
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A69" s="47" t="n">
         <f aca="false">'Stress Test'!A14</f>
         <v>75</v>
       </c>
-      <c r="B69" s="86" t="n">
+      <c r="B69" s="85" t="n">
         <f aca="false">'Stress Test'!C14</f>
         <v>11901125.1186676</v>
       </c>
-      <c r="C69" s="86" t="n">
+      <c r="C69" s="85" t="n">
         <f aca="false">'Stress Test'!E14</f>
         <v>18522419.560609</v>
       </c>
-      <c r="D69" s="86" t="n">
+      <c r="D69" s="85" t="n">
         <f aca="false">'Stress Test'!F14</f>
         <v>22907732.9718814</v>
       </c>
-      <c r="E69" s="87" t="n">
+      <c r="E69" s="48" t="n">
         <f aca="false">IFERROR(('Withdrawal Plan'!J13+'Withdrawal Plan'!K13+'Withdrawal Plan'!L13+'Withdrawal Plan'!M13)/Portfolio!H22*100,0)</f>
         <v>1.50980706631961</v>
       </c>
-      <c r="F69" s="87" t="n">
+      <c r="F69" s="48" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="85" t="n">
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A70" s="47" t="n">
         <f aca="false">'Stress Test'!A15</f>
         <v>76</v>
       </c>
-      <c r="B70" s="86" t="n">
+      <c r="B70" s="85" t="n">
         <f aca="false">'Stress Test'!C15</f>
         <v>12252920.1039489</v>
       </c>
-      <c r="C70" s="86" t="n">
+      <c r="C70" s="85" t="n">
         <f aca="false">'Stress Test'!E15</f>
         <v>19879963.1059923</v>
       </c>
-      <c r="D70" s="86" t="n">
+      <c r="D70" s="85" t="n">
         <f aca="false">'Stress Test'!F15</f>
         <v>25074256.2496042</v>
       </c>
-      <c r="E70" s="87" t="n">
+      <c r="E70" s="48" t="n">
         <f aca="false">IFERROR(('Withdrawal Plan'!J14+'Withdrawal Plan'!K14+'Withdrawal Plan'!L14+'Withdrawal Plan'!M14)/Portfolio!H23*100,0)</f>
         <v>1.4253359836682</v>
       </c>
-      <c r="F70" s="87" t="n">
+      <c r="F70" s="48" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="85" t="n">
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A71" s="47" t="n">
         <f aca="false">'Stress Test'!A16</f>
         <v>77</v>
       </c>
-      <c r="B71" s="86" t="n">
+      <c r="B71" s="85" t="n">
         <f aca="false">'Stress Test'!C16</f>
         <v>12619861.9643205</v>
       </c>
-      <c r="C71" s="86" t="n">
+      <c r="C71" s="85" t="n">
         <f aca="false">'Stress Test'!E16</f>
         <v>21347185.2106853</v>
       </c>
-      <c r="D71" s="86" t="n">
+      <c r="D71" s="85" t="n">
         <f aca="false">'Stress Test'!F16</f>
         <v>27458506.9307783</v>
       </c>
-      <c r="E71" s="87" t="n">
+      <c r="E71" s="48" t="n">
         <f aca="false">IFERROR(('Withdrawal Plan'!J15+'Withdrawal Plan'!K15+'Withdrawal Plan'!L15+'Withdrawal Plan'!M15)/Portfolio!H24*100,0)</f>
         <v>1.34187072849199</v>
       </c>
-      <c r="F71" s="87" t="n">
+      <c r="F71" s="48" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="85" t="n">
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A72" s="47" t="n">
         <f aca="false">'Stress Test'!A17</f>
         <v>78</v>
       </c>
-      <c r="B72" s="86" t="n">
+      <c r="B72" s="85" t="n">
         <f aca="false">'Stress Test'!C17</f>
         <v>13002578.7054862</v>
       </c>
-      <c r="C72" s="86" t="n">
+      <c r="C72" s="85" t="n">
         <f aca="false">'Stress Test'!E17</f>
         <v>22932882.290133</v>
       </c>
-      <c r="D72" s="86" t="n">
+      <c r="D72" s="85" t="n">
         <f aca="false">'Stress Test'!F17</f>
         <v>30082279.8864489</v>
       </c>
-      <c r="E72" s="87" t="n">
+      <c r="E72" s="48" t="n">
         <f aca="false">IFERROR(('Withdrawal Plan'!J16+'Withdrawal Plan'!K16+'Withdrawal Plan'!L16+'Withdrawal Plan'!M16)/Portfolio!H25*100,0)</f>
         <v>1.25995620828742</v>
       </c>
-      <c r="F72" s="87" t="n">
+      <c r="F72" s="48" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="85" t="n">
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A73" s="47" t="n">
         <f aca="false">'Stress Test'!A18</f>
         <v>79</v>
       </c>
-      <c r="B73" s="86" t="n">
+      <c r="B73" s="85" t="n">
         <f aca="false">'Stress Test'!C18</f>
         <v>13401723.7693359</v>
       </c>
-      <c r="C73" s="86" t="n">
+      <c r="C73" s="85" t="n">
         <f aca="false">'Stress Test'!E18</f>
         <v>24646554.7889739</v>
       </c>
-      <c r="D73" s="86" t="n">
+      <c r="D73" s="85" t="n">
         <f aca="false">'Stress Test'!F18</f>
         <v>32969549.7907241</v>
       </c>
-      <c r="E73" s="87" t="n">
+      <c r="E73" s="48" t="n">
         <f aca="false">IFERROR(('Withdrawal Plan'!J17+'Withdrawal Plan'!K17+'Withdrawal Plan'!L17+'Withdrawal Plan'!M17)/Portfolio!H26*100,0)</f>
         <v>1.18007033156995</v>
       </c>
-      <c r="F73" s="87" t="n">
+      <c r="F73" s="48" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="85" t="n">
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A74" s="47" t="n">
         <f aca="false">'Stress Test'!A19</f>
         <v>80</v>
       </c>
-      <c r="B74" s="86" t="n">
+      <c r="B74" s="85" t="n">
         <f aca="false">'Stress Test'!C19</f>
         <v>13817977.0474267</v>
       </c>
-      <c r="C74" s="86" t="n">
+      <c r="C74" s="85" t="n">
         <f aca="false">'Stress Test'!E19</f>
         <v>26498463.4994091</v>
       </c>
-      <c r="D74" s="86" t="n">
+      <c r="D74" s="85" t="n">
         <f aca="false">'Stress Test'!F19</f>
         <v>36146689.0971138</v>
       </c>
-      <c r="E74" s="87" t="n">
+      <c r="E74" s="48" t="n">
         <f aca="false">IFERROR(('Withdrawal Plan'!J18+'Withdrawal Plan'!K18+'Withdrawal Plan'!L18+'Withdrawal Plan'!M18)/Portfolio!H27*100,0)</f>
         <v>1.10261999981401</v>
       </c>
-      <c r="F74" s="87" t="n">
+      <c r="F74" s="48" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="85" t="n">
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A75" s="47" t="n">
         <f aca="false">'Stress Test'!A20</f>
         <v>81</v>
       </c>
-      <c r="B75" s="86" t="n">
+      <c r="B75" s="85" t="n">
         <f aca="false">'Stress Test'!C20</f>
         <v>14252045.93431</v>
       </c>
-      <c r="C75" s="86" t="n">
+      <c r="C75" s="85" t="n">
         <f aca="false">'Stress Test'!E20</f>
         <v>28499690.3843481</v>
       </c>
-      <c r="D75" s="86" t="n">
+      <c r="D75" s="85" t="n">
         <f aca="false">'Stress Test'!F20</f>
         <v>39642707.8118115</v>
       </c>
-      <c r="E75" s="87" t="n">
+      <c r="E75" s="48" t="n">
         <f aca="false">IFERROR(('Withdrawal Plan'!J19+'Withdrawal Plan'!K19+'Withdrawal Plan'!L19+'Withdrawal Plan'!M19)/Portfolio!H28*100,0)</f>
         <v>1.02793999619742</v>
       </c>
-      <c r="F75" s="87" t="n">
+      <c r="F75" s="48" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="85" t="n">
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A76" s="47" t="n">
         <f aca="false">'Stress Test'!A21</f>
         <v>82</v>
       </c>
-      <c r="B76" s="86" t="n">
+      <c r="B76" s="85" t="n">
         <f aca="false">'Stress Test'!C21</f>
         <v>14704666.4222536</v>
       </c>
-      <c r="C76" s="86" t="n">
+      <c r="C76" s="85" t="n">
         <f aca="false">'Stress Test'!E21</f>
         <v>30662204.2656672</v>
       </c>
-      <c r="D76" s="86" t="n">
+      <c r="D76" s="85" t="n">
         <f aca="false">'Stress Test'!F21</f>
         <v>43489517.2435639</v>
       </c>
-      <c r="E76" s="87" t="n">
+      <c r="E76" s="48" t="n">
         <f aca="false">IFERROR(('Withdrawal Plan'!J20+'Withdrawal Plan'!K20+'Withdrawal Plan'!L20+'Withdrawal Plan'!M20)/Portfolio!H29*100,0)</f>
         <v>0.956294378941346</v>
       </c>
-      <c r="F76" s="87" t="n">
+      <c r="F76" s="48" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="85" t="n">
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A77" s="47" t="n">
         <f aca="false">'Stress Test'!A22</f>
         <v>83</v>
       </c>
-      <c r="B77" s="86" t="n">
+      <c r="B77" s="85" t="n">
         <f aca="false">'Stress Test'!C22</f>
         <v>15176604.2389627</v>
       </c>
-      <c r="C77" s="86" t="n">
+      <c r="C77" s="85" t="n">
         <f aca="false">'Stress Test'!E22</f>
         <v>32998931.7667395</v>
       </c>
-      <c r="D77" s="86" t="n">
+      <c r="D77" s="85" t="n">
         <f aca="false">'Stress Test'!F22</f>
         <v>47722220.1277392</v>
       </c>
-      <c r="E77" s="87" t="n">
+      <c r="E77" s="48" t="n">
         <f aca="false">IFERROR(('Withdrawal Plan'!J21+'Withdrawal Plan'!K21+'Withdrawal Plan'!L21+'Withdrawal Plan'!M21)/Portfolio!H30*100,0)</f>
         <v>0.887879909078267</v>
       </c>
-      <c r="F77" s="87" t="n">
+      <c r="F77" s="48" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="85" t="n">
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A78" s="47" t="n">
         <f aca="false">'Stress Test'!A23</f>
         <v>84</v>
       </c>
-      <c r="B78" s="86" t="n">
+      <c r="B78" s="85" t="n">
         <f aca="false">'Stress Test'!C23</f>
         <v>15668656.0299681</v>
       </c>
-      <c r="C78" s="86" t="n">
+      <c r="C78" s="85" t="n">
         <f aca="false">'Stress Test'!E23</f>
         <v>35523833.9295256</v>
       </c>
-      <c r="D78" s="86" t="n">
+      <c r="D78" s="85" t="n">
         <f aca="false">'Stress Test'!F23</f>
         <v>52379429.76196</v>
       </c>
-      <c r="E78" s="87" t="n">
+      <c r="E78" s="48" t="n">
         <f aca="false">IFERROR(('Withdrawal Plan'!J22+'Withdrawal Plan'!K22+'Withdrawal Plan'!L22+'Withdrawal Plan'!M22)/Portfolio!H31*100,0)</f>
         <v>0.822831014932614</v>
       </c>
-      <c r="F78" s="87" t="n">
+      <c r="F78" s="48" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="85" t="n">
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A79" s="47" t="n">
         <f aca="false">'Stress Test'!A24</f>
         <v>85</v>
       </c>
-      <c r="B79" s="86" t="n">
+      <c r="B79" s="85" t="n">
         <f aca="false">'Stress Test'!C24</f>
         <v>16181650.587414</v>
       </c>
-      <c r="C79" s="86" t="n">
+      <c r="C79" s="85" t="n">
         <f aca="false">'Stress Test'!E24</f>
         <v>38251988.9601348</v>
       </c>
-      <c r="D79" s="86" t="n">
+      <c r="D79" s="85" t="n">
         <f aca="false">'Stress Test'!F24</f>
         <v>57503621.0544032</v>
       </c>
-      <c r="E79" s="87" t="n">
+      <c r="E79" s="48" t="n">
         <f aca="false">IFERROR(('Withdrawal Plan'!J23+'Withdrawal Plan'!K23+'Withdrawal Plan'!L23+'Withdrawal Plan'!M23)/Portfolio!H32*100,0)</f>
         <v>0.761225809389379</v>
       </c>
-      <c r="F79" s="87" t="n">
+      <c r="F79" s="48" t="n">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix Excel already-retired scenario: stop adding contributions when retired
Portfolio tab:
- Row 3 (current age): Trad 401k and HSA contributions wrapped with
  IF(Inputs!B4<Inputs!B5, ..., 0) — no contributions if already retired
- Rows 4–11 (working years): IF(A{r}<Inputs!B5,...) guard on both
  Trad 401k contrib and HSA contrib columns
- Tabs titles (Portfolio, Withdrawal Plan, Roth Conversion) updated
  to pull ages dynamically from Inputs!B4/B5/B6

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/retirement_planner.xlsx
+++ b/retirement_planner.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="208">
   <si>
     <t xml:space="preserve">RETIREMENT PLANNING MODEL — INPUTS</t>
   </si>
@@ -207,9 +207,6 @@
   </si>
   <si>
     <t xml:space="preserve">Note: Mortgage balance is auto-calculated from monthly payment, years remaining &amp; rate. Common state rates: NJ 4.5%, WA 6.0%, CA 5.5%, TX 3.5%, FL 4.0%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ROTH CONVERSION PLAN  (Ages 65–85)</t>
   </si>
   <si>
     <t xml:space="preserve">Age</t>
@@ -268,9 +265,6 @@
   </si>
   <si>
     <t xml:space="preserve">Tier 5: MAGI &gt; $750,000 — $4,170/person/yr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ANNUAL WITHDRAWAL PLAN  (Ages 65–85)</t>
   </si>
   <si>
     <t xml:space="preserve">Living+Infl
@@ -504,9 +498,6 @@
   <si>
     <t xml:space="preserve">Fed Tax
 (Single) ($)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PORTFOLIO BALANCE PROJECTION  (Ages 56–85)</t>
   </si>
   <si>
     <t xml:space="preserve">Trad 401k
@@ -3284,11 +3275,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="81615781"/>
-        <c:axId val="39758053"/>
+        <c:axId val="5279268"/>
+        <c:axId val="33845831"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="81615781"/>
+        <c:axId val="5279268"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3353,7 +3344,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="39758053"/>
+        <c:crossAx val="33845831"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3361,7 +3352,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="39758053"/>
+        <c:axId val="33845831"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3435,7 +3426,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="81615781"/>
+        <c:crossAx val="5279268"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4576,11 +4567,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="9351744"/>
-        <c:axId val="64287517"/>
+        <c:axId val="71553550"/>
+        <c:axId val="39761404"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="9351744"/>
+        <c:axId val="71553550"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4645,7 +4636,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="64287517"/>
+        <c:crossAx val="39761404"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4653,7 +4644,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="64287517"/>
+        <c:axId val="39761404"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4727,7 +4718,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="9351744"/>
+        <c:crossAx val="71553550"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -5466,11 +5457,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="27381142"/>
-        <c:axId val="95898223"/>
+        <c:axId val="36840282"/>
+        <c:axId val="66208012"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="27381142"/>
+        <c:axId val="36840282"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5535,7 +5526,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="95898223"/>
+        <c:crossAx val="66208012"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5543,7 +5534,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="95898223"/>
+        <c:axId val="66208012"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5617,7 +5608,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="27381142"/>
+        <c:crossAx val="36840282"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -6146,11 +6137,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="47487095"/>
-        <c:axId val="55775517"/>
+        <c:axId val="81062037"/>
+        <c:axId val="8298479"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="47487095"/>
+        <c:axId val="81062037"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6215,7 +6206,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="55775517"/>
+        <c:crossAx val="8298479"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -6223,7 +6214,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="55775517"/>
+        <c:axId val="8298479"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6297,7 +6288,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="47487095"/>
+        <c:crossAx val="81062037"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -7227,9 +7218,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>21</xdr:col>
-      <xdr:colOff>549720</xdr:colOff>
+      <xdr:colOff>548640</xdr:colOff>
       <xdr:row>32</xdr:row>
-      <xdr:rowOff>43200</xdr:rowOff>
+      <xdr:rowOff>42120</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -7238,7 +7229,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="8881200" y="438120"/>
-        <a:ext cx="8638200" cy="5758200"/>
+        <a:ext cx="8637120" cy="5757120"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -7257,9 +7248,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>21</xdr:col>
-      <xdr:colOff>549720</xdr:colOff>
+      <xdr:colOff>548640</xdr:colOff>
       <xdr:row>64</xdr:row>
-      <xdr:rowOff>43200</xdr:rowOff>
+      <xdr:rowOff>42120</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -7268,7 +7259,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="8881200" y="6534000"/>
-        <a:ext cx="8638200" cy="5758200"/>
+        <a:ext cx="8637120" cy="5757120"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -7287,9 +7278,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>744120</xdr:colOff>
+      <xdr:colOff>743040</xdr:colOff>
       <xdr:row>111</xdr:row>
-      <xdr:rowOff>43560</xdr:rowOff>
+      <xdr:rowOff>42480</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -7298,7 +7289,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="0" y="15487560"/>
-        <a:ext cx="8638560" cy="5758560"/>
+        <a:ext cx="8637480" cy="5757480"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -7317,9 +7308,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>21</xdr:col>
-      <xdr:colOff>550080</xdr:colOff>
+      <xdr:colOff>549000</xdr:colOff>
       <xdr:row>111</xdr:row>
-      <xdr:rowOff>43560</xdr:rowOff>
+      <xdr:rowOff>42480</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -7328,7 +7319,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="8881200" y="15487560"/>
-        <a:ext cx="8638560" cy="5758560"/>
+        <a:ext cx="8637480" cy="5757480"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -8013,96 +8004,96 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="16" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="B1" s="16"/>
     </row>
     <row r="2" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="83" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="B2" s="84" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="85" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="B3" s="86" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="87" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="B4" s="88" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="85" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="B5" s="86" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="87" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="B6" s="88" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="85" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="B7" s="86" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="87" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="B8" s="88" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="85" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="B9" s="86" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="87" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="B10" s="88" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="85" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="B11" s="86" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="87" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="B12" s="88" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
     </row>
   </sheetData>
@@ -8132,7 +8123,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="89" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="B1" s="89"/>
       <c r="C1" s="89"/>
@@ -8156,28 +8147,28 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="90" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B3" s="90" t="s">
+        <v>189</v>
+      </c>
+      <c r="C3" s="90" t="s">
+        <v>190</v>
+      </c>
+      <c r="D3" s="90" t="s">
+        <v>191</v>
+      </c>
+      <c r="E3" s="90" t="s">
         <v>192</v>
       </c>
-      <c r="C3" s="90" t="s">
+      <c r="F3" s="90" t="s">
         <v>193</v>
       </c>
-      <c r="D3" s="90" t="s">
+      <c r="G3" s="90" t="s">
         <v>194</v>
       </c>
-      <c r="E3" s="90" t="s">
+      <c r="H3" s="90" t="s">
         <v>195</v>
-      </c>
-      <c r="F3" s="90" t="s">
-        <v>196</v>
-      </c>
-      <c r="G3" s="90" t="s">
-        <v>197</v>
-      </c>
-      <c r="H3" s="90" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9202,37 +9193,37 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="90" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B35" s="90" t="s">
+        <v>196</v>
+      </c>
+      <c r="C35" s="90" t="s">
+        <v>197</v>
+      </c>
+      <c r="D35" s="90" t="s">
+        <v>198</v>
+      </c>
+      <c r="E35" s="90" t="s">
         <v>199</v>
       </c>
-      <c r="C35" s="90" t="s">
+      <c r="F35" s="90" t="s">
         <v>200</v>
       </c>
-      <c r="D35" s="90" t="s">
+      <c r="G35" s="90" t="s">
         <v>201</v>
       </c>
-      <c r="E35" s="90" t="s">
+      <c r="H35" s="90" t="s">
         <v>202</v>
       </c>
-      <c r="F35" s="90" t="s">
+      <c r="I35" s="90" t="s">
         <v>203</v>
       </c>
-      <c r="G35" s="90" t="s">
+      <c r="J35" s="90" t="s">
         <v>204</v>
       </c>
-      <c r="H35" s="90" t="s">
+      <c r="K35" s="90" t="s">
         <v>205</v>
-      </c>
-      <c r="I35" s="90" t="s">
-        <v>206</v>
-      </c>
-      <c r="J35" s="90" t="s">
-        <v>207</v>
-      </c>
-      <c r="K35" s="90" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10203,22 +10194,22 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="90" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B58" s="90" t="s">
+        <v>122</v>
+      </c>
+      <c r="C58" s="90" t="s">
         <v>124</v>
       </c>
-      <c r="C58" s="90" t="s">
-        <v>126</v>
-      </c>
       <c r="D58" s="90" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="E58" s="90" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="F58" s="90" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10782,8 +10773,9 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="16" t="s">
-        <v>59</v>
+      <c r="A1" s="16" t="str">
+        <f aca="false">IFERROR("ROTH CONVERSION PLAN  (Ages "&amp;TEXT(Inputs!B5,"0")&amp;"–"&amp;TEXT(Inputs!B6,"0"),"ROTH CONVERSION PLAN")</f>
+        <v>ROTH CONVERSION PLAN  (Ages 65–85</v>
       </c>
       <c r="B1" s="16"/>
       <c r="C1" s="16"/>
@@ -10797,34 +10789,34 @@
     </row>
     <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="B2" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="B2" s="17" t="s">
+      <c r="C2" s="17" t="s">
         <v>61</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="D2" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="D2" s="17" t="s">
+      <c r="E2" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="E2" s="17" t="s">
+      <c r="F2" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="F2" s="17" t="s">
+      <c r="G2" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="G2" s="17" t="s">
+      <c r="H2" s="17" t="s">
         <v>66</v>
       </c>
-      <c r="H2" s="17" t="s">
+      <c r="I2" s="17" t="s">
         <v>67</v>
       </c>
-      <c r="I2" s="17" t="s">
+      <c r="J2" s="17" t="s">
         <v>68</v>
-      </c>
-      <c r="J2" s="17" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11690,37 +11682,37 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="9" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="28" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="29" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="30" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="31" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="32" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="33" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -11761,8 +11753,9 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="16" t="s">
-        <v>77</v>
+      <c r="A1" s="16" t="str">
+        <f aca="false">IFERROR("ANNUAL WITHDRAWAL PLAN  (Ages "&amp;TEXT(Inputs!B5,"0")&amp;"–"&amp;TEXT(Inputs!B6,"0"),"ANNUAL WITHDRAWAL PLAN")</f>
+        <v>ANNUAL WITHDRAWAL PLAN  (Ages 65–85</v>
       </c>
       <c r="B1" s="16"/>
       <c r="C1" s="16"/>
@@ -11782,52 +11775,52 @@
     </row>
     <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="17" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B2" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="C2" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="D2" s="17" t="s">
         <v>78</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="E2" s="17" t="s">
         <v>79</v>
       </c>
-      <c r="D2" s="17" t="s">
+      <c r="F2" s="17" t="s">
         <v>80</v>
       </c>
-      <c r="E2" s="17" t="s">
+      <c r="G2" s="17" t="s">
         <v>81</v>
       </c>
-      <c r="F2" s="17" t="s">
+      <c r="H2" s="17" t="s">
         <v>82</v>
       </c>
-      <c r="G2" s="17" t="s">
+      <c r="I2" s="17" t="s">
         <v>83</v>
       </c>
-      <c r="H2" s="17" t="s">
+      <c r="J2" s="17" t="s">
         <v>84</v>
       </c>
-      <c r="I2" s="17" t="s">
+      <c r="K2" s="17" t="s">
         <v>85</v>
       </c>
-      <c r="J2" s="17" t="s">
+      <c r="L2" s="17" t="s">
         <v>86</v>
       </c>
-      <c r="K2" s="17" t="s">
+      <c r="M2" s="17" t="s">
         <v>87</v>
       </c>
-      <c r="L2" s="17" t="s">
+      <c r="N2" s="17" t="s">
+        <v>65</v>
+      </c>
+      <c r="O2" s="17" t="s">
         <v>88</v>
       </c>
-      <c r="M2" s="17" t="s">
+      <c r="P2" s="17" t="s">
         <v>89</v>
-      </c>
-      <c r="N2" s="17" t="s">
-        <v>66</v>
-      </c>
-      <c r="O2" s="17" t="s">
-        <v>90</v>
-      </c>
-      <c r="P2" s="17" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13229,7 +13222,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="40" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B1" s="40"/>
       <c r="C1" s="40"/>
@@ -13241,12 +13234,12 @@
       <c r="I1" s="40"/>
       <c r="J1" s="40"/>
       <c r="L1" s="41" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="42" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B2" s="42"/>
       <c r="C2" s="42"/>
@@ -13260,34 +13253,34 @@
     </row>
     <row r="3" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="43" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B3" s="43" t="s">
+        <v>93</v>
+      </c>
+      <c r="C3" s="43" t="s">
+        <v>94</v>
+      </c>
+      <c r="D3" s="43" t="s">
         <v>95</v>
       </c>
-      <c r="C3" s="43" t="s">
+      <c r="E3" s="43" t="s">
         <v>96</v>
       </c>
-      <c r="D3" s="43" t="s">
+      <c r="F3" s="43" t="s">
         <v>97</v>
       </c>
-      <c r="E3" s="43" t="s">
+      <c r="G3" s="43" t="s">
         <v>98</v>
       </c>
-      <c r="F3" s="43" t="s">
+      <c r="H3" s="43" t="s">
         <v>99</v>
       </c>
-      <c r="G3" s="43" t="s">
+      <c r="I3" s="43" t="s">
+        <v>88</v>
+      </c>
+      <c r="J3" s="43" t="s">
         <v>100</v>
-      </c>
-      <c r="H3" s="43" t="s">
-        <v>101</v>
-      </c>
-      <c r="I3" s="43" t="s">
-        <v>90</v>
-      </c>
-      <c r="J3" s="43" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13809,7 +13802,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="49" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B15" s="50"/>
       <c r="C15" s="51"/>
@@ -13915,7 +13908,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="40" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B1" s="40"/>
       <c r="C1" s="40"/>
@@ -13932,7 +13925,7 @@
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="42" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B2" s="42"/>
       <c r="C2" s="42"/>
@@ -13949,46 +13942,46 @@
     </row>
     <row r="3" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="43" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B3" s="43" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C3" s="43" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D3" s="43" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E3" s="43" t="s">
+        <v>104</v>
+      </c>
+      <c r="F3" s="43" t="s">
+        <v>105</v>
+      </c>
+      <c r="G3" s="43" t="s">
         <v>106</v>
       </c>
-      <c r="F3" s="43" t="s">
+      <c r="H3" s="43" t="s">
         <v>107</v>
       </c>
-      <c r="G3" s="43" t="s">
+      <c r="I3" s="43" t="s">
         <v>108</v>
       </c>
-      <c r="H3" s="43" t="s">
+      <c r="J3" s="43" t="s">
+        <v>65</v>
+      </c>
+      <c r="K3" s="43" t="s">
+        <v>66</v>
+      </c>
+      <c r="L3" s="43" t="s">
         <v>109</v>
       </c>
-      <c r="I3" s="43" t="s">
+      <c r="M3" s="43" t="s">
         <v>110</v>
       </c>
-      <c r="J3" s="43" t="s">
-        <v>66</v>
-      </c>
-      <c r="K3" s="43" t="s">
-        <v>67</v>
-      </c>
-      <c r="L3" s="43" t="s">
+      <c r="N3" s="43" t="s">
         <v>111</v>
-      </c>
-      <c r="M3" s="43" t="s">
-        <v>112</v>
-      </c>
-      <c r="N3" s="43" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15221,7 +15214,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="40" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B1" s="40"/>
       <c r="C1" s="40"/>
@@ -15234,7 +15227,7 @@
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="42" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B2" s="42"/>
       <c r="C2" s="42"/>
@@ -15247,28 +15240,28 @@
     </row>
     <row r="3" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="43" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B3" s="43" t="s">
+        <v>114</v>
+      </c>
+      <c r="C3" s="43" t="s">
+        <v>115</v>
+      </c>
+      <c r="D3" s="43" t="s">
         <v>116</v>
       </c>
-      <c r="C3" s="43" t="s">
+      <c r="E3" s="43" t="s">
         <v>117</v>
       </c>
-      <c r="D3" s="43" t="s">
+      <c r="F3" s="43" t="s">
         <v>118</v>
       </c>
-      <c r="E3" s="43" t="s">
+      <c r="G3" s="43" t="s">
         <v>119</v>
       </c>
-      <c r="F3" s="43" t="s">
+      <c r="H3" s="43" t="s">
         <v>120</v>
-      </c>
-      <c r="G3" s="43" t="s">
-        <v>121</v>
-      </c>
-      <c r="H3" s="43" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15966,19 +15959,19 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="65" t="s">
+        <v>121</v>
+      </c>
+      <c r="C26" s="66" t="s">
+        <v>122</v>
+      </c>
+      <c r="D26" s="66" t="s">
         <v>123</v>
       </c>
-      <c r="C26" s="66" t="s">
+      <c r="E26" s="66" t="s">
         <v>124</v>
       </c>
-      <c r="D26" s="66" t="s">
+      <c r="F26" s="66" t="s">
         <v>125</v>
-      </c>
-      <c r="E26" s="66" t="s">
-        <v>126</v>
-      </c>
-      <c r="F26" s="66" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16001,7 +15994,7 @@
     </row>
     <row r="28" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="42" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B28" s="42"/>
       <c r="C28" s="42"/>
@@ -16049,7 +16042,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="40" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B1" s="40"/>
       <c r="C1" s="40"/>
@@ -16065,7 +16058,7 @@
     </row>
     <row r="2" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="42" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B2" s="42"/>
       <c r="C2" s="42"/>
@@ -16081,62 +16074,62 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="68" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C4" s="69" t="n">
         <v>75</v>
       </c>
       <c r="D4" s="70" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="68" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C5" s="71" t="n">
         <v>0.2</v>
       </c>
       <c r="D5" s="70" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="43" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B6" s="43" t="s">
+        <v>133</v>
+      </c>
+      <c r="C6" s="43" t="s">
+        <v>82</v>
+      </c>
+      <c r="D6" s="43" t="s">
+        <v>83</v>
+      </c>
+      <c r="E6" s="43" t="s">
+        <v>134</v>
+      </c>
+      <c r="F6" s="43" t="s">
         <v>135</v>
       </c>
-      <c r="C6" s="43" t="s">
-        <v>84</v>
-      </c>
-      <c r="D6" s="43" t="s">
-        <v>85</v>
-      </c>
-      <c r="E6" s="43" t="s">
+      <c r="G6" s="43" t="s">
         <v>136</v>
       </c>
-      <c r="F6" s="43" t="s">
+      <c r="H6" s="43" t="s">
+        <v>81</v>
+      </c>
+      <c r="I6" s="43" t="s">
         <v>137</v>
       </c>
-      <c r="G6" s="43" t="s">
+      <c r="J6" s="43" t="s">
         <v>138</v>
       </c>
-      <c r="H6" s="43" t="s">
-        <v>83</v>
-      </c>
-      <c r="I6" s="43" t="s">
-        <v>139</v>
-      </c>
-      <c r="J6" s="43" t="s">
-        <v>140</v>
-      </c>
       <c r="K6" s="43" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="L6" s="43" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17201,8 +17194,9 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="16" t="s">
-        <v>141</v>
+      <c r="A1" s="16" t="str">
+        <f aca="false">IFERROR("PORTFOLIO BALANCE PROJECTION  (Ages "&amp;TEXT(Inputs!B4,"0")&amp;"–"&amp;TEXT(Inputs!B6,"0"),"PORTFOLIO BALANCE PROJECTION")</f>
+        <v>PORTFOLIO BALANCE PROJECTION  (Ages 56–85</v>
       </c>
       <c r="B1" s="16"/>
       <c r="C1" s="16"/>
@@ -17215,31 +17209,31 @@
     </row>
     <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="17" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B2" s="17" t="s">
+        <v>139</v>
+      </c>
+      <c r="C2" s="17" t="s">
+        <v>140</v>
+      </c>
+      <c r="D2" s="17" t="s">
+        <v>141</v>
+      </c>
+      <c r="E2" s="17" t="s">
         <v>142</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="F2" s="17" t="s">
         <v>143</v>
       </c>
-      <c r="D2" s="17" t="s">
+      <c r="G2" s="17" t="s">
         <v>144</v>
       </c>
-      <c r="E2" s="17" t="s">
+      <c r="H2" s="17" t="s">
         <v>145</v>
       </c>
-      <c r="F2" s="17" t="s">
+      <c r="I2" s="17" t="s">
         <v>146</v>
-      </c>
-      <c r="G2" s="17" t="s">
-        <v>147</v>
-      </c>
-      <c r="H2" s="17" t="s">
-        <v>148</v>
-      </c>
-      <c r="I2" s="17" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17247,7 +17241,7 @@
         <v>56</v>
       </c>
       <c r="B3" s="73" t="n">
-        <f aca="false">Inputs!B9+Inputs!B11*(1+Inputs!B12/100)</f>
+        <f aca="false">Inputs!B9+IF(Inputs!B4&lt;Inputs!B5,Inputs!B11*(1+Inputs!B12/100),0)</f>
         <v>3037518.75</v>
       </c>
       <c r="C3" s="73" t="n">
@@ -17263,7 +17257,7 @@
         <v>54000</v>
       </c>
       <c r="F3" s="73" t="n">
-        <f aca="false">(Inputs!B14+Inputs!B15)*(1+Inputs!B19)</f>
+        <f aca="false">(Inputs!B14+IF(Inputs!B4&lt;Inputs!B5,Inputs!B15,0))*(1+Inputs!B19)</f>
         <v>116640</v>
       </c>
       <c r="G3" s="73" t="n">
@@ -17284,7 +17278,7 @@
         <v>57</v>
       </c>
       <c r="B4" s="73" t="n">
-        <f aca="false">B3*(1+Inputs!B19)+Inputs!B11*(1+Inputs!B12/100)</f>
+        <f aca="false">B3*(1+Inputs!B19)+IF(A4&lt;Inputs!B5,Inputs!B11*(1+Inputs!B12/100),0)</f>
         <v>3318039</v>
       </c>
       <c r="C4" s="73" t="n">
@@ -17300,7 +17294,7 @@
         <v>58320</v>
       </c>
       <c r="F4" s="73" t="n">
-        <f aca="false">(F3+Inputs!B15)*(1+Inputs!B19)</f>
+        <f aca="false">(F3+IF(A4&lt;Inputs!B5,Inputs!B15,0))*(1+Inputs!B19)</f>
         <v>134611.2</v>
       </c>
       <c r="G4" s="73" t="n">
@@ -17321,7 +17315,7 @@
         <v>58</v>
       </c>
       <c r="B5" s="73" t="n">
-        <f aca="false">B4*(1+Inputs!B19)+Inputs!B11*(1+Inputs!B12/100)</f>
+        <f aca="false">B4*(1+Inputs!B19)+IF(A5&lt;Inputs!B5,Inputs!B11*(1+Inputs!B12/100),0)</f>
         <v>3621000.87</v>
       </c>
       <c r="C5" s="73" t="n">
@@ -17337,7 +17331,7 @@
         <v>62985.6</v>
       </c>
       <c r="F5" s="73" t="n">
-        <f aca="false">(F4+Inputs!B15)*(1+Inputs!B19)</f>
+        <f aca="false">(F4+IF(A5&lt;Inputs!B5,Inputs!B15,0))*(1+Inputs!B19)</f>
         <v>154020.096</v>
       </c>
       <c r="G5" s="73" t="n">
@@ -17358,7 +17352,7 @@
         <v>59</v>
       </c>
       <c r="B6" s="73" t="n">
-        <f aca="false">B5*(1+Inputs!B19)+Inputs!B11*(1+Inputs!B12/100)</f>
+        <f aca="false">B5*(1+Inputs!B19)+IF(A6&lt;Inputs!B5,Inputs!B11*(1+Inputs!B12/100),0)</f>
         <v>3948199.6896</v>
       </c>
       <c r="C6" s="73" t="n">
@@ -17374,7 +17368,7 @@
         <v>68024.448</v>
       </c>
       <c r="F6" s="73" t="n">
-        <f aca="false">(F5+Inputs!B15)*(1+Inputs!B19)</f>
+        <f aca="false">(F5+IF(A6&lt;Inputs!B5,Inputs!B15,0))*(1+Inputs!B19)</f>
         <v>174981.70368</v>
       </c>
       <c r="G6" s="73" t="n">
@@ -17395,7 +17389,7 @@
         <v>60</v>
       </c>
       <c r="B7" s="73" t="n">
-        <f aca="false">B6*(1+Inputs!B19)+Inputs!B11*(1+Inputs!B12/100)</f>
+        <f aca="false">B6*(1+Inputs!B19)+IF(A7&lt;Inputs!B5,Inputs!B11*(1+Inputs!B12/100),0)</f>
         <v>4301574.414768</v>
       </c>
       <c r="C7" s="73" t="n">
@@ -17411,7 +17405,7 @@
         <v>73466.40384</v>
       </c>
       <c r="F7" s="73" t="n">
-        <f aca="false">(F6+Inputs!B15)*(1+Inputs!B19)</f>
+        <f aca="false">(F6+IF(A7&lt;Inputs!B5,Inputs!B15,0))*(1+Inputs!B19)</f>
         <v>197620.2399744</v>
       </c>
       <c r="G7" s="73" t="n">
@@ -17432,7 +17426,7 @@
         <v>61</v>
       </c>
       <c r="B8" s="73" t="n">
-        <f aca="false">B7*(1+Inputs!B19)+Inputs!B11*(1+Inputs!B12/100)</f>
+        <f aca="false">B7*(1+Inputs!B19)+IF(A8&lt;Inputs!B5,Inputs!B11*(1+Inputs!B12/100),0)</f>
         <v>4683219.11794944</v>
       </c>
       <c r="C8" s="73" t="n">
@@ -17448,7 +17442,7 @@
         <v>79343.7161472</v>
       </c>
       <c r="F8" s="73" t="n">
-        <f aca="false">(F7+Inputs!B15)*(1+Inputs!B19)</f>
+        <f aca="false">(F7+IF(A8&lt;Inputs!B5,Inputs!B15,0))*(1+Inputs!B19)</f>
         <v>222069.859172352</v>
       </c>
       <c r="G8" s="73" t="n">
@@ -17469,7 +17463,7 @@
         <v>62</v>
       </c>
       <c r="B9" s="73" t="n">
-        <f aca="false">B8*(1+Inputs!B19)+Inputs!B11*(1+Inputs!B12/100)</f>
+        <f aca="false">B8*(1+Inputs!B19)+IF(A9&lt;Inputs!B5,Inputs!B11*(1+Inputs!B12/100),0)</f>
         <v>5095395.3973854</v>
       </c>
       <c r="C9" s="73" t="n">
@@ -17485,7 +17479,7 @@
         <v>85691.213438976</v>
       </c>
       <c r="F9" s="73" t="n">
-        <f aca="false">(F8+Inputs!B15)*(1+Inputs!B19)</f>
+        <f aca="false">(F8+IF(A9&lt;Inputs!B5,Inputs!B15,0))*(1+Inputs!B19)</f>
         <v>248475.44790614</v>
       </c>
       <c r="G9" s="73" t="n">
@@ -17506,7 +17500,7 @@
         <v>63</v>
       </c>
       <c r="B10" s="73" t="n">
-        <f aca="false">B9*(1+Inputs!B19)+Inputs!B11*(1+Inputs!B12/100)</f>
+        <f aca="false">B9*(1+Inputs!B19)+IF(A10&lt;Inputs!B5,Inputs!B11*(1+Inputs!B12/100),0)</f>
         <v>5540545.77917623</v>
       </c>
       <c r="C10" s="73" t="n">
@@ -17522,7 +17516,7 @@
         <v>92546.5105140941</v>
       </c>
       <c r="F10" s="73" t="n">
-        <f aca="false">(F9+Inputs!B15)*(1+Inputs!B19)</f>
+        <f aca="false">(F9+IF(A10&lt;Inputs!B5,Inputs!B15,0))*(1+Inputs!B19)</f>
         <v>276993.483738632</v>
       </c>
       <c r="G10" s="73" t="n">
@@ -17543,7 +17537,7 @@
         <v>64</v>
       </c>
       <c r="B11" s="73" t="n">
-        <f aca="false">B10*(1+Inputs!B19)+Inputs!B11*(1+Inputs!B12/100)</f>
+        <f aca="false">B10*(1+Inputs!B19)+IF(A11&lt;Inputs!B5,Inputs!B11*(1+Inputs!B12/100),0)</f>
         <v>6021308.19151033</v>
       </c>
       <c r="C11" s="73" t="n">
@@ -17559,7 +17553,7 @@
         <v>99950.2313552217</v>
       </c>
       <c r="F11" s="73" t="n">
-        <f aca="false">(F10+Inputs!B15)*(1+Inputs!B19)</f>
+        <f aca="false">(F10+IF(A11&lt;Inputs!B5,Inputs!B15,0))*(1+Inputs!B19)</f>
         <v>307792.962437722</v>
       </c>
       <c r="G11" s="73" t="n">
@@ -18354,7 +18348,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="76" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B34" s="76"/>
       <c r="C34" s="76"/>
@@ -18395,7 +18389,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="16" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="B1" s="16"/>
       <c r="C1" s="16"/>
@@ -18403,21 +18397,21 @@
     </row>
     <row r="2" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="77" t="s">
+        <v>149</v>
+      </c>
+      <c r="B2" s="77" t="s">
+        <v>150</v>
+      </c>
+      <c r="C2" s="77" t="s">
+        <v>151</v>
+      </c>
+      <c r="D2" s="77" t="s">
         <v>152</v>
-      </c>
-      <c r="B2" s="77" t="s">
-        <v>153</v>
-      </c>
-      <c r="C2" s="77" t="s">
-        <v>154</v>
-      </c>
-      <c r="D2" s="77" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="78" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="B3" s="79" t="n">
         <f aca="false">Inputs!B22</f>
@@ -18434,7 +18428,7 @@
     </row>
     <row r="4" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="78" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="B4" s="80" t="n">
         <f aca="false">Inputs!B22*12</f>
@@ -18451,7 +18445,7 @@
     </row>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="78" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="B5" s="81" t="n">
         <f aca="false">85-65</f>
@@ -18468,7 +18462,7 @@
     </row>
     <row r="6" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="78" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="B6" s="80" t="n">
         <f aca="false">Inputs!B22*12*20</f>
@@ -18485,30 +18479,30 @@
     </row>
     <row r="7" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="78" t="s">
+        <v>157</v>
+      </c>
+      <c r="B7" s="81" t="s">
+        <v>158</v>
+      </c>
+      <c r="C7" s="81" t="s">
+        <v>159</v>
+      </c>
+      <c r="D7" s="81" t="s">
         <v>160</v>
-      </c>
-      <c r="B7" s="81" t="s">
-        <v>161</v>
-      </c>
-      <c r="C7" s="81" t="s">
-        <v>162</v>
-      </c>
-      <c r="D7" s="81" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="78" t="s">
+        <v>161</v>
+      </c>
+      <c r="B8" s="82" t="s">
+        <v>162</v>
+      </c>
+      <c r="C8" s="82" t="s">
+        <v>163</v>
+      </c>
+      <c r="D8" s="82" t="s">
         <v>164</v>
-      </c>
-      <c r="B8" s="82" t="s">
-        <v>165</v>
-      </c>
-      <c r="C8" s="82" t="s">
-        <v>166</v>
-      </c>
-      <c r="D8" s="82" t="s">
-        <v>167</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sync Excel Portfolio net worth to deduct remaining mortgage balance
Column I (Net Worth) previously added home value + appreciation but
did not subtract the outstanding mortgage balance. Now uses the same
amortization formula as the web version: PMT*(1-(1+r)^-n)/r using
monthly rate and months remaining from each projected age. Also
respects the 'Pay Off at Retirement' flag (Inputs!B51). Column header
updated to 'Net Worth (Home Equity)' to match web version.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/retirement_planner.xlsx
+++ b/retirement_planner.xlsx
@@ -529,8 +529,7 @@
   </si>
   <si>
     <t xml:space="preserve">Net Worth
-+Home ($)
-(home appreciates)</t>
+(Home Equity) ($)</t>
   </si>
   <si>
     <t xml:space="preserve">Blue rows = working years (accumulation)  ·  Orange rows = RMD years (age 73+)  ·  White/cream = retirement years  ·  Net Worth includes home value appreciating at Inputs!B52 rate per year</t>
@@ -3275,11 +3274,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="48485914"/>
-        <c:axId val="89333867"/>
+        <c:axId val="96453926"/>
+        <c:axId val="42635581"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="48485914"/>
+        <c:axId val="96453926"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3344,7 +3343,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="89333867"/>
+        <c:crossAx val="42635581"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3352,7 +3351,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="89333867"/>
+        <c:axId val="42635581"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3426,7 +3425,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="48485914"/>
+        <c:crossAx val="96453926"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4567,11 +4566,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="24832143"/>
-        <c:axId val="83548538"/>
+        <c:axId val="15244717"/>
+        <c:axId val="2634638"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="24832143"/>
+        <c:axId val="15244717"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4636,7 +4635,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="83548538"/>
+        <c:crossAx val="2634638"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4644,7 +4643,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="83548538"/>
+        <c:axId val="2634638"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4718,7 +4717,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="24832143"/>
+        <c:crossAx val="15244717"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -5457,11 +5456,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="84775994"/>
-        <c:axId val="36776677"/>
+        <c:axId val="9936751"/>
+        <c:axId val="54546250"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="84775994"/>
+        <c:axId val="9936751"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5526,7 +5525,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="36776677"/>
+        <c:crossAx val="54546250"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5534,7 +5533,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="36776677"/>
+        <c:axId val="54546250"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5608,7 +5607,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="84775994"/>
+        <c:crossAx val="9936751"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -6137,11 +6136,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="68259432"/>
-        <c:axId val="83951454"/>
+        <c:axId val="63135169"/>
+        <c:axId val="46458575"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="68259432"/>
+        <c:axId val="63135169"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6206,7 +6205,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="83951454"/>
+        <c:crossAx val="46458575"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -6214,7 +6213,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="83951454"/>
+        <c:axId val="46458575"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6288,7 +6287,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="68259432"/>
+        <c:crossAx val="63135169"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -7218,9 +7217,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>21</xdr:col>
-      <xdr:colOff>548280</xdr:colOff>
+      <xdr:colOff>547920</xdr:colOff>
       <xdr:row>32</xdr:row>
-      <xdr:rowOff>41760</xdr:rowOff>
+      <xdr:rowOff>41400</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -7229,7 +7228,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="8881200" y="438120"/>
-        <a:ext cx="8636760" cy="5756760"/>
+        <a:ext cx="8636400" cy="5756400"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -7248,9 +7247,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>21</xdr:col>
-      <xdr:colOff>548280</xdr:colOff>
+      <xdr:colOff>547920</xdr:colOff>
       <xdr:row>64</xdr:row>
-      <xdr:rowOff>41760</xdr:rowOff>
+      <xdr:rowOff>41400</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -7259,7 +7258,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="8881200" y="6534000"/>
-        <a:ext cx="8636760" cy="5756760"/>
+        <a:ext cx="8636400" cy="5756400"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -7278,9 +7277,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>742680</xdr:colOff>
+      <xdr:colOff>742320</xdr:colOff>
       <xdr:row>111</xdr:row>
-      <xdr:rowOff>42120</xdr:rowOff>
+      <xdr:rowOff>41760</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -7289,7 +7288,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="0" y="15487560"/>
-        <a:ext cx="8637120" cy="5757120"/>
+        <a:ext cx="8636760" cy="5756760"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -7308,9 +7307,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>21</xdr:col>
-      <xdr:colOff>548640</xdr:colOff>
+      <xdr:colOff>548280</xdr:colOff>
       <xdr:row>111</xdr:row>
-      <xdr:rowOff>42120</xdr:rowOff>
+      <xdr:rowOff>41760</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -7319,7 +7318,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="8881200" y="15487560"/>
-        <a:ext cx="8637120" cy="5757120"/>
+        <a:ext cx="8636760" cy="5756760"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -8202,7 +8201,7 @@
       </c>
       <c r="H4" s="91" t="n">
         <f aca="false">Portfolio!I3</f>
-        <v>5368958.75</v>
+        <v>4948165.75</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8236,7 +8235,7 @@
       </c>
       <c r="H5" s="91" t="n">
         <f aca="false">Portfolio!I4</f>
-        <v>5816634.2</v>
+        <v>5404751.2</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8270,7 +8269,7 @@
       </c>
       <c r="H6" s="91" t="n">
         <f aca="false">Portfolio!I5</f>
-        <v>6298863.686</v>
+        <v>5896488.686</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8304,7 +8303,7 @@
       </c>
       <c r="H7" s="91" t="n">
         <f aca="false">Portfolio!I6</f>
-        <v>6818354.83088</v>
+        <v>6426123.83088</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8338,7 +8337,7 @@
       </c>
       <c r="H8" s="91" t="n">
         <f aca="false">Portfolio!I7</f>
-        <v>7378029.3158504</v>
+        <v>6996622.3158504</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8372,7 +8371,7 @@
       </c>
       <c r="H9" s="91" t="n">
         <f aca="false">Portfolio!I8</f>
-        <v>7981039.89030093</v>
+        <v>7611181.89030093</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8406,7 +8405,7 @@
       </c>
       <c r="H10" s="91" t="n">
         <f aca="false">Portfolio!I9</f>
-        <v>8630788.73727072</v>
+        <v>8273252.73727072</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8440,7 +8439,7 @@
       </c>
       <c r="H11" s="91" t="n">
         <f aca="false">Portfolio!I10</f>
-        <v>9330947.30275665</v>
+        <v>8986558.30275665</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8474,7 +8473,7 @@
       </c>
       <c r="H12" s="91" t="n">
         <f aca="false">Portfolio!I11</f>
-        <v>10085477.7057241</v>
+        <v>9755115.70572414</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8508,7 +8507,7 @@
       </c>
       <c r="H13" s="91" t="n">
         <f aca="false">Portfolio!I12</f>
-        <v>7176214.2581915</v>
+        <v>6860820.2581915</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8542,7 +8541,7 @@
       </c>
       <c r="H14" s="91" t="n">
         <f aca="false">Portfolio!I13</f>
-        <v>7309003.73491522</v>
+        <v>7009578.73491522</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8576,7 +8575,7 @@
       </c>
       <c r="H15" s="91" t="n">
         <f aca="false">Portfolio!I14</f>
-        <v>7504625.73989991</v>
+        <v>7222239.73989991</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8610,7 +8609,7 @@
       </c>
       <c r="H16" s="91" t="n">
         <f aca="false">Portfolio!I15</f>
-        <v>7725274.094312</v>
+        <v>7461069.094312</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8644,7 +8643,7 @@
       </c>
       <c r="H17" s="91" t="n">
         <f aca="false">Portfolio!I16</f>
-        <v>7972801.02656446</v>
+        <v>7727993.02656446</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8678,7 +8677,7 @@
       </c>
       <c r="H18" s="91" t="n">
         <f aca="false">Portfolio!I17</f>
-        <v>8249201.28231558</v>
+        <v>8025090.28231558</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8712,7 +8711,7 @@
       </c>
       <c r="H19" s="91" t="n">
         <f aca="false">Portfolio!I18</f>
-        <v>8556623.29742627</v>
+        <v>8354595.29742627</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8746,7 +8745,7 @@
       </c>
       <c r="H20" s="91" t="n">
         <f aca="false">Portfolio!I19</f>
-        <v>8897381.25509478</v>
+        <v>8718915.25509478</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8780,7 +8779,7 @@
       </c>
       <c r="H21" s="91" t="n">
         <f aca="false">Portfolio!I20</f>
-        <v>9273968.09748204</v>
+        <v>9120642.09748204</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8814,7 +8813,7 @@
       </c>
       <c r="H22" s="91" t="n">
         <f aca="false">Portfolio!I21</f>
-        <v>9689069.56774696</v>
+        <v>9562567.56774696</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8848,7 +8847,7 @@
       </c>
       <c r="H23" s="91" t="n">
         <f aca="false">Portfolio!I22</f>
-        <v>10145579.3644652</v>
+        <v>10047697.3644652</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8882,7 +8881,7 @@
       </c>
       <c r="H24" s="91" t="n">
         <f aca="false">Portfolio!I23</f>
-        <v>10646615.4969424</v>
+        <v>10579269.4969424</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8916,7 +8915,7 @@
       </c>
       <c r="H25" s="91" t="n">
         <f aca="false">Portfolio!I24</f>
-        <v>11195537.9369923</v>
+        <v>11160773.9369923</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17269,8 +17268,8 @@
         <v>4568958.75</v>
       </c>
       <c r="I3" s="75" t="n">
-        <f aca="false">H3+Inputs!B36*POWER(1+Inputs!B52,VALUE(A3)-Inputs!B4)</f>
-        <v>5368958.75</v>
+        <f aca="false">H3+Inputs!B36*POWER(1+Inputs!B52,VALUE(A3)-Inputs!B4)-IFERROR(IF(Inputs!B48&lt;=0,0,IF(AND(Inputs!B51=1,A3&gt;=Inputs!B5),0,IF(MAX(0,Inputs!B48*12-(A3-Inputs!B4)*12)&lt;=0,0,IF(Inputs!B49=0,Inputs!B30*MAX(0,Inputs!B48*12-(A3-Inputs!B4)*12),ROUND(Inputs!B30*(1-POWER(1+Inputs!B49/12,-MAX(0,Inputs!B48*12-(A3-Inputs!B4)*12)))/(Inputs!B49/12),0))))),0)</f>
+        <v>4948165.75</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17306,8 +17305,8 @@
         <v>4980634.2</v>
       </c>
       <c r="I4" s="75" t="n">
-        <f aca="false">H4+Inputs!B36*POWER(1+Inputs!B52,VALUE(A4)-Inputs!B4)</f>
-        <v>5816634.2</v>
+        <f aca="false">H4+Inputs!B36*POWER(1+Inputs!B52,VALUE(A4)-Inputs!B4)-IFERROR(IF(Inputs!B48&lt;=0,0,IF(AND(Inputs!B51=1,A4&gt;=Inputs!B5),0,IF(MAX(0,Inputs!B48*12-(A4-Inputs!B4)*12)&lt;=0,0,IF(Inputs!B49=0,Inputs!B30*MAX(0,Inputs!B48*12-(A4-Inputs!B4)*12),ROUND(Inputs!B30*(1-POWER(1+Inputs!B49/12,-MAX(0,Inputs!B48*12-(A4-Inputs!B4)*12)))/(Inputs!B49/12),0))))),0)</f>
+        <v>5404751.2</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17343,8 +17342,8 @@
         <v>5425243.686</v>
       </c>
       <c r="I5" s="75" t="n">
-        <f aca="false">H5+Inputs!B36*POWER(1+Inputs!B52,VALUE(A5)-Inputs!B4)</f>
-        <v>6298863.686</v>
+        <f aca="false">H5+Inputs!B36*POWER(1+Inputs!B52,VALUE(A5)-Inputs!B4)-IFERROR(IF(Inputs!B48&lt;=0,0,IF(AND(Inputs!B51=1,A5&gt;=Inputs!B5),0,IF(MAX(0,Inputs!B48*12-(A5-Inputs!B4)*12)&lt;=0,0,IF(Inputs!B49=0,Inputs!B30*MAX(0,Inputs!B48*12-(A5-Inputs!B4)*12),ROUND(Inputs!B30*(1-POWER(1+Inputs!B49/12,-MAX(0,Inputs!B48*12-(A5-Inputs!B4)*12)))/(Inputs!B49/12),0))))),0)</f>
+        <v>5896488.686</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17380,8 +17379,8 @@
         <v>5905421.93088</v>
       </c>
       <c r="I6" s="75" t="n">
-        <f aca="false">H6+Inputs!B36*POWER(1+Inputs!B52,VALUE(A6)-Inputs!B4)</f>
-        <v>6818354.83088</v>
+        <f aca="false">H6+Inputs!B36*POWER(1+Inputs!B52,VALUE(A6)-Inputs!B4)-IFERROR(IF(Inputs!B48&lt;=0,0,IF(AND(Inputs!B51=1,A6&gt;=Inputs!B5),0,IF(MAX(0,Inputs!B48*12-(A6-Inputs!B4)*12)&lt;=0,0,IF(Inputs!B49=0,Inputs!B30*MAX(0,Inputs!B48*12-(A6-Inputs!B4)*12),ROUND(Inputs!B30*(1-POWER(1+Inputs!B49/12,-MAX(0,Inputs!B48*12-(A6-Inputs!B4)*12)))/(Inputs!B49/12),0))))),0)</f>
+        <v>6426123.83088</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17417,8 +17416,8 @@
         <v>6424014.4353504</v>
       </c>
       <c r="I7" s="75" t="n">
-        <f aca="false">H7+Inputs!B36*POWER(1+Inputs!B52,VALUE(A7)-Inputs!B4)</f>
-        <v>7378029.3158504</v>
+        <f aca="false">H7+Inputs!B36*POWER(1+Inputs!B52,VALUE(A7)-Inputs!B4)-IFERROR(IF(Inputs!B48&lt;=0,0,IF(AND(Inputs!B51=1,A7&gt;=Inputs!B5),0,IF(MAX(0,Inputs!B48*12-(A7-Inputs!B4)*12)&lt;=0,0,IF(Inputs!B49=0,Inputs!B30*MAX(0,Inputs!B48*12-(A7-Inputs!B4)*12),ROUND(Inputs!B30*(1-POWER(1+Inputs!B49/12,-MAX(0,Inputs!B48*12-(A7-Inputs!B4)*12)))/(Inputs!B49/12),0))))),0)</f>
+        <v>6996622.3158504</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17454,8 +17453,8 @@
         <v>6984094.34017843</v>
       </c>
       <c r="I8" s="75" t="n">
-        <f aca="false">H8+Inputs!B36*POWER(1+Inputs!B52,VALUE(A8)-Inputs!B4)</f>
-        <v>7981039.89030093</v>
+        <f aca="false">H8+Inputs!B36*POWER(1+Inputs!B52,VALUE(A8)-Inputs!B4)-IFERROR(IF(Inputs!B48&lt;=0,0,IF(AND(Inputs!B51=1,A8&gt;=Inputs!B5),0,IF(MAX(0,Inputs!B48*12-(A8-Inputs!B4)*12)&lt;=0,0,IF(Inputs!B49=0,Inputs!B30*MAX(0,Inputs!B48*12-(A8-Inputs!B4)*12),ROUND(Inputs!B30*(1-POWER(1+Inputs!B49/12,-MAX(0,Inputs!B48*12-(A8-Inputs!B4)*12)))/(Inputs!B49/12),0))))),0)</f>
+        <v>7611181.89030093</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17491,8 +17490,8 @@
         <v>7588980.63739271</v>
       </c>
       <c r="I9" s="75" t="n">
-        <f aca="false">H9+Inputs!B36*POWER(1+Inputs!B52,VALUE(A9)-Inputs!B4)</f>
-        <v>8630788.73727072</v>
+        <f aca="false">H9+Inputs!B36*POWER(1+Inputs!B52,VALUE(A9)-Inputs!B4)-IFERROR(IF(Inputs!B48&lt;=0,0,IF(AND(Inputs!B51=1,A9&gt;=Inputs!B5),0,IF(MAX(0,Inputs!B48*12-(A9-Inputs!B4)*12)&lt;=0,0,IF(Inputs!B49=0,Inputs!B30*MAX(0,Inputs!B48*12-(A9-Inputs!B4)*12),ROUND(Inputs!B30*(1-POWER(1+Inputs!B49/12,-MAX(0,Inputs!B48*12-(A9-Inputs!B4)*12)))/(Inputs!B49/12),0))))),0)</f>
+        <v>8273252.73727072</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17528,8 +17527,8 @@
         <v>8242257.83838413</v>
       </c>
       <c r="I10" s="75" t="n">
-        <f aca="false">H10+Inputs!B36*POWER(1+Inputs!B52,VALUE(A10)-Inputs!B4)</f>
-        <v>9330947.30275665</v>
+        <f aca="false">H10+Inputs!B36*POWER(1+Inputs!B52,VALUE(A10)-Inputs!B4)-IFERROR(IF(Inputs!B48&lt;=0,0,IF(AND(Inputs!B51=1,A10&gt;=Inputs!B5),0,IF(MAX(0,Inputs!B48*12-(A10-Inputs!B4)*12)&lt;=0,0,IF(Inputs!B49=0,Inputs!B30*MAX(0,Inputs!B48*12-(A10-Inputs!B4)*12),ROUND(Inputs!B30*(1-POWER(1+Inputs!B49/12,-MAX(0,Inputs!B48*12-(A10-Inputs!B4)*12)))/(Inputs!B49/12),0))))),0)</f>
+        <v>8986558.30275665</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17565,8 +17564,8 @@
         <v>8947797.21545486</v>
       </c>
       <c r="I11" s="75" t="n">
-        <f aca="false">H11+Inputs!B36*POWER(1+Inputs!B52,VALUE(A11)-Inputs!B4)</f>
-        <v>10085477.7057241</v>
+        <f aca="false">H11+Inputs!B36*POWER(1+Inputs!B52,VALUE(A11)-Inputs!B4)-IFERROR(IF(Inputs!B48&lt;=0,0,IF(AND(Inputs!B51=1,A11&gt;=Inputs!B5),0,IF(MAX(0,Inputs!B48*12-(A11-Inputs!B4)*12)&lt;=0,0,IF(Inputs!B49=0,Inputs!B30*MAX(0,Inputs!B48*12-(A11-Inputs!B4)*12),ROUND(Inputs!B30*(1-POWER(1+Inputs!B49/12,-MAX(0,Inputs!B48*12-(A11-Inputs!B4)*12)))/(Inputs!B49/12),0))))),0)</f>
+        <v>9755115.70572414</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17602,8 +17601,8 @@
         <v>5987338.14586009</v>
       </c>
       <c r="I12" s="37" t="n">
-        <f aca="false">H12+Inputs!B36*POWER(1+Inputs!B52,VALUE(A12)-Inputs!B4)</f>
-        <v>7176214.2581915</v>
+        <f aca="false">H12+Inputs!B36*POWER(1+Inputs!B52,VALUE(A12)-Inputs!B4)-IFERROR(IF(Inputs!B48&lt;=0,0,IF(AND(Inputs!B51=1,A12&gt;=Inputs!B5),0,IF(MAX(0,Inputs!B48*12-(A12-Inputs!B4)*12)&lt;=0,0,IF(Inputs!B49=0,Inputs!B30*MAX(0,Inputs!B48*12-(A12-Inputs!B4)*12),ROUND(Inputs!B30*(1-POWER(1+Inputs!B49/12,-MAX(0,Inputs!B48*12-(A12-Inputs!B4)*12)))/(Inputs!B49/12),0))))),0)</f>
+        <v>6860820.2581915</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17639,8 +17638,8 @@
         <v>6066628.1975289</v>
       </c>
       <c r="I13" s="35" t="n">
-        <f aca="false">H13+Inputs!B36*POWER(1+Inputs!B52,VALUE(A13)-Inputs!B4)</f>
-        <v>7309003.73491522</v>
+        <f aca="false">H13+Inputs!B36*POWER(1+Inputs!B52,VALUE(A13)-Inputs!B4)-IFERROR(IF(Inputs!B48&lt;=0,0,IF(AND(Inputs!B51=1,A13&gt;=Inputs!B5),0,IF(MAX(0,Inputs!B48*12-(A13-Inputs!B4)*12)&lt;=0,0,IF(Inputs!B49=0,Inputs!B30*MAX(0,Inputs!B48*12-(A13-Inputs!B4)*12),ROUND(Inputs!B30*(1-POWER(1+Inputs!B49/12,-MAX(0,Inputs!B48*12-(A13-Inputs!B4)*12)))/(Inputs!B49/12),0))))),0)</f>
+        <v>7009578.73491522</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17676,8 +17675,8 @@
         <v>6206343.30333121</v>
       </c>
       <c r="I14" s="37" t="n">
-        <f aca="false">H14+Inputs!B36*POWER(1+Inputs!B52,VALUE(A14)-Inputs!B4)</f>
-        <v>7504625.73989991</v>
+        <f aca="false">H14+Inputs!B36*POWER(1+Inputs!B52,VALUE(A14)-Inputs!B4)-IFERROR(IF(Inputs!B48&lt;=0,0,IF(AND(Inputs!B51=1,A14&gt;=Inputs!B5),0,IF(MAX(0,Inputs!B48*12-(A14-Inputs!B4)*12)&lt;=0,0,IF(Inputs!B49=0,Inputs!B30*MAX(0,Inputs!B48*12-(A14-Inputs!B4)*12),ROUND(Inputs!B30*(1-POWER(1+Inputs!B49/12,-MAX(0,Inputs!B48*12-(A14-Inputs!B4)*12)))/(Inputs!B49/12),0))))),0)</f>
+        <v>7222239.73989991</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17713,8 +17712,8 @@
         <v>6368568.94809771</v>
       </c>
       <c r="I15" s="35" t="n">
-        <f aca="false">H15+Inputs!B36*POWER(1+Inputs!B52,VALUE(A15)-Inputs!B4)</f>
-        <v>7725274.094312</v>
+        <f aca="false">H15+Inputs!B36*POWER(1+Inputs!B52,VALUE(A15)-Inputs!B4)-IFERROR(IF(Inputs!B48&lt;=0,0,IF(AND(Inputs!B51=1,A15&gt;=Inputs!B5),0,IF(MAX(0,Inputs!B48*12-(A15-Inputs!B4)*12)&lt;=0,0,IF(Inputs!B49=0,Inputs!B30*MAX(0,Inputs!B48*12-(A15-Inputs!B4)*12),ROUND(Inputs!B30*(1-POWER(1+Inputs!B49/12,-MAX(0,Inputs!B48*12-(A15-Inputs!B4)*12)))/(Inputs!B49/12),0))))),0)</f>
+        <v>7461069.094312</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17750,8 +17749,8 @@
         <v>6555044.14877053</v>
       </c>
       <c r="I16" s="37" t="n">
-        <f aca="false">H16+Inputs!B36*POWER(1+Inputs!B52,VALUE(A16)-Inputs!B4)</f>
-        <v>7972801.02656446</v>
+        <f aca="false">H16+Inputs!B36*POWER(1+Inputs!B52,VALUE(A16)-Inputs!B4)-IFERROR(IF(Inputs!B48&lt;=0,0,IF(AND(Inputs!B51=1,A16&gt;=Inputs!B5),0,IF(MAX(0,Inputs!B48*12-(A16-Inputs!B4)*12)&lt;=0,0,IF(Inputs!B49=0,Inputs!B30*MAX(0,Inputs!B48*12-(A16-Inputs!B4)*12),ROUND(Inputs!B30*(1-POWER(1+Inputs!B49/12,-MAX(0,Inputs!B48*12-(A16-Inputs!B4)*12)))/(Inputs!B49/12),0))))),0)</f>
+        <v>7727993.02656446</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17787,8 +17786,8 @@
         <v>6767645.34502092</v>
       </c>
       <c r="I17" s="35" t="n">
-        <f aca="false">H17+Inputs!B36*POWER(1+Inputs!B52,VALUE(A17)-Inputs!B4)</f>
-        <v>8249201.28231558</v>
+        <f aca="false">H17+Inputs!B36*POWER(1+Inputs!B52,VALUE(A17)-Inputs!B4)-IFERROR(IF(Inputs!B48&lt;=0,0,IF(AND(Inputs!B51=1,A17&gt;=Inputs!B5),0,IF(MAX(0,Inputs!B48*12-(A17-Inputs!B4)*12)&lt;=0,0,IF(Inputs!B49=0,Inputs!B30*MAX(0,Inputs!B48*12-(A17-Inputs!B4)*12),ROUND(Inputs!B30*(1-POWER(1+Inputs!B49/12,-MAX(0,Inputs!B48*12-(A17-Inputs!B4)*12)))/(Inputs!B49/12),0))))),0)</f>
+        <v>8025090.28231558</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17824,8 +17823,8 @@
         <v>7008397.34295334</v>
       </c>
       <c r="I18" s="37" t="n">
-        <f aca="false">H18+Inputs!B36*POWER(1+Inputs!B52,VALUE(A18)-Inputs!B4)</f>
-        <v>8556623.29742627</v>
+        <f aca="false">H18+Inputs!B36*POWER(1+Inputs!B52,VALUE(A18)-Inputs!B4)-IFERROR(IF(Inputs!B48&lt;=0,0,IF(AND(Inputs!B51=1,A18&gt;=Inputs!B5),0,IF(MAX(0,Inputs!B48*12-(A18-Inputs!B4)*12)&lt;=0,0,IF(Inputs!B49=0,Inputs!B30*MAX(0,Inputs!B48*12-(A18-Inputs!B4)*12),ROUND(Inputs!B30*(1-POWER(1+Inputs!B49/12,-MAX(0,Inputs!B48*12-(A18-Inputs!B4)*12)))/(Inputs!B49/12),0))))),0)</f>
+        <v>8354595.29742627</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17861,8 +17860,8 @@
         <v>7279485.13267057</v>
       </c>
       <c r="I19" s="35" t="n">
-        <f aca="false">H19+Inputs!B36*POWER(1+Inputs!B52,VALUE(A19)-Inputs!B4)</f>
-        <v>8897381.25509478</v>
+        <f aca="false">H19+Inputs!B36*POWER(1+Inputs!B52,VALUE(A19)-Inputs!B4)-IFERROR(IF(Inputs!B48&lt;=0,0,IF(AND(Inputs!B51=1,A19&gt;=Inputs!B5),0,IF(MAX(0,Inputs!B48*12-(A19-Inputs!B4)*12)&lt;=0,0,IF(Inputs!B49=0,Inputs!B30*MAX(0,Inputs!B48*12-(A19-Inputs!B4)*12),ROUND(Inputs!B30*(1-POWER(1+Inputs!B49/12,-MAX(0,Inputs!B48*12-(A19-Inputs!B4)*12)))/(Inputs!B49/12),0))))),0)</f>
+        <v>8718915.25509478</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17898,8 +17897,8 @@
         <v>7583266.64954875</v>
       </c>
       <c r="I20" s="39" t="n">
-        <f aca="false">H20+Inputs!B36*POWER(1+Inputs!B52,VALUE(A20)-Inputs!B4)</f>
-        <v>9273968.09748204</v>
+        <f aca="false">H20+Inputs!B36*POWER(1+Inputs!B52,VALUE(A20)-Inputs!B4)-IFERROR(IF(Inputs!B48&lt;=0,0,IF(AND(Inputs!B51=1,A20&gt;=Inputs!B5),0,IF(MAX(0,Inputs!B48*12-(A20-Inputs!B4)*12)&lt;=0,0,IF(Inputs!B49=0,Inputs!B30*MAX(0,Inputs!B48*12-(A20-Inputs!B4)*12),ROUND(Inputs!B30*(1-POWER(1+Inputs!B49/12,-MAX(0,Inputs!B48*12-(A20-Inputs!B4)*12)))/(Inputs!B49/12),0))))),0)</f>
+        <v>9120642.09748204</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17935,8 +17934,8 @@
         <v>7922286.55465667</v>
       </c>
       <c r="I21" s="39" t="n">
-        <f aca="false">H21+Inputs!B36*POWER(1+Inputs!B52,VALUE(A21)-Inputs!B4)</f>
-        <v>9689069.56774696</v>
+        <f aca="false">H21+Inputs!B36*POWER(1+Inputs!B52,VALUE(A21)-Inputs!B4)-IFERROR(IF(Inputs!B48&lt;=0,0,IF(AND(Inputs!B51=1,A21&gt;=Inputs!B5),0,IF(MAX(0,Inputs!B48*12-(A21-Inputs!B4)*12)&lt;=0,0,IF(Inputs!B49=0,Inputs!B30*MAX(0,Inputs!B48*12-(A21-Inputs!B4)*12),ROUND(Inputs!B30*(1-POWER(1+Inputs!B49/12,-MAX(0,Inputs!B48*12-(A21-Inputs!B4)*12)))/(Inputs!B49/12),0))))),0)</f>
+        <v>9562567.56774696</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17972,8 +17971,8 @@
         <v>8299291.11578583</v>
       </c>
       <c r="I22" s="39" t="n">
-        <f aca="false">H22+Inputs!B36*POWER(1+Inputs!B52,VALUE(A22)-Inputs!B4)</f>
-        <v>10145579.3644652</v>
+        <f aca="false">H22+Inputs!B36*POWER(1+Inputs!B52,VALUE(A22)-Inputs!B4)-IFERROR(IF(Inputs!B48&lt;=0,0,IF(AND(Inputs!B51=1,A22&gt;=Inputs!B5),0,IF(MAX(0,Inputs!B48*12-(A22-Inputs!B4)*12)&lt;=0,0,IF(Inputs!B49=0,Inputs!B30*MAX(0,Inputs!B48*12-(A22-Inputs!B4)*12),ROUND(Inputs!B30*(1-POWER(1+Inputs!B49/12,-MAX(0,Inputs!B48*12-(A22-Inputs!B4)*12)))/(Inputs!B49/12),0))))),0)</f>
+        <v>10047697.3644652</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18009,8 +18008,8 @@
         <v>8717244.27707245</v>
       </c>
       <c r="I23" s="39" t="n">
-        <f aca="false">H23+Inputs!B36*POWER(1+Inputs!B52,VALUE(A23)-Inputs!B4)</f>
-        <v>10646615.4969424</v>
+        <f aca="false">H23+Inputs!B36*POWER(1+Inputs!B52,VALUE(A23)-Inputs!B4)-IFERROR(IF(Inputs!B48&lt;=0,0,IF(AND(Inputs!B51=1,A23&gt;=Inputs!B5),0,IF(MAX(0,Inputs!B48*12-(A23-Inputs!B4)*12)&lt;=0,0,IF(Inputs!B49=0,Inputs!B30*MAX(0,Inputs!B48*12-(A23-Inputs!B4)*12),ROUND(Inputs!B30*(1-POWER(1+Inputs!B49/12,-MAX(0,Inputs!B48*12-(A23-Inputs!B4)*12)))/(Inputs!B49/12),0))))),0)</f>
+        <v>10579269.4969424</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18046,8 +18045,8 @@
         <v>9179345.01222822</v>
       </c>
       <c r="I24" s="39" t="n">
-        <f aca="false">H24+Inputs!B36*POWER(1+Inputs!B52,VALUE(A24)-Inputs!B4)</f>
-        <v>11195537.9369923</v>
+        <f aca="false">H24+Inputs!B36*POWER(1+Inputs!B52,VALUE(A24)-Inputs!B4)-IFERROR(IF(Inputs!B48&lt;=0,0,IF(AND(Inputs!B51=1,A24&gt;=Inputs!B5),0,IF(MAX(0,Inputs!B48*12-(A24-Inputs!B4)*12)&lt;=0,0,IF(Inputs!B49=0,Inputs!B30*MAX(0,Inputs!B48*12-(A24-Inputs!B4)*12),ROUND(Inputs!B30*(1-POWER(1+Inputs!B49/12,-MAX(0,Inputs!B48*12-(A24-Inputs!B4)*12)))/(Inputs!B49/12),0))))),0)</f>
+        <v>11160773.9369923</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18083,7 +18082,7 @@
         <v>9689046.06399511</v>
       </c>
       <c r="I25" s="39" t="n">
-        <f aca="false">H25+Inputs!B36*POWER(1+Inputs!B52,VALUE(A25)-Inputs!B4)</f>
+        <f aca="false">H25+Inputs!B36*POWER(1+Inputs!B52,VALUE(A25)-Inputs!B4)-IFERROR(IF(Inputs!B48&lt;=0,0,IF(AND(Inputs!B51=1,A25&gt;=Inputs!B5),0,IF(MAX(0,Inputs!B48*12-(A25-Inputs!B4)*12)&lt;=0,0,IF(Inputs!B49=0,Inputs!B30*MAX(0,Inputs!B48*12-(A25-Inputs!B4)*12),ROUND(Inputs!B30*(1-POWER(1+Inputs!B49/12,-MAX(0,Inputs!B48*12-(A25-Inputs!B4)*12)))/(Inputs!B49/12),0))))),0)</f>
         <v>11795967.6703736</v>
       </c>
     </row>
@@ -18120,7 +18119,7 @@
         <v>10250074.1806457</v>
       </c>
       <c r="I26" s="39" t="n">
-        <f aca="false">H26+Inputs!B36*POWER(1+Inputs!B52,VALUE(A26)-Inputs!B4)</f>
+        <f aca="false">H26+Inputs!B36*POWER(1+Inputs!B52,VALUE(A26)-Inputs!B4)-IFERROR(IF(Inputs!B48&lt;=0,0,IF(AND(Inputs!B51=1,A26&gt;=Inputs!B5),0,IF(MAX(0,Inputs!B48*12-(A26-Inputs!B4)*12)&lt;=0,0,IF(Inputs!B49=0,Inputs!B30*MAX(0,Inputs!B48*12-(A26-Inputs!B4)*12),ROUND(Inputs!B30*(1-POWER(1+Inputs!B49/12,-MAX(0,Inputs!B48*12-(A26-Inputs!B4)*12)))/(Inputs!B49/12),0))))),0)</f>
         <v>12451807.2593111</v>
       </c>
     </row>
@@ -18157,7 +18156,7 @@
         <v>10866451.9692128</v>
       </c>
       <c r="I27" s="39" t="n">
-        <f aca="false">H27+Inputs!B36*POWER(1+Inputs!B52,VALUE(A27)-Inputs!B4)</f>
+        <f aca="false">H27+Inputs!B36*POWER(1+Inputs!B52,VALUE(A27)-Inputs!B4)-IFERROR(IF(Inputs!B48&lt;=0,0,IF(AND(Inputs!B51=1,A27&gt;=Inputs!B5),0,IF(MAX(0,Inputs!B48*12-(A27-Inputs!B4)*12)&lt;=0,0,IF(Inputs!B49=0,Inputs!B30*MAX(0,Inputs!B48*12-(A27-Inputs!B4)*12),ROUND(Inputs!B30*(1-POWER(1+Inputs!B49/12,-MAX(0,Inputs!B48*12-(A27-Inputs!B4)*12)))/(Inputs!B49/12),0))))),0)</f>
         <v>13167263.0364182</v>
       </c>
     </row>
@@ -18194,7 +18193,7 @@
         <v>11542521.4947042</v>
       </c>
       <c r="I28" s="39" t="n">
-        <f aca="false">H28+Inputs!B36*POWER(1+Inputs!B52,VALUE(A28)-Inputs!B4)</f>
+        <f aca="false">H28+Inputs!B36*POWER(1+Inputs!B52,VALUE(A28)-Inputs!B4)-IFERROR(IF(Inputs!B48&lt;=0,0,IF(AND(Inputs!B51=1,A28&gt;=Inputs!B5),0,IF(MAX(0,Inputs!B48*12-(A28-Inputs!B4)*12)&lt;=0,0,IF(Inputs!B49=0,Inputs!B30*MAX(0,Inputs!B48*12-(A28-Inputs!B4)*12),ROUND(Inputs!B30*(1-POWER(1+Inputs!B49/12,-MAX(0,Inputs!B48*12-(A28-Inputs!B4)*12)))/(Inputs!B49/12),0))))),0)</f>
         <v>13946869.0599338</v>
       </c>
     </row>
@@ -18231,7 +18230,7 @@
         <v>12282969.7648941</v>
       </c>
       <c r="I29" s="39" t="n">
-        <f aca="false">H29+Inputs!B36*POWER(1+Inputs!B52,VALUE(A29)-Inputs!B4)</f>
+        <f aca="false">H29+Inputs!B36*POWER(1+Inputs!B52,VALUE(A29)-Inputs!B4)-IFERROR(IF(Inputs!B48&lt;=0,0,IF(AND(Inputs!B51=1,A29&gt;=Inputs!B5),0,IF(MAX(0,Inputs!B48*12-(A29-Inputs!B4)*12)&lt;=0,0,IF(Inputs!B49=0,Inputs!B30*MAX(0,Inputs!B48*12-(A29-Inputs!B4)*12),ROUND(Inputs!B30*(1-POWER(1+Inputs!B49/12,-MAX(0,Inputs!B48*12-(A29-Inputs!B4)*12)))/(Inputs!B49/12),0))))),0)</f>
         <v>14795512.9705591</v>
       </c>
     </row>
@@ -18268,7 +18267,7 @@
         <v>13092856.2514479</v>
       </c>
       <c r="I30" s="39" t="n">
-        <f aca="false">H30+Inputs!B36*POWER(1+Inputs!B52,VALUE(A30)-Inputs!B4)</f>
+        <f aca="false">H30+Inputs!B36*POWER(1+Inputs!B52,VALUE(A30)-Inputs!B4)-IFERROR(IF(Inputs!B48&lt;=0,0,IF(AND(Inputs!B51=1,A30&gt;=Inputs!B5),0,IF(MAX(0,Inputs!B48*12-(A30-Inputs!B4)*12)&lt;=0,0,IF(Inputs!B49=0,Inputs!B30*MAX(0,Inputs!B48*12-(A30-Inputs!B4)*12),ROUND(Inputs!B30*(1-POWER(1+Inputs!B49/12,-MAX(0,Inputs!B48*12-(A30-Inputs!B4)*12)))/(Inputs!B49/12),0))))),0)</f>
         <v>15718463.9013678</v>
       </c>
     </row>
@@ -18305,7 +18304,7 @@
         <v>13977642.6101926</v>
       </c>
       <c r="I31" s="39" t="n">
-        <f aca="false">H31+Inputs!B36*POWER(1+Inputs!B52,VALUE(A31)-Inputs!B4)</f>
+        <f aca="false">H31+Inputs!B36*POWER(1+Inputs!B52,VALUE(A31)-Inputs!B4)-IFERROR(IF(Inputs!B48&lt;=0,0,IF(AND(Inputs!B51=1,A31&gt;=Inputs!B5),0,IF(MAX(0,Inputs!B48*12-(A31-Inputs!B4)*12)&lt;=0,0,IF(Inputs!B49=0,Inputs!B30*MAX(0,Inputs!B48*12-(A31-Inputs!B4)*12),ROUND(Inputs!B30*(1-POWER(1+Inputs!B49/12,-MAX(0,Inputs!B48*12-(A31-Inputs!B4)*12)))/(Inputs!B49/12),0))))),0)</f>
         <v>16721402.604359</v>
       </c>
     </row>
@@ -18342,7 +18341,7 @@
         <v>14943224.7763668</v>
       </c>
       <c r="I32" s="39" t="n">
-        <f aca="false">H32+Inputs!B36*POWER(1+Inputs!B52,VALUE(A32)-Inputs!B4)</f>
+        <f aca="false">H32+Inputs!B36*POWER(1+Inputs!B52,VALUE(A32)-Inputs!B4)-IFERROR(IF(Inputs!B48&lt;=0,0,IF(AND(Inputs!B51=1,A32&gt;=Inputs!B5),0,IF(MAX(0,Inputs!B48*12-(A32-Inputs!B4)*12)&lt;=0,0,IF(Inputs!B49=0,Inputs!B30*MAX(0,Inputs!B48*12-(A32-Inputs!B4)*12),ROUND(Inputs!B30*(1-POWER(1+Inputs!B49/12,-MAX(0,Inputs!B48*12-(A32-Inputs!B4)*12)))/(Inputs!B49/12),0))))),0)</f>
         <v>17810453.9702706</v>
       </c>
     </row>

</xml_diff>